<commit_message>
plan de compras: sin la carga de Cassio del martes 06/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F55DFD4-0008-42D6-9667-93576920F21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B5A0B3-74E7-4B60-AF2D-52250EAD9DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,12 +110,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1525" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1520" uniqueCount="678">
   <si>
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 30/09/2026 17:20 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 30/09/2026 17:24 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>18840</v>
+        <v>17904</v>
       </c>
       <c r="D8" s="7">
         <f>Demanda!H9</f>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="H8" s="7">
         <f ca="1">Proyeccion!L8</f>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="I8" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="H9" s="7">
         <f ca="1">Proyeccion!L9</f>
-        <v>22614</v>
+        <v>22678</v>
       </c>
       <c r="I9" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="H10" s="7">
         <f ca="1">Proyeccion!L10</f>
-        <v>22578</v>
+        <v>22642</v>
       </c>
       <c r="I10" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="H11" s="7">
         <f ca="1">Proyeccion!L11</f>
-        <v>22642</v>
+        <v>22706</v>
       </c>
       <c r="I11" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="H12" s="7">
         <f ca="1">Proyeccion!L12</f>
-        <v>22706</v>
+        <v>22770</v>
       </c>
       <c r="I12" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="H13" s="7">
         <f ca="1">Proyeccion!L13</f>
-        <v>22770</v>
+        <v>22834</v>
       </c>
       <c r="I13" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="H14" s="7">
         <f ca="1">Proyeccion!L14</f>
-        <v>22834</v>
+        <v>22898</v>
       </c>
       <c r="I14" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="H15" s="7">
         <f ca="1">Proyeccion!L15</f>
-        <v>22898</v>
+        <v>22962</v>
       </c>
       <c r="I15" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="H16" s="7">
         <f ca="1">Proyeccion!L16</f>
-        <v>22962</v>
+        <v>23026</v>
       </c>
       <c r="I16" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="H17" s="7">
         <f ca="1">Proyeccion!L17</f>
-        <v>23026</v>
+        <v>23090</v>
       </c>
       <c r="I17" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H18" s="7">
         <f ca="1">Proyeccion!L18</f>
-        <v>23090</v>
+        <v>23154</v>
       </c>
       <c r="I18" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="B10" s="24">
         <f ca="1">AVERAGEIFS(PrCobertura,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8.1907058823529404</v>
+        <v>8.1194117647058821</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>303</v>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="B12" s="25">
         <f ca="1">SUMIFS(PrACargar,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>307</v>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="B19" s="24">
         <f ca="1">AVERAGEIFS(PrCamiones,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>13.5</v>
+        <v>13.25</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>320</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B20" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BR",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.61492559579308548</v>
+        <v>0.60808502562156008</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>322</v>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="B21" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"PY",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.36549434975571549</v>
+        <v>0.37198709432529892</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>3</v>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="B22" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>1.9580054451199046E-2</v>
+        <v>1.9927880053141014E-2</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>3</v>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="B23" s="12">
         <f ca="1">SUMIFS(CgCosto,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>382339.83999999973</v>
+        <v>375703.59999999974</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>326</v>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="B27" s="25">
         <f>COUNTIFS(CgEstado,"Dictado",CgCuenta,1)</f>
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>334</v>
@@ -5312,7 +5312,7 @@
       </c>
       <c r="O7">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7" t="s">
         <v>3</v>
@@ -11820,17 +11820,17 @@
         <v>58</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="G28" s="8">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="H28" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I28" s="9" t="s">
         <v>199</v>
@@ -11858,7 +11858,7 @@
       </c>
       <c r="P28" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>7146.72</v>
       </c>
       <c r="Q28" s="9" t="s">
         <v>225</v>
@@ -11896,10 +11896,10 @@
         <v>58</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G29" s="8">
         <v>1008</v>
@@ -11969,20 +11969,20 @@
         <v>mar</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>210</v>
+        <v>3</v>
       </c>
       <c r="G30" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H30" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I30" s="9" t="s">
         <v>199</v>
@@ -11990,11 +11990,11 @@
       <c r="J30" s="6"/>
       <c r="K30">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L30" s="5">
         <f t="shared" si="4"/>
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="M30" s="5">
         <f t="shared" si="5"/>
@@ -12006,22 +12006,22 @@
       </c>
       <c r="O30" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P30" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q30" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="R30" s="5">
         <f t="shared" si="9"/>
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="S30" s="5">
         <f t="shared" si="10"/>
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="T30" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -12048,7 +12048,7 @@
         <v>59</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -12089,7 +12089,7 @@
         <v>6860</v>
       </c>
       <c r="Q31" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="R31" s="5">
         <f t="shared" si="9"/>
@@ -12114,27 +12114,27 @@
         <v>28</v>
       </c>
       <c r="B32" s="6">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>mié</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>3</v>
+        <v>210</v>
       </c>
       <c r="G32" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H32" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I32" s="9" t="s">
         <v>199</v>
@@ -12142,7 +12142,7 @@
       <c r="J32" s="6"/>
       <c r="K32">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L32" s="5">
         <f t="shared" si="4"/>
@@ -12158,22 +12158,22 @@
       </c>
       <c r="O32" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P32" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q32" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="R32" s="5">
         <f t="shared" si="9"/>
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="S32" s="5">
         <f t="shared" si="10"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="T32" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -12200,10 +12200,10 @@
         <v>58</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="G33" s="8">
         <v>1008</v>
@@ -12273,20 +12273,20 @@
         <v>mié</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>206</v>
+        <v>3</v>
       </c>
       <c r="G34" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H34" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I34" s="9" t="s">
         <v>199</v>
@@ -12294,11 +12294,11 @@
       <c r="J34" s="6"/>
       <c r="K34">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L34" s="5">
         <f t="shared" si="4"/>
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="M34" s="5">
         <f t="shared" si="5"/>
@@ -12310,18 +12310,18 @@
       </c>
       <c r="O34" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P34" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q34" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="R34" s="5">
         <f t="shared" si="9"/>
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="S34" s="5">
         <f t="shared" si="10"/>
@@ -12342,27 +12342,27 @@
         <v>31</v>
       </c>
       <c r="B35" s="6">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="1"/>
-        <v>mié</v>
+        <v>vie</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>3</v>
+        <v>210</v>
       </c>
       <c r="G35" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H35" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I35" s="9" t="s">
         <v>199</v>
@@ -12370,15 +12370,15 @@
       <c r="J35" s="6"/>
       <c r="K35">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L35" s="5">
         <f t="shared" si="4"/>
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="M35" s="5">
         <f t="shared" si="5"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="N35">
         <f t="shared" si="6"/>
@@ -12386,18 +12386,18 @@
       </c>
       <c r="O35" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P35" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q35" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="R35" s="5">
         <f t="shared" si="9"/>
-        <v>46307</v>
+        <v>46310</v>
       </c>
       <c r="S35" s="5">
         <f t="shared" si="10"/>
@@ -12428,10 +12428,10 @@
         <v>58</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G36" s="8">
         <v>1008</v>
@@ -12504,10 +12504,10 @@
         <v>58</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G37" s="8">
         <v>1008</v>
@@ -12580,10 +12580,10 @@
         <v>58</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="G38" s="8">
         <v>1008</v>
@@ -12656,7 +12656,7 @@
         <v>58</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>206</v>
@@ -12722,27 +12722,27 @@
         <v>36</v>
       </c>
       <c r="B40" s="6">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>sáb</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="G40" s="8">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="H40" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I40" s="9" t="s">
         <v>199</v>
@@ -12754,7 +12754,7 @@
       </c>
       <c r="L40" s="5">
         <f t="shared" si="4"/>
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="M40" s="5">
         <f t="shared" si="5"/>
@@ -12770,14 +12770,14 @@
       </c>
       <c r="P40" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6636.24</v>
       </c>
       <c r="Q40" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="R40" s="5">
         <f t="shared" si="9"/>
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="S40" s="5">
         <f t="shared" si="10"/>
@@ -12798,39 +12798,39 @@
         <v>37</v>
       </c>
       <c r="B41" s="6">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="1"/>
-        <v>sáb</v>
+        <v>lun</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>218</v>
+        <v>3</v>
       </c>
       <c r="G41" s="8">
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="H41" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>199</v>
+        <v>234</v>
       </c>
       <c r="J41" s="6"/>
       <c r="K41">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L41" s="5">
         <f t="shared" si="4"/>
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="M41" s="5">
         <f t="shared" si="5"/>
@@ -12842,18 +12842,18 @@
       </c>
       <c r="O41" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P41" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>6860</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="R41" s="5">
         <f t="shared" si="9"/>
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="S41" s="5">
         <f t="shared" si="10"/>
@@ -13178,43 +13178,43 @@
         <v>42</v>
       </c>
       <c r="B46" s="6">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>vie</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G46" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H46" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I46" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L46" s="5">
         <f t="shared" si="4"/>
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="M46" s="5">
         <f t="shared" si="5"/>
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="N46">
         <f t="shared" si="6"/>
@@ -13222,22 +13222,22 @@
       </c>
       <c r="O46" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P46" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q46" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="R46" s="5">
         <f t="shared" si="9"/>
-        <v>46312</v>
+        <v>46317</v>
       </c>
       <c r="S46" s="5">
         <f t="shared" si="10"/>
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="T46" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -13786,39 +13786,39 @@
         <v>50</v>
       </c>
       <c r="B54" s="6">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>lun</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G54" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H54" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I54" s="9" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="J54" s="6"/>
       <c r="K54">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L54" s="5">
         <f t="shared" si="4"/>
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="M54" s="5">
         <f t="shared" si="5"/>
@@ -13830,18 +13830,18 @@
       </c>
       <c r="O54" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P54" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q54" s="9" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="R54" s="5">
         <f t="shared" si="9"/>
-        <v>46317</v>
+        <v>46319</v>
       </c>
       <c r="S54" s="5">
         <f t="shared" si="10"/>
@@ -14166,43 +14166,43 @@
         <v>55</v>
       </c>
       <c r="B59" s="6">
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>vie</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G59" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H59" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I59" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L59" s="5">
         <f t="shared" si="4"/>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="M59" s="5">
         <f t="shared" si="5"/>
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="N59">
         <f t="shared" si="6"/>
@@ -14210,22 +14210,22 @@
       </c>
       <c r="O59" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P59" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q59" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="R59" s="5">
         <f t="shared" si="9"/>
-        <v>46319</v>
+        <v>46324</v>
       </c>
       <c r="S59" s="5">
         <f t="shared" si="10"/>
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="T59" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -14774,7 +14774,7 @@
         <v>63</v>
       </c>
       <c r="B67" s="6">
-        <v>46318</v>
+        <v>46325</v>
       </c>
       <c r="C67" t="str">
         <f t="shared" si="1"/>
@@ -14806,11 +14806,11 @@
       </c>
       <c r="L67" s="5">
         <f t="shared" si="4"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="M67" s="5">
         <f t="shared" si="5"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="N67">
         <f t="shared" si="6"/>
@@ -14829,11 +14829,11 @@
       </c>
       <c r="R67" s="5">
         <f t="shared" si="9"/>
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="S67" s="5">
         <f t="shared" si="10"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="T67" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -15382,7 +15382,7 @@
         <v>71</v>
       </c>
       <c r="B75" s="6">
-        <v>46325</v>
+        <v>46332</v>
       </c>
       <c r="C75" t="str">
         <f t="shared" si="14"/>
@@ -15414,11 +15414,11 @@
       </c>
       <c r="L75" s="5">
         <f t="shared" si="17"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="M75" s="5">
         <f t="shared" si="18"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="N75">
         <f t="shared" si="19"/>
@@ -15437,11 +15437,11 @@
       </c>
       <c r="R75" s="5">
         <f t="shared" si="22"/>
-        <v>46331</v>
+        <v>46338</v>
       </c>
       <c r="S75" s="5">
         <f t="shared" si="23"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="T75" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -15990,7 +15990,7 @@
         <v>79</v>
       </c>
       <c r="B83" s="6">
-        <v>46332</v>
+        <v>46339</v>
       </c>
       <c r="C83" t="str">
         <f t="shared" si="14"/>
@@ -16022,11 +16022,11 @@
       </c>
       <c r="L83" s="5">
         <f t="shared" si="17"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="M83" s="5">
         <f t="shared" si="18"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="N83">
         <f t="shared" si="19"/>
@@ -16045,11 +16045,11 @@
       </c>
       <c r="R83" s="5">
         <f t="shared" si="22"/>
-        <v>46338</v>
+        <v>46345</v>
       </c>
       <c r="S83" s="5">
         <f t="shared" si="23"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="T83" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -16598,7 +16598,7 @@
         <v>87</v>
       </c>
       <c r="B91" s="6">
-        <v>46339</v>
+        <v>46346</v>
       </c>
       <c r="C91" t="str">
         <f t="shared" si="14"/>
@@ -16630,11 +16630,11 @@
       </c>
       <c r="L91" s="5">
         <f t="shared" si="17"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="M91" s="5">
         <f t="shared" si="18"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="N91">
         <f t="shared" si="19"/>
@@ -16653,11 +16653,11 @@
       </c>
       <c r="R91" s="5">
         <f t="shared" si="22"/>
-        <v>46345</v>
+        <v>46352</v>
       </c>
       <c r="S91" s="5">
         <f t="shared" si="23"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="T91" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -17206,7 +17206,7 @@
         <v>95</v>
       </c>
       <c r="B99" s="6">
-        <v>46346</v>
+        <v>46353</v>
       </c>
       <c r="C99" t="str">
         <f t="shared" si="14"/>
@@ -17238,11 +17238,11 @@
       </c>
       <c r="L99" s="5">
         <f t="shared" si="17"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="M99" s="5">
         <f t="shared" si="18"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="N99">
         <f t="shared" si="19"/>
@@ -17261,11 +17261,11 @@
       </c>
       <c r="R99" s="5">
         <f t="shared" si="22"/>
-        <v>46352</v>
+        <v>46359</v>
       </c>
       <c r="S99" s="5">
         <f t="shared" si="23"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="T99" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -17814,7 +17814,7 @@
         <v>103</v>
       </c>
       <c r="B107" s="6">
-        <v>46353</v>
+        <v>46360</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="14"/>
@@ -17846,11 +17846,11 @@
       </c>
       <c r="L107" s="5">
         <f t="shared" si="17"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="M107" s="5">
         <f t="shared" si="18"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="N107">
         <f t="shared" si="19"/>
@@ -17869,11 +17869,11 @@
       </c>
       <c r="R107" s="5">
         <f t="shared" si="22"/>
-        <v>46359</v>
+        <v>46366</v>
       </c>
       <c r="S107" s="5">
         <f t="shared" si="23"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="T107" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -18422,7 +18422,7 @@
         <v>111</v>
       </c>
       <c r="B115" s="6">
-        <v>46360</v>
+        <v>46367</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="14"/>
@@ -18454,11 +18454,11 @@
       </c>
       <c r="L115" s="5">
         <f t="shared" si="17"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="M115" s="5">
         <f t="shared" si="18"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="N115">
         <f t="shared" si="19"/>
@@ -18477,11 +18477,11 @@
       </c>
       <c r="R115" s="5">
         <f t="shared" si="22"/>
-        <v>46366</v>
+        <v>46373</v>
       </c>
       <c r="S115" s="5">
         <f t="shared" si="23"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="T115" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19030,7 +19030,7 @@
         <v>119</v>
       </c>
       <c r="B123" s="6">
-        <v>46367</v>
+        <v>46374</v>
       </c>
       <c r="C123" t="str">
         <f t="shared" si="14"/>
@@ -19062,11 +19062,11 @@
       </c>
       <c r="L123" s="5">
         <f t="shared" si="17"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="M123" s="5">
         <f t="shared" si="18"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="N123">
         <f t="shared" si="19"/>
@@ -19085,11 +19085,11 @@
       </c>
       <c r="R123" s="5">
         <f t="shared" si="22"/>
-        <v>46373</v>
+        <v>46380</v>
       </c>
       <c r="S123" s="5">
         <f t="shared" si="23"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="T123" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19633,75 +19633,61 @@
       </c>
     </row>
     <row r="131" spans="1:21">
-      <c r="A131">
+      <c r="A131" t="str">
         <f t="shared" si="13"/>
-        <v>127</v>
-      </c>
-      <c r="B131" s="6">
-        <v>46374</v>
-      </c>
+        <v/>
+      </c>
+      <c r="B131" s="6"/>
       <c r="C131" t="str">
         <f t="shared" si="14"/>
-        <v>vie</v>
-      </c>
-      <c r="D131" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E131" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="F131" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G131" s="8">
-        <v>1008</v>
-      </c>
-      <c r="H131" s="7">
+        <v/>
+      </c>
+      <c r="D131" s="9"/>
+      <c r="E131" s="9"/>
+      <c r="F131" s="9"/>
+      <c r="G131" s="8"/>
+      <c r="H131" s="7" t="str">
         <f t="shared" si="15"/>
-        <v>1008</v>
-      </c>
-      <c r="I131" s="9" t="s">
-        <v>237</v>
-      </c>
+        <v/>
+      </c>
+      <c r="I131" s="9"/>
       <c r="J131" s="6"/>
-      <c r="K131">
+      <c r="K131" t="str">
         <f t="shared" si="16"/>
-        <v>3</v>
-      </c>
-      <c r="L131" s="5">
+        <v/>
+      </c>
+      <c r="L131" s="5" t="str">
         <f t="shared" si="17"/>
-        <v>46377</v>
-      </c>
-      <c r="M131" s="5">
+        <v/>
+      </c>
+      <c r="M131" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>46377</v>
-      </c>
-      <c r="N131">
+        <v/>
+      </c>
+      <c r="N131" t="str">
         <f t="shared" si="19"/>
-        <v>1</v>
-      </c>
-      <c r="O131" s="10">
+        <v/>
+      </c>
+      <c r="O131" s="10" t="str">
         <f t="shared" si="20"/>
-        <v>7.09</v>
-      </c>
-      <c r="P131" s="7">
+        <v/>
+      </c>
+      <c r="P131" s="7" t="str">
         <f t="shared" si="21"/>
-        <v>7146.72</v>
-      </c>
-      <c r="Q131" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="R131" s="5">
+        <v/>
+      </c>
+      <c r="Q131" s="9"/>
+      <c r="R131" s="5" t="str">
         <f t="shared" si="22"/>
-        <v>46380</v>
-      </c>
-      <c r="S131" s="5">
+        <v/>
+      </c>
+      <c r="S131" s="5" t="str">
         <f t="shared" si="23"/>
-        <v>46377</v>
-      </c>
-      <c r="T131" s="7">
-        <f t="shared" ca="1" si="24"/>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="T131" s="7" t="str">
+        <f t="shared" si="24"/>
+        <v/>
       </c>
       <c r="U131" t="str">
         <f t="shared" si="25"/>
@@ -30500,11 +30486,11 @@
       </c>
       <c r="D8" s="7">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="2"/>
-        <v>18840</v>
+        <v>17904</v>
       </c>
       <c r="F8" s="7">
         <f>ROUND(Demanda!H8,0)</f>
@@ -30512,7 +30498,7 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" si="3"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="H8" s="7">
         <f ca="1">SUM($K$6:K7)*CajasProm</f>
@@ -30520,7 +30506,7 @@
       </c>
       <c r="I8" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="J8" s="21">
         <f t="shared" si="5"/>
@@ -30532,11 +30518,11 @@
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="M8" s="22">
         <f ca="1">IF(Demanda!H9=0,"",L8/(Demanda!H9/DiasVenta))</f>
-        <v>8.7310588235294109</v>
+        <v>8.4007058823529412</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30544,11 +30530,11 @@
       </c>
       <c r="O8" s="7">
         <f>O7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L8,0)</f>
-        <v>11460</v>
+        <v>10524</v>
       </c>
       <c r="P8" s="22">
         <f>IF(Demanda!L9=0,"",O8/(Demanda!L9/DiasVenta))</f>
-        <v>6.555439031366193</v>
+        <v>6.0200209743540851</v>
       </c>
       <c r="Q8" s="7">
         <f>Q7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M8,0)</f>
@@ -30582,7 +30568,7 @@
       </c>
       <c r="C9" s="7">
         <f t="shared" si="10"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="1"/>
@@ -30598,7 +30584,7 @@
       </c>
       <c r="G9" s="7">
         <f t="shared" si="3"/>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="H9" s="7">
         <f ca="1">SUM($K$6:K8)*CajasProm</f>
@@ -30606,7 +30592,7 @@
       </c>
       <c r="I9" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="J9" s="21">
         <f t="shared" si="5"/>
@@ -30614,27 +30600,27 @@
       </c>
       <c r="K9" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22614</v>
+        <v>22678</v>
       </c>
       <c r="M9" s="22">
         <f ca="1">IF(Demanda!H10=0,"",L9/(Demanda!H10/DiasVenta))</f>
-        <v>7.9814117647058822</v>
+        <v>8.0039999999999996</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 4</v>
+        <v>CARGAR 5</v>
       </c>
       <c r="O9" s="7">
         <f>O8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L9,0)</f>
-        <v>6947</v>
+        <v>6011</v>
       </c>
       <c r="P9" s="22">
         <f>IF(Demanda!L10=0,"",O9/(Demanda!L10/DiasVenta))</f>
-        <v>3.9738773953665745</v>
+        <v>3.4384593383544666</v>
       </c>
       <c r="Q9" s="7">
         <f>Q8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M9,0)</f>
@@ -30668,7 +30654,7 @@
       </c>
       <c r="C10" s="7">
         <f t="shared" si="10"/>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
@@ -30684,15 +30670,15 @@
       </c>
       <c r="G10" s="7">
         <f t="shared" si="3"/>
-        <v>14578</v>
+        <v>13642</v>
       </c>
       <c r="H10" s="7">
         <f ca="1">SUM($K$6:K9)*CajasProm</f>
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="I10" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>18578</v>
+        <v>18642</v>
       </c>
       <c r="J10" s="21">
         <f t="shared" si="5"/>
@@ -30704,11 +30690,11 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22578</v>
+        <v>22642</v>
       </c>
       <c r="M10" s="22">
         <f ca="1">IF(Demanda!H11=0,"",L10/(Demanda!H11/DiasVenta))</f>
-        <v>7.9687058823529409</v>
+        <v>7.9912941176470582</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30716,11 +30702,11 @@
       </c>
       <c r="O10" s="7">
         <f>O9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L10,0)</f>
-        <v>4522</v>
+        <v>3586</v>
       </c>
       <c r="P10" s="22">
         <f>IF(Demanda!L11=0,"",O10/(Demanda!L11/DiasVenta))</f>
-        <v>2.586709886547812</v>
+        <v>2.0512918295357041</v>
       </c>
       <c r="Q10" s="7">
         <f>Q9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M10,0)</f>
@@ -30754,7 +30740,7 @@
       </c>
       <c r="C11" s="7">
         <f t="shared" si="10"/>
-        <v>14578</v>
+        <v>13642</v>
       </c>
       <c r="D11" s="7">
         <f t="shared" si="1"/>
@@ -30770,15 +30756,15 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" si="3"/>
-        <v>5642</v>
+        <v>4706</v>
       </c>
       <c r="H11" s="7">
         <f ca="1">SUM($K$6:K10)*CajasProm</f>
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="I11" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13642</v>
+        <v>13706</v>
       </c>
       <c r="J11" s="21">
         <f t="shared" si="5"/>
@@ -30790,11 +30776,11 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22642</v>
+        <v>22706</v>
       </c>
       <c r="M11" s="22">
         <f ca="1">IF(Demanda!H12=0,"",L11/(Demanda!H12/DiasVenta))</f>
-        <v>7.9912941176470582</v>
+        <v>8.0138823529411756</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30802,11 +30788,11 @@
       </c>
       <c r="O11" s="7">
         <f>O10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L11,0)</f>
-        <v>2097</v>
+        <v>1161</v>
       </c>
       <c r="P11" s="22">
         <f>IF(Demanda!L12=0,"",O11/(Demanda!L12/DiasVenta))</f>
-        <v>1.1995423777290495</v>
+        <v>0.6641243207169415</v>
       </c>
       <c r="Q11" s="7">
         <f>Q10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M11,0)</f>
@@ -30840,7 +30826,7 @@
       </c>
       <c r="C12" s="7">
         <f t="shared" si="10"/>
-        <v>5642</v>
+        <v>4706</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="1"/>
@@ -30856,15 +30842,15 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" si="3"/>
-        <v>-3294</v>
+        <v>-4230</v>
       </c>
       <c r="H12" s="7">
         <f ca="1">SUM($K$6:K11)*CajasProm</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13706</v>
+        <v>13770</v>
       </c>
       <c r="J12" s="21">
         <f t="shared" si="5"/>
@@ -30876,11 +30862,11 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22706</v>
+        <v>22770</v>
       </c>
       <c r="M12" s="22">
         <f ca="1">IF(Demanda!H13=0,"",L12/(Demanda!H13/DiasVenta))</f>
-        <v>8.0138823529411756</v>
+        <v>8.0364705882352929</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30888,11 +30874,11 @@
       </c>
       <c r="O12" s="7">
         <f>O11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L12,0)</f>
-        <v>-328</v>
+        <v>-1264</v>
       </c>
       <c r="P12" s="22">
         <f>IF(Demanda!L13=0,"",O12/(Demanda!L13/DiasVenta))</f>
-        <v>-0.18762513108971302</v>
+        <v>-0.72304318810182089</v>
       </c>
       <c r="Q12" s="7">
         <f>Q11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M12,0)</f>
@@ -30926,7 +30912,7 @@
       </c>
       <c r="C13" s="7">
         <f t="shared" si="10"/>
-        <v>-3294</v>
+        <v>-4230</v>
       </c>
       <c r="D13" s="7">
         <f t="shared" si="1"/>
@@ -30942,15 +30928,15 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" si="3"/>
-        <v>-12230</v>
+        <v>-13166</v>
       </c>
       <c r="H13" s="7">
         <f ca="1">SUM($K$6:K12)*CajasProm</f>
-        <v>26000</v>
+        <v>27000</v>
       </c>
       <c r="I13" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13770</v>
+        <v>13834</v>
       </c>
       <c r="J13" s="21">
         <f t="shared" si="5"/>
@@ -30962,11 +30948,11 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22770</v>
+        <v>22834</v>
       </c>
       <c r="M13" s="22">
         <f ca="1">IF(Demanda!H14=0,"",L13/(Demanda!H14/DiasVenta))</f>
-        <v>8.0364705882352929</v>
+        <v>8.0590588235294121</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30974,11 +30960,11 @@
       </c>
       <c r="O13" s="7">
         <f>O12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L13,0)</f>
-        <v>-2753</v>
+        <v>-3689</v>
       </c>
       <c r="P13" s="22">
         <f>IF(Demanda!L14=0,"",O13/(Demanda!L14/DiasVenta))</f>
-        <v>-1.5747926399084755</v>
+        <v>-2.1102106969205834</v>
       </c>
       <c r="Q13" s="7">
         <f>Q12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M13,0)</f>
@@ -31012,7 +30998,7 @@
       </c>
       <c r="C14" s="7">
         <f t="shared" si="10"/>
-        <v>-12230</v>
+        <v>-13166</v>
       </c>
       <c r="D14" s="7">
         <f t="shared" si="1"/>
@@ -31028,15 +31014,15 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" si="3"/>
-        <v>-21166</v>
+        <v>-22102</v>
       </c>
       <c r="H14" s="7">
         <f ca="1">SUM($K$6:K13)*CajasProm</f>
-        <v>35000</v>
+        <v>36000</v>
       </c>
       <c r="I14" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13834</v>
+        <v>13898</v>
       </c>
       <c r="J14" s="21">
         <f t="shared" si="5"/>
@@ -31048,11 +31034,11 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22834</v>
+        <v>22898</v>
       </c>
       <c r="M14" s="22">
         <f ca="1">IF(Demanda!H15=0,"",L14/(Demanda!H15/DiasVenta))</f>
-        <v>8.0590588235294121</v>
+        <v>8.0816470588235294</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31060,11 +31046,11 @@
       </c>
       <c r="O14" s="7">
         <f>O13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L14,0)</f>
-        <v>-5178</v>
+        <v>-6114</v>
       </c>
       <c r="P14" s="22">
         <f>IF(Demanda!L15=0,"",O14/(Demanda!L15/DiasVenta))</f>
-        <v>-2.961960148727238</v>
+        <v>-3.4973782057393459</v>
       </c>
       <c r="Q14" s="7">
         <f>Q13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M14,0)</f>
@@ -31098,7 +31084,7 @@
       </c>
       <c r="C15" s="7">
         <f t="shared" si="10"/>
-        <v>-21166</v>
+        <v>-22102</v>
       </c>
       <c r="D15" s="7">
         <f t="shared" si="1"/>
@@ -31114,15 +31100,15 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" si="3"/>
-        <v>-30102</v>
+        <v>-31038</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">SUM($K$6:K14)*CajasProm</f>
-        <v>44000</v>
+        <v>45000</v>
       </c>
       <c r="I15" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13898</v>
+        <v>13962</v>
       </c>
       <c r="J15" s="21">
         <f t="shared" si="5"/>
@@ -31134,11 +31120,11 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22898</v>
+        <v>22962</v>
       </c>
       <c r="M15" s="22">
         <f ca="1">IF(Demanda!H16=0,"",L15/(Demanda!H16/DiasVenta))</f>
-        <v>8.0816470588235294</v>
+        <v>8.1042352941176468</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31146,11 +31132,11 @@
       </c>
       <c r="O15" s="7">
         <f>O14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L15,0)</f>
-        <v>-7603</v>
+        <v>-8539</v>
       </c>
       <c r="P15" s="22">
         <f>IF(Demanda!L16=0,"",O15/(Demanda!L16/DiasVenta))</f>
-        <v>-4.3491276575460001</v>
+        <v>-4.8845457145581079</v>
       </c>
       <c r="Q15" s="7">
         <f>Q14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M15,0)</f>
@@ -31184,7 +31170,7 @@
       </c>
       <c r="C16" s="7">
         <f t="shared" si="10"/>
-        <v>-30102</v>
+        <v>-31038</v>
       </c>
       <c r="D16" s="7">
         <f t="shared" si="1"/>
@@ -31200,15 +31186,15 @@
       </c>
       <c r="G16" s="7">
         <f t="shared" si="3"/>
-        <v>-39038</v>
+        <v>-39974</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">SUM($K$6:K15)*CajasProm</f>
-        <v>53000</v>
+        <v>54000</v>
       </c>
       <c r="I16" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>13962</v>
+        <v>14026</v>
       </c>
       <c r="J16" s="21">
         <f t="shared" si="5"/>
@@ -31220,11 +31206,11 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22962</v>
+        <v>23026</v>
       </c>
       <c r="M16" s="22">
         <f ca="1">IF(Demanda!H17=0,"",L16/(Demanda!H17/DiasVenta))</f>
-        <v>8.1042352941176468</v>
+        <v>8.1268235294117641</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31232,11 +31218,11 @@
       </c>
       <c r="O16" s="7">
         <f>O15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L16,0)</f>
-        <v>-10028</v>
+        <v>-10964</v>
       </c>
       <c r="P16" s="22">
         <f>IF(Demanda!L17=0,"",O16/(Demanda!L17/DiasVenta))</f>
-        <v>-5.736295166364763</v>
+        <v>-6.2717132233768709</v>
       </c>
       <c r="Q16" s="7">
         <f>Q15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M16,0)</f>
@@ -31270,7 +31256,7 @@
       </c>
       <c r="C17" s="7">
         <f t="shared" si="10"/>
-        <v>-39038</v>
+        <v>-39974</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="1"/>
@@ -31286,15 +31272,15 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>-47974</v>
+        <v>-48910</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">SUM($K$6:K16)*CajasProm</f>
-        <v>62000</v>
+        <v>63000</v>
       </c>
       <c r="I17" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>14026</v>
+        <v>14090</v>
       </c>
       <c r="J17" s="21">
         <f t="shared" si="5"/>
@@ -31306,11 +31292,11 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>23026</v>
+        <v>23090</v>
       </c>
       <c r="M17" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L17/(Demanda!H18/DiasVenta))</f>
-        <v>8.1268235294117641</v>
+        <v>8.1494117647058815</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31318,11 +31304,11 @@
       </c>
       <c r="O17" s="7">
         <f>O16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L17,0)</f>
-        <v>-12453</v>
+        <v>-13389</v>
       </c>
       <c r="P17" s="22">
         <f>IF(Demanda!L18=0,"",O17/(Demanda!L18/DiasVenta))</f>
-        <v>-7.1234626751835251</v>
+        <v>-7.6588807321956329</v>
       </c>
       <c r="Q17" s="7">
         <f>Q16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M17,0)</f>
@@ -31356,7 +31342,7 @@
       </c>
       <c r="C18" s="7">
         <f t="shared" si="10"/>
-        <v>-47974</v>
+        <v>-48910</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="1"/>
@@ -31372,15 +31358,15 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" si="3"/>
-        <v>-56910</v>
+        <v>-57846</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">SUM($K$6:K17)*CajasProm</f>
-        <v>71000</v>
+        <v>72000</v>
       </c>
       <c r="I18" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>14090</v>
+        <v>14154</v>
       </c>
       <c r="J18" s="21">
         <f t="shared" si="5"/>
@@ -31392,11 +31378,11 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>23090</v>
+        <v>23154</v>
       </c>
       <c r="M18" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L18/(Demanda!H18/DiasVenta))</f>
-        <v>8.1494117647058815</v>
+        <v>8.1719999999999988</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31404,11 +31390,11 @@
       </c>
       <c r="O18" s="7">
         <f>O17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L18,0)</f>
-        <v>-14878</v>
+        <v>-15814</v>
       </c>
       <c r="P18" s="22">
         <f>IF(Demanda!L18=0,"",O18/(Demanda!L18/DiasVenta))</f>
-        <v>-8.510630184002288</v>
+        <v>-9.046048241014395</v>
       </c>
       <c r="Q18" s="7">
         <f>Q17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M18,0)</f>
@@ -31634,7 +31620,7 @@
       </c>
       <c r="B8" s="7">
         <f ca="1">IF(A8="","",Proyeccion!I8)</f>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="C8" s="3">
         <f ca="1">IF(A8="","",Proyeccion!K8)</f>
@@ -31654,7 +31640,7 @@
       </c>
       <c r="G8" s="22">
         <f ca="1">IF(A8="","",Proyeccion!M8)</f>
-        <v>8.7310588235294109</v>
+        <v>8.4007058823529412</v>
       </c>
       <c r="H8" t="str">
         <f ca="1">IF(A8="","",Proyeccion!N8)</f>
@@ -31662,7 +31648,7 @@
       </c>
       <c r="I8" t="str">
         <f ca="1">IF(A8="","","Sab "&amp;TEXT(A8,"dd/mm")&amp;": "&amp;FIXED(B8,0)&amp;" cajas - descargan "&amp;Proyeccion!D8&amp;" - vende "&amp;FIXED(Proyeccion!F8,0)&amp;IF(C8&gt;0," -&gt; cargar "&amp;C8&amp;" mas hasta el "&amp;TEXT(Proyeccion!J8,"dd/mm")&amp;" ("&amp;E8&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 10/10: 24.738 cajas - descargan 19 - vende 17.000 -&gt; ok</v>
+        <v>Sab 10/10: 23.802 cajas - descargan 18 - vende 17.000 -&gt; ok</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -31672,11 +31658,11 @@
       </c>
       <c r="B9" s="7">
         <f ca="1">IF(A9="","",Proyeccion!I9)</f>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="C9" s="3">
         <f ca="1">IF(A9="","",Proyeccion!K9)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="str">
         <f ca="1">IF(A9="","","BR "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B9-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B9-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31692,15 +31678,15 @@
       </c>
       <c r="G9" s="22">
         <f ca="1">IF(A9="","",Proyeccion!M9)</f>
-        <v>7.9814117647058822</v>
+        <v>8.0039999999999996</v>
       </c>
       <c r="H9" t="str">
         <f ca="1">IF(A9="","",Proyeccion!N9)</f>
-        <v>CARGAR 4</v>
+        <v>CARGAR 5</v>
       </c>
       <c r="I9" t="str">
         <f ca="1">IF(A9="","","Sab "&amp;TEXT(A9,"dd/mm")&amp;": "&amp;FIXED(B9,0)&amp;" cajas - descargan "&amp;Proyeccion!D9&amp;" - vende "&amp;FIXED(Proyeccion!F9,0)&amp;IF(C9&gt;0," -&gt; cargar "&amp;C9&amp;" mas hasta el "&amp;TEXT(Proyeccion!J9,"dd/mm")&amp;" ("&amp;E9&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 17/10: 18.614 cajas - descargan 11 - vende 17.000 -&gt; cargar 4 mas hasta el 13/10 (Bolivia; BR hasta el 14/10)</v>
+        <v>Sab 17/10: 17.678 cajas - descargan 11 - vende 17.000 -&gt; cargar 5 mas hasta el 13/10 (Bolivia; BR hasta el 14/10)</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -31710,7 +31696,7 @@
       </c>
       <c r="B10" s="7">
         <f ca="1">IF(A10="","",Proyeccion!I10)</f>
-        <v>18578</v>
+        <v>18642</v>
       </c>
       <c r="C10" s="3">
         <f ca="1">IF(A10="","",Proyeccion!K10)</f>
@@ -31730,7 +31716,7 @@
       </c>
       <c r="G10" s="22">
         <f ca="1">IF(A10="","",Proyeccion!M10)</f>
-        <v>7.9687058823529409</v>
+        <v>7.9912941176470582</v>
       </c>
       <c r="H10" t="str">
         <f ca="1">IF(A10="","",Proyeccion!N10)</f>
@@ -31738,7 +31724,7 @@
       </c>
       <c r="I10" t="str">
         <f ca="1">IF(A10="","","Sab "&amp;TEXT(A10,"dd/mm")&amp;": "&amp;FIXED(B10,0)&amp;" cajas - descargan "&amp;Proyeccion!D10&amp;" - vende "&amp;FIXED(Proyeccion!F10,0)&amp;IF(C10&gt;0," -&gt; cargar "&amp;C10&amp;" mas hasta el "&amp;TEXT(Proyeccion!J10,"dd/mm")&amp;" ("&amp;E10&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B10-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 24/10: 18.578 cajas - descargan 13 - vende 17.000 -&gt; cargar 4 mas hasta el 20/10 (Bolivia; BR hasta el 21/10)</v>
+        <v>Sab 24/10: 18.642 cajas - descargan 13 - vende 17.000 -&gt; cargar 4 mas hasta el 20/10 (Bolivia; BR hasta el 21/10)</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -31748,7 +31734,7 @@
       </c>
       <c r="B11" s="7">
         <f ca="1">IF(A11="","",Proyeccion!I11)</f>
-        <v>13642</v>
+        <v>13706</v>
       </c>
       <c r="C11" s="3">
         <f ca="1">IF(A11="","",Proyeccion!K11)</f>
@@ -31768,7 +31754,7 @@
       </c>
       <c r="G11" s="22">
         <f ca="1">IF(A11="","",Proyeccion!M11)</f>
-        <v>7.9912941176470582</v>
+        <v>8.0138823529411756</v>
       </c>
       <c r="H11" t="str">
         <f ca="1">IF(A11="","",Proyeccion!N11)</f>
@@ -31776,7 +31762,7 @@
       </c>
       <c r="I11" t="str">
         <f ca="1">IF(A11="","","Sab "&amp;TEXT(A11,"dd/mm")&amp;": "&amp;FIXED(B11,0)&amp;" cajas - descargan "&amp;Proyeccion!D11&amp;" - vende "&amp;FIXED(Proyeccion!F11,0)&amp;IF(C11&gt;0," -&gt; cargar "&amp;C11&amp;" mas hasta el "&amp;TEXT(Proyeccion!J11,"dd/mm")&amp;" ("&amp;E11&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B11-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 31/10: 13.642 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 27/10 (Bolivia; BR hasta el 28/10)</v>
+        <v>Sab 31/10: 13.706 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 27/10 (Bolivia; BR hasta el 28/10)</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -31786,7 +31772,7 @@
       </c>
       <c r="B12" s="7">
         <f ca="1">IF(A12="","",Proyeccion!I12)</f>
-        <v>13706</v>
+        <v>13770</v>
       </c>
       <c r="C12" s="3">
         <f ca="1">IF(A12="","",Proyeccion!K12)</f>
@@ -31806,7 +31792,7 @@
       </c>
       <c r="G12" s="22">
         <f ca="1">IF(A12="","",Proyeccion!M12)</f>
-        <v>8.0138823529411756</v>
+        <v>8.0364705882352929</v>
       </c>
       <c r="H12" t="str">
         <f ca="1">IF(A12="","",Proyeccion!N12)</f>
@@ -31814,7 +31800,7 @@
       </c>
       <c r="I12" t="str">
         <f ca="1">IF(A12="","","Sab "&amp;TEXT(A12,"dd/mm")&amp;": "&amp;FIXED(B12,0)&amp;" cajas - descargan "&amp;Proyeccion!D12&amp;" - vende "&amp;FIXED(Proyeccion!F12,0)&amp;IF(C12&gt;0," -&gt; cargar "&amp;C12&amp;" mas hasta el "&amp;TEXT(Proyeccion!J12,"dd/mm")&amp;" ("&amp;E12&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B12-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 07/11: 13.706 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
+        <v>Sab 07/11: 13.770 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -31824,7 +31810,7 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IF(A13="","",Proyeccion!I13)</f>
-        <v>13770</v>
+        <v>13834</v>
       </c>
       <c r="C13" s="3">
         <f ca="1">IF(A13="","",Proyeccion!K13)</f>
@@ -31844,7 +31830,7 @@
       </c>
       <c r="G13" s="22">
         <f ca="1">IF(A13="","",Proyeccion!M13)</f>
-        <v>8.0364705882352929</v>
+        <v>8.0590588235294121</v>
       </c>
       <c r="H13" t="str">
         <f ca="1">IF(A13="","",Proyeccion!N13)</f>
@@ -31852,7 +31838,7 @@
       </c>
       <c r="I13" t="str">
         <f ca="1">IF(A13="","","Sab "&amp;TEXT(A13,"dd/mm")&amp;": "&amp;FIXED(B13,0)&amp;" cajas - descargan "&amp;Proyeccion!D13&amp;" - vende "&amp;FIXED(Proyeccion!F13,0)&amp;IF(C13&gt;0," -&gt; cargar "&amp;C13&amp;" mas hasta el "&amp;TEXT(Proyeccion!J13,"dd/mm")&amp;" ("&amp;E13&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 14/11: 13.770 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
+        <v>Sab 14/11: 13.834 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -31862,7 +31848,7 @@
       </c>
       <c r="B14" s="7">
         <f ca="1">IF(A14="","",Proyeccion!I14)</f>
-        <v>13834</v>
+        <v>13898</v>
       </c>
       <c r="C14" s="3">
         <f ca="1">IF(A14="","",Proyeccion!K14)</f>
@@ -31882,7 +31868,7 @@
       </c>
       <c r="G14" s="22">
         <f ca="1">IF(A14="","",Proyeccion!M14)</f>
-        <v>8.0590588235294121</v>
+        <v>8.0816470588235294</v>
       </c>
       <c r="H14" t="str">
         <f ca="1">IF(A14="","",Proyeccion!N14)</f>
@@ -31890,7 +31876,7 @@
       </c>
       <c r="I14" t="str">
         <f ca="1">IF(A14="","","Sab "&amp;TEXT(A14,"dd/mm")&amp;": "&amp;FIXED(B14,0)&amp;" cajas - descargan "&amp;Proyeccion!D14&amp;" - vende "&amp;FIXED(Proyeccion!F14,0)&amp;IF(C14&gt;0," -&gt; cargar "&amp;C14&amp;" mas hasta el "&amp;TEXT(Proyeccion!J14,"dd/mm")&amp;" ("&amp;E14&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 21/11: 13.834 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
+        <v>Sab 21/11: 13.898 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -31900,7 +31886,7 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(A15="","",Proyeccion!I15)</f>
-        <v>13898</v>
+        <v>13962</v>
       </c>
       <c r="C15" s="3">
         <f ca="1">IF(A15="","",Proyeccion!K15)</f>
@@ -31920,7 +31906,7 @@
       </c>
       <c r="G15" s="22">
         <f ca="1">IF(A15="","",Proyeccion!M15)</f>
-        <v>8.0816470588235294</v>
+        <v>8.1042352941176468</v>
       </c>
       <c r="H15" t="str">
         <f ca="1">IF(A15="","",Proyeccion!N15)</f>
@@ -31928,7 +31914,7 @@
       </c>
       <c r="I15" t="str">
         <f ca="1">IF(A15="","","Sab "&amp;TEXT(A15,"dd/mm")&amp;": "&amp;FIXED(B15,0)&amp;" cajas - descargan "&amp;Proyeccion!D15&amp;" - vende "&amp;FIXED(Proyeccion!F15,0)&amp;IF(C15&gt;0," -&gt; cargar "&amp;C15&amp;" mas hasta el "&amp;TEXT(Proyeccion!J15,"dd/mm")&amp;" ("&amp;E15&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B15-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 28/11: 13.898 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
+        <v>Sab 28/11: 13.962 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -31938,7 +31924,7 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(A16="","",Proyeccion!I16)</f>
-        <v>13962</v>
+        <v>14026</v>
       </c>
       <c r="C16" s="3">
         <f ca="1">IF(A16="","",Proyeccion!K16)</f>
@@ -31958,7 +31944,7 @@
       </c>
       <c r="G16" s="22">
         <f ca="1">IF(A16="","",Proyeccion!M16)</f>
-        <v>8.1042352941176468</v>
+        <v>8.1268235294117641</v>
       </c>
       <c r="H16" t="str">
         <f ca="1">IF(A16="","",Proyeccion!N16)</f>
@@ -31966,7 +31952,7 @@
       </c>
       <c r="I16" t="str">
         <f ca="1">IF(A16="","","Sab "&amp;TEXT(A16,"dd/mm")&amp;": "&amp;FIXED(B16,0)&amp;" cajas - descargan "&amp;Proyeccion!D16&amp;" - vende "&amp;FIXED(Proyeccion!F16,0)&amp;IF(C16&gt;0," -&gt; cargar "&amp;C16&amp;" mas hasta el "&amp;TEXT(Proyeccion!J16,"dd/mm")&amp;" ("&amp;E16&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B16-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 05/12: 13.962 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
+        <v>Sab 05/12: 14.026 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -31976,7 +31962,7 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(A17="","",Proyeccion!I17)</f>
-        <v>14026</v>
+        <v>14090</v>
       </c>
       <c r="C17" s="3">
         <f ca="1">IF(A17="","",Proyeccion!K17)</f>
@@ -31996,7 +31982,7 @@
       </c>
       <c r="G17" s="22">
         <f ca="1">IF(A17="","",Proyeccion!M17)</f>
-        <v>8.1268235294117641</v>
+        <v>8.1494117647058815</v>
       </c>
       <c r="H17" t="str">
         <f ca="1">IF(A17="","",Proyeccion!N17)</f>
@@ -32004,7 +31990,7 @@
       </c>
       <c r="I17" t="str">
         <f ca="1">IF(A17="","","Sab "&amp;TEXT(A17,"dd/mm")&amp;": "&amp;FIXED(B17,0)&amp;" cajas - descargan "&amp;Proyeccion!D17&amp;" - vende "&amp;FIXED(Proyeccion!F17,0)&amp;IF(C17&gt;0," -&gt; cargar "&amp;C17&amp;" mas hasta el "&amp;TEXT(Proyeccion!J17,"dd/mm")&amp;" ("&amp;E17&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B17-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 12/12: 14.026 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
+        <v>Sab 12/12: 14.090 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -32014,7 +32000,7 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(A18="","",Proyeccion!I18)</f>
-        <v>14090</v>
+        <v>14154</v>
       </c>
       <c r="C18" s="3">
         <f ca="1">IF(A18="","",Proyeccion!K18)</f>
@@ -32034,7 +32020,7 @@
       </c>
       <c r="G18" s="22">
         <f ca="1">IF(A18="","",Proyeccion!M18)</f>
-        <v>8.1494117647058815</v>
+        <v>8.1719999999999988</v>
       </c>
       <c r="H18" t="str">
         <f ca="1">IF(A18="","",Proyeccion!N18)</f>
@@ -32042,7 +32028,7 @@
       </c>
       <c r="I18" t="str">
         <f ca="1">IF(A18="","","Sab "&amp;TEXT(A18,"dd/mm")&amp;": "&amp;FIXED(B18,0)&amp;" cajas - descargan "&amp;Proyeccion!D18&amp;" - vende "&amp;FIXED(Proyeccion!F18,0)&amp;IF(C18&gt;0," -&gt; cargar "&amp;C18&amp;" mas hasta el "&amp;TEXT(Proyeccion!J18,"dd/mm")&amp;" ("&amp;E18&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B18-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 19/12: 14.090 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
+        <v>Sab 19/12: 14.154 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="33.950000000000003" customHeight="1">
@@ -32267,11 +32253,11 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>11460</v>
+        <v>10524</v>
       </c>
       <c r="C13" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>6.555439031366193</v>
+        <v>6.0200209743540851</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(B13="","",IF(B13&lt;0,"FALTA",IF(C13&lt;2,"CRITICO",IF(C13&lt;CoberturaObjetivo,"JUSTO",IF(C13&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32330,11 +32316,11 @@
       </c>
       <c r="B16" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="C16" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>8.7310588235294109</v>
+        <v>8.4007058823529412</v>
       </c>
       <c r="D16" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
@@ -32378,11 +32364,11 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>6947</v>
+        <v>6011</v>
       </c>
       <c r="C20" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>3.9738773953665745</v>
+        <v>3.4384593383544666</v>
       </c>
       <c r="D20" t="str">
         <f ca="1">IF(B20="","",IF(B20&lt;0,"FALTA",IF(C20&lt;2,"CRITICO",IF(C20&lt;CoberturaObjetivo,"JUSTO",IF(C20&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32441,19 +32427,19 @@
       </c>
       <c r="B23" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="C23" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>7.9814117647058822</v>
+        <v>8.0039999999999996</v>
       </c>
       <c r="D23" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>CARGAR 4</v>
+        <v>CARGAR 5</v>
       </c>
       <c r="E23" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 4 camion(es) mas hasta el mar 13/10 para cerrar en 22.500</v>
+        <v>cargar 5 camion(es) mas hasta el mar 13/10 para cerrar en 22.500</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30">
@@ -32498,7 +32484,7 @@
     <row r="29" spans="1:5">
       <c r="A29" s="45" t="str">
         <f>"Dictados que Aloha aun no tiene: "&amp;COUNTIFS(CgEstado,"Dictado",CgCuenta,1)&amp;" camiones. Pasan a Aloha cuando se cargan en el sistema."</f>
-        <v>Dictados que Aloha aun no tiene: 33 camiones. Pasan a Aloha cuando se cargan en el sistema.</v>
+        <v>Dictados que Aloha aun no tiene: 32 camiones. Pasan a Aloha cuando se cargan en el sistema.</v>
       </c>
       <c r="B29" s="46"/>
       <c r="C29" s="46"/>
@@ -32508,7 +32494,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 18.866 cajas (4.032 menos que el plan) y el 10/10 en 18.790 (plan: 24.738).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 18.866 cajas (4.032 menos que el plan) y el 10/10 en 18.790 (plan: 23.802).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32825,7 +32811,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>18840</v>
+        <v>17904</v>
       </c>
       <c r="D8" s="7">
         <f>Proyeccion!F8</f>
@@ -32833,7 +32819,7 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>28038</v>
+        <v>27102</v>
       </c>
       <c r="F8">
         <f ca="1">IF(AND(E8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-E8)/CajasProm,0),0)</f>
@@ -32841,7 +32827,7 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
       <c r="H8">
         <f ca="1">IF(AND(G8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-G8)/CajasProm,0),0)</f>
@@ -32849,7 +32835,7 @@
       </c>
       <c r="I8" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>21438</v>
+        <v>20502</v>
       </c>
       <c r="J8">
         <f ca="1">IF(AND(I8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-I8)/CajasProm,0),0)</f>
@@ -32869,15 +32855,15 @@
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>21798</v>
+        <v>20862</v>
       </c>
       <c r="O8" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>23738</v>
+        <v>22802</v>
       </c>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>24738</v>
+        <v>23802</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -32899,7 +32885,7 @@
       </c>
       <c r="E9" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>23614</v>
+        <v>22678</v>
       </c>
       <c r="F9">
         <f ca="1">IF(AND(E9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-E9)/CajasProm,0),0)</f>
@@ -32907,43 +32893,43 @@
       </c>
       <c r="G9" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>18614</v>
+        <v>17678</v>
       </c>
       <c r="H9">
         <f ca="1">IF(AND(G9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-G9)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I9" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>15614</v>
+        <v>14678</v>
       </c>
       <c r="J9">
         <f ca="1">IF(AND(I9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-I9)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
-        <v>16824</v>
+        <v>15888</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22614</v>
+        <v>21678</v>
       </c>
       <c r="M9">
         <f ca="1">IF(AND(L9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-L9)/CajasProm,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>15674</v>
+        <v>14738</v>
       </c>
       <c r="O9" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>17614</v>
+        <v>16678</v>
       </c>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>18614</v>
+        <v>17678</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -32965,15 +32951,15 @@
       </c>
       <c r="E10" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>21278</v>
+        <v>20342</v>
       </c>
       <c r="F10">
         <f ca="1">IF(AND(E10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-E10)/CajasProm,0),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>18578</v>
+        <v>18642</v>
       </c>
       <c r="H10">
         <f ca="1">IF(AND(G10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-G10)/CajasProm,0),0)</f>
@@ -32981,7 +32967,7 @@
       </c>
       <c r="I10" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>16878</v>
+        <v>16942</v>
       </c>
       <c r="J10">
         <f ca="1">IF(AND(I10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-I10)/CajasProm,0),0)</f>
@@ -32993,7 +32979,7 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>18578</v>
+        <v>18642</v>
       </c>
       <c r="M10">
         <f ca="1">IF(AND(L10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-L10)/CajasProm,0),0)</f>
@@ -33001,15 +32987,15 @@
       </c>
       <c r="N10" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>15638</v>
+        <v>15702</v>
       </c>
       <c r="O10" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>17578</v>
+        <v>17642</v>
       </c>
       <c r="P10" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>18578</v>
+        <v>18642</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -33031,7 +33017,7 @@
       </c>
       <c r="E11" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>16042</v>
+        <v>16106</v>
       </c>
       <c r="F11">
         <f ca="1">IF(AND(E11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-E11)/CajasProm,0),0)</f>
@@ -33039,7 +33025,7 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13642</v>
+        <v>13706</v>
       </c>
       <c r="H11">
         <f ca="1">IF(AND(G11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-G11)/CajasProm,0),0)</f>
@@ -33047,7 +33033,7 @@
       </c>
       <c r="I11" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12242</v>
+        <v>12306</v>
       </c>
       <c r="J11">
         <f ca="1">IF(AND(I11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-I11)/CajasProm,0),0)</f>
@@ -33059,7 +33045,7 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13642</v>
+        <v>13706</v>
       </c>
       <c r="M11">
         <f ca="1">IF(AND(L11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-L11)/CajasProm,0),0)</f>
@@ -33067,15 +33053,15 @@
       </c>
       <c r="N11" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>10702</v>
+        <v>10766</v>
       </c>
       <c r="O11" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12642</v>
+        <v>12706</v>
       </c>
       <c r="P11" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13642</v>
+        <v>13706</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -33097,7 +33083,7 @@
       </c>
       <c r="E12" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15806</v>
+        <v>15870</v>
       </c>
       <c r="F12">
         <f ca="1">IF(AND(E12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-E12)/CajasProm,0),0)</f>
@@ -33105,7 +33091,7 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13706</v>
+        <v>13770</v>
       </c>
       <c r="H12">
         <f ca="1">IF(AND(G12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-G12)/CajasProm,0),0)</f>
@@ -33113,7 +33099,7 @@
       </c>
       <c r="I12" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12606</v>
+        <v>12670</v>
       </c>
       <c r="J12">
         <f ca="1">IF(AND(I12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-I12)/CajasProm,0),0)</f>
@@ -33125,7 +33111,7 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13706</v>
+        <v>13770</v>
       </c>
       <c r="M12">
         <f ca="1">IF(AND(L12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-L12)/CajasProm,0),0)</f>
@@ -33133,15 +33119,15 @@
       </c>
       <c r="N12" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>10766</v>
+        <v>10830</v>
       </c>
       <c r="O12" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12706</v>
+        <v>12770</v>
       </c>
       <c r="P12" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13706</v>
+        <v>13770</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -33163,7 +33149,7 @@
       </c>
       <c r="E13" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15570</v>
+        <v>15634</v>
       </c>
       <c r="F13">
         <f ca="1">IF(AND(E13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-E13)/CajasProm,0),0)</f>
@@ -33171,7 +33157,7 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13770</v>
+        <v>13834</v>
       </c>
       <c r="H13">
         <f ca="1">IF(AND(G13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-G13)/CajasProm,0),0)</f>
@@ -33179,7 +33165,7 @@
       </c>
       <c r="I13" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>11970</v>
+        <v>12034</v>
       </c>
       <c r="J13">
         <f ca="1">IF(AND(I13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-I13)/CajasProm,0),0)</f>
@@ -33191,7 +33177,7 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13770</v>
+        <v>13834</v>
       </c>
       <c r="M13">
         <f ca="1">IF(AND(L13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-L13)/CajasProm,0),0)</f>
@@ -33199,15 +33185,15 @@
       </c>
       <c r="N13" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>10830</v>
+        <v>10894</v>
       </c>
       <c r="O13" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12770</v>
+        <v>12834</v>
       </c>
       <c r="P13" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13770</v>
+        <v>13834</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -33229,7 +33215,7 @@
       </c>
       <c r="E14" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15334</v>
+        <v>15398</v>
       </c>
       <c r="F14">
         <f ca="1">IF(AND(E14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-E14)/CajasProm,0),0)</f>
@@ -33237,7 +33223,7 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13834</v>
+        <v>13898</v>
       </c>
       <c r="H14">
         <f ca="1">IF(AND(G14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-G14)/CajasProm,0),0)</f>
@@ -33245,7 +33231,7 @@
       </c>
       <c r="I14" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12334</v>
+        <v>12398</v>
       </c>
       <c r="J14">
         <f ca="1">IF(AND(I14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-I14)/CajasProm,0),0)</f>
@@ -33257,7 +33243,7 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13834</v>
+        <v>13898</v>
       </c>
       <c r="M14">
         <f ca="1">IF(AND(L14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-L14)/CajasProm,0),0)</f>
@@ -33265,15 +33251,15 @@
       </c>
       <c r="N14" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>10894</v>
+        <v>10958</v>
       </c>
       <c r="O14" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12834</v>
+        <v>12898</v>
       </c>
       <c r="P14" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13834</v>
+        <v>13898</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -33295,7 +33281,7 @@
       </c>
       <c r="E15" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>16098</v>
+        <v>16162</v>
       </c>
       <c r="F15">
         <f ca="1">IF(AND(E15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-E15)/CajasProm,0),0)</f>
@@ -33303,7 +33289,7 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13898</v>
+        <v>13962</v>
       </c>
       <c r="H15">
         <f ca="1">IF(AND(G15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-G15)/CajasProm,0),0)</f>
@@ -33311,7 +33297,7 @@
       </c>
       <c r="I15" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12698</v>
+        <v>12762</v>
       </c>
       <c r="J15">
         <f ca="1">IF(AND(I15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-I15)/CajasProm,0),0)</f>
@@ -33323,7 +33309,7 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13898</v>
+        <v>13962</v>
       </c>
       <c r="M15">
         <f ca="1">IF(AND(L15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-L15)/CajasProm,0),0)</f>
@@ -33331,15 +33317,15 @@
       </c>
       <c r="N15" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>10958</v>
+        <v>11022</v>
       </c>
       <c r="O15" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12898</v>
+        <v>12962</v>
       </c>
       <c r="P15" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13898</v>
+        <v>13962</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -33361,7 +33347,7 @@
       </c>
       <c r="E16" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15862</v>
+        <v>15926</v>
       </c>
       <c r="F16">
         <f ca="1">IF(AND(E16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-E16)/CajasProm,0),0)</f>
@@ -33369,7 +33355,7 @@
       </c>
       <c r="G16" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>13962</v>
+        <v>14026</v>
       </c>
       <c r="H16">
         <f ca="1">IF(AND(G16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-G16)/CajasProm,0),0)</f>
@@ -33377,7 +33363,7 @@
       </c>
       <c r="I16" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12062</v>
+        <v>12126</v>
       </c>
       <c r="J16">
         <f ca="1">IF(AND(I16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-I16)/CajasProm,0),0)</f>
@@ -33389,7 +33375,7 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>13962</v>
+        <v>14026</v>
       </c>
       <c r="M16">
         <f ca="1">IF(AND(L16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-L16)/CajasProm,0),0)</f>
@@ -33397,15 +33383,15 @@
       </c>
       <c r="N16" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>11022</v>
+        <v>11086</v>
       </c>
       <c r="O16" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>12962</v>
+        <v>13026</v>
       </c>
       <c r="P16" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13962</v>
+        <v>14026</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -33427,7 +33413,7 @@
       </c>
       <c r="E17" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15626</v>
+        <v>15690</v>
       </c>
       <c r="F17">
         <f ca="1">IF(AND(E17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-E17)/CajasProm,0),0)</f>
@@ -33435,7 +33421,7 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>14026</v>
+        <v>14090</v>
       </c>
       <c r="H17">
         <f ca="1">IF(AND(G17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-G17)/CajasProm,0),0)</f>
@@ -33443,7 +33429,7 @@
       </c>
       <c r="I17" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12426</v>
+        <v>12490</v>
       </c>
       <c r="J17">
         <f ca="1">IF(AND(I17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-I17)/CajasProm,0),0)</f>
@@ -33455,7 +33441,7 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>14026</v>
+        <v>14090</v>
       </c>
       <c r="M17">
         <f ca="1">IF(AND(L17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-L17)/CajasProm,0),0)</f>
@@ -33463,15 +33449,15 @@
       </c>
       <c r="N17" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>11086</v>
+        <v>11150</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>13026</v>
+        <v>13090</v>
       </c>
       <c r="P17" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14026</v>
+        <v>14090</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -33493,7 +33479,7 @@
       </c>
       <c r="E18" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>15390</v>
+        <v>15454</v>
       </c>
       <c r="F18">
         <f ca="1">IF(AND(E18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-E18)/CajasProm,0),0)</f>
@@ -33501,7 +33487,7 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>14090</v>
+        <v>14154</v>
       </c>
       <c r="H18">
         <f ca="1">IF(AND(G18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-G18)/CajasProm,0),0)</f>
@@ -33509,7 +33495,7 @@
       </c>
       <c r="I18" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>12790</v>
+        <v>12854</v>
       </c>
       <c r="J18">
         <f ca="1">IF(AND(I18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-I18)/CajasProm,0),0)</f>
@@ -33521,7 +33507,7 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>14090</v>
+        <v>14154</v>
       </c>
       <c r="M18">
         <f ca="1">IF(AND(L18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-L18)/CajasProm,0),0)</f>
@@ -33529,15 +33515,15 @@
       </c>
       <c r="N18" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>11150</v>
+        <v>11214</v>
       </c>
       <c r="O18" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>13090</v>
+        <v>13154</v>
       </c>
       <c r="P18" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14090</v>
+        <v>14154</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="63.95" customHeight="1">

</xml_diff>

<commit_message>
plan de compras: las descargas de domingo suman a la semana que arranca (WhatsApp, simulador y Excel)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36283C1A-FBB3-4A4B-8CB7-9A1043A13AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9CEF13-A5C3-44BB-ADF2-072D89D470EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -115,7 +115,7 @@
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 01/10/2026 12:30 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 01/10/2026 12:33 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C6" s="7">
         <f>Proyeccion!E6</f>
-        <v>980</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7">
         <f>Demanda!H7</f>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="H6" s="7">
         <f ca="1">Proyeccion!L6</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="I6" s="7" t="str">
         <f t="shared" ref="I6:I18" si="3">IF(CapFisica="","",CapFisica)</f>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="C7" s="7">
         <f>Proyeccion!E7</f>
-        <v>10946</v>
+        <v>11926</v>
       </c>
       <c r="D7" s="7">
         <f>Demanda!H8</f>
@@ -4787,7 +4787,7 @@
       </c>
       <c r="B19" s="24">
         <f ca="1">AVERAGEIFS(PrCamiones,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>13.25</v>
+        <v>13.5</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>320</v>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="B20" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BR",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.62637237396953238</v>
+        <v>0.61492559579308548</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>322</v>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="B21" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"PY",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.35368309083311172</v>
+        <v>0.36549434975571549</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>3</v>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B22" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>1.9944535197355926E-2</v>
+        <v>1.9580054451199046E-2</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>3</v>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="B23" s="12">
         <f ca="1">SUMIFS(CgCosto,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>375479.83999999973</v>
+        <v>382339.83999999973</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>326</v>
@@ -5945,7 +5945,7 @@
       </c>
       <c r="N17">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17">
         <f t="shared" ca="1" si="1"/>
@@ -10100,8 +10100,8 @@
         <v>46292</v>
       </c>
       <c r="M5" s="5">
-        <f t="shared" ref="M5:M68" si="5">IF(L5="","",L5-WEEKDAY(L5,2)+1)</f>
-        <v>46286</v>
+        <f t="shared" ref="M5:M68" si="5">IF(L5="","",IF(WEEKDAY(L5,2)=7,L5+1,L5-WEEKDAY(L5,2)+1))</f>
+        <v>46293</v>
       </c>
       <c r="N5">
         <f t="shared" ref="N5:N68" si="6">IF(L5="","",IF(L5&gt;FechaConteo,1,0)*IF(I5="Supuesto",SupPY,IF(I5="Supuesto BR",SupBR,1)))</f>
@@ -10123,8 +10123,8 @@
         <v>46292</v>
       </c>
       <c r="S5" s="5">
-        <f t="shared" ref="S5:S68" si="10">IF(R5="","",R5-WEEKDAY(R5,2)+1)</f>
-        <v>46286</v>
+        <f t="shared" ref="S5:S68" si="10">IF(R5="","",IF(WEEKDAY(R5,2)=7,R5+1,R5-WEEKDAY(R5,2)+1))</f>
+        <v>46293</v>
       </c>
       <c r="T5" s="7">
         <f t="shared" ref="T5:T68" ca="1" si="11">IF(B5="","",IF(AND(B5&lt;=FechaHoy,J5="",I5&lt;&gt;"Supuesto",I5&lt;&gt;"Simulado"),H5,0))</f>
@@ -10732,7 +10732,7 @@
       </c>
       <c r="S13" s="5">
         <f t="shared" si="10"/>
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="T13" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="S31" s="5">
         <f t="shared" si="10"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="T31" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="S32" s="5">
         <f t="shared" si="10"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="T32" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -14964,7 +14964,7 @@
         <v>46328</v>
       </c>
       <c r="M69" s="5">
-        <f t="shared" ref="M69:M132" si="18">IF(L69="","",L69-WEEKDAY(L69,2)+1)</f>
+        <f t="shared" ref="M69:M132" si="18">IF(L69="","",IF(WEEKDAY(L69,2)=7,L69+1,L69-WEEKDAY(L69,2)+1))</f>
         <v>46328</v>
       </c>
       <c r="N69">
@@ -14987,7 +14987,7 @@
         <v>46331</v>
       </c>
       <c r="S69" s="5">
-        <f t="shared" ref="S69:S132" si="23">IF(R69="","",R69-WEEKDAY(R69,2)+1)</f>
+        <f t="shared" ref="S69:S132" si="23">IF(R69="","",IF(WEEKDAY(R69,2)=7,R69+1,R69-WEEKDAY(R69,2)+1))</f>
         <v>46328</v>
       </c>
       <c r="T69" s="7">
@@ -19788,7 +19788,7 @@
         <v/>
       </c>
       <c r="M133" s="5" t="str">
-        <f t="shared" ref="M133:M196" si="31">IF(L133="","",L133-WEEKDAY(L133,2)+1)</f>
+        <f t="shared" ref="M133:M196" si="31">IF(L133="","",IF(WEEKDAY(L133,2)=7,L133+1,L133-WEEKDAY(L133,2)+1))</f>
         <v/>
       </c>
       <c r="N133" t="str">
@@ -19809,7 +19809,7 @@
         <v/>
       </c>
       <c r="S133" s="5" t="str">
-        <f t="shared" ref="S133:S196" si="36">IF(R133="","",R133-WEEKDAY(R133,2)+1)</f>
+        <f t="shared" ref="S133:S196" si="36">IF(R133="","",IF(WEEKDAY(R133,2)=7,R133+1,R133-WEEKDAY(R133,2)+1))</f>
         <v/>
       </c>
       <c r="T133" s="7" t="str">
@@ -23756,7 +23756,7 @@
         <v/>
       </c>
       <c r="M197" s="5" t="str">
-        <f t="shared" ref="M197:M260" si="44">IF(L197="","",L197-WEEKDAY(L197,2)+1)</f>
+        <f t="shared" ref="M197:M260" si="44">IF(L197="","",IF(WEEKDAY(L197,2)=7,L197+1,L197-WEEKDAY(L197,2)+1))</f>
         <v/>
       </c>
       <c r="N197" t="str">
@@ -23777,7 +23777,7 @@
         <v/>
       </c>
       <c r="S197" s="5" t="str">
-        <f t="shared" ref="S197:S260" si="49">IF(R197="","",R197-WEEKDAY(R197,2)+1)</f>
+        <f t="shared" ref="S197:S260" si="49">IF(R197="","",IF(WEEKDAY(R197,2)=7,R197+1,R197-WEEKDAY(R197,2)+1))</f>
         <v/>
       </c>
       <c r="T197" s="7" t="str">
@@ -27724,7 +27724,7 @@
         <v/>
       </c>
       <c r="M261" s="5" t="str">
-        <f t="shared" ref="M261:M324" si="57">IF(L261="","",L261-WEEKDAY(L261,2)+1)</f>
+        <f t="shared" ref="M261:M324" si="57">IF(L261="","",IF(WEEKDAY(L261,2)=7,L261+1,L261-WEEKDAY(L261,2)+1))</f>
         <v/>
       </c>
       <c r="N261" t="str">
@@ -27745,7 +27745,7 @@
         <v/>
       </c>
       <c r="S261" s="5" t="str">
-        <f t="shared" ref="S261:S324" si="62">IF(R261="","",R261-WEEKDAY(R261,2)+1)</f>
+        <f t="shared" ref="S261:S324" si="62">IF(R261="","",IF(WEEKDAY(R261,2)=7,R261+1,R261-WEEKDAY(R261,2)+1))</f>
         <v/>
       </c>
       <c r="T261" s="7" t="str">
@@ -30317,11 +30317,11 @@
       </c>
       <c r="D6" s="7">
         <f t="shared" ref="D6:D18" si="1">COUNTIFS(CgSemana,A6,CgCuenta,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="7">
         <f t="shared" ref="E6:E18" si="2">SUMIFS(CgCajas,CgSemana,A6,CgCuenta,1)</f>
-        <v>980</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7">
         <f>ROUND(Demanda!H6*MAX(0,MIN(DiasVenta,B6-FechaConteo))/DiasVenta,0)</f>
@@ -30329,7 +30329,7 @@
       </c>
       <c r="G6" s="7">
         <f t="shared" ref="G6:G18" si="3">C6+E6-F6</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="H6" s="7">
         <f>0</f>
@@ -30337,7 +30337,7 @@
       </c>
       <c r="I6" s="12">
         <f t="shared" ref="I6:I18" si="4">G6+H6</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="J6" s="21">
         <f t="shared" ref="J6:J18" si="5">B6-MAX(LagBR,LagPY)-AtrasoDias</f>
@@ -30349,11 +30349,11 @@
       </c>
       <c r="L6" s="7">
         <f t="shared" ref="L6:L18" ca="1" si="7">I6+K6*CajasProm</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="M6" s="22">
         <f ca="1">IF(Demanda!H7=0,"",L6/(Demanda!H7/DiasVenta))</f>
-        <v>10.482000000000001</v>
+        <v>10.114500000000001</v>
       </c>
       <c r="N6" t="str">
         <f t="shared" ref="N6:N18" ca="1" si="8">IF(I6&lt;0,"FALTA",IF(K6&gt;0,"CARGAR "&amp;K6,IF(I6&lt;MinimoSabado,"BAJO MINIMO (limite pasado)",IF(AND(M6&lt;&gt;"",M6&gt;VidaVerde),"EXCESO (merma)","OK"))))</f>
@@ -30369,11 +30369,11 @@
       </c>
       <c r="Q6" s="7">
         <f>ConteoPY+SUMIFS(CgCajas,CgSemana,A6,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M6*MAX(0,MIN(DiasVenta,B6-FechaConteo))/DiasVenta,0)</f>
-        <v>14653</v>
+        <v>13673</v>
       </c>
       <c r="R6" s="22">
         <f>IF(Demanda!M7=0,"",Q6/(Demanda!M7/DiasVenta))</f>
-        <v>13.946383248730964</v>
+        <v>13.013642131979694</v>
       </c>
       <c r="S6" s="7">
         <f>ConteoBO+SUMIFS(CgCajas,CgSemana,A6,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N6*MAX(0,MIN(DiasVenta,B6-FechaConteo))/DiasVenta,0)</f>
@@ -30399,15 +30399,15 @@
       </c>
       <c r="C7" s="7">
         <f t="shared" ref="C7:C18" si="10">G6</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="D7" s="7">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="7">
         <f t="shared" si="2"/>
-        <v>10946</v>
+        <v>11926</v>
       </c>
       <c r="F7" s="7">
         <f>ROUND(Demanda!H7,0)</f>
@@ -32497,7 +32497,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 18.866 cajas (4.032 menos que el plan) y el 10/10 en 18.790 (plan: 24.766).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.830 (plan: 24.766).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="C6" s="7">
         <f>Proyeccion!E6</f>
-        <v>980</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7">
         <f>Proyeccion!F6</f>
@@ -32690,7 +32690,7 @@
       </c>
       <c r="E6" s="7">
         <f>ConteoTotal+C6-ROUND(D6*0.9,0)</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="F6">
         <f ca="1">IF(AND(E6&lt;MinimoSabado,Proyeccion!J6&gt;=FechaHoy),ROUNDUP((MinimoSabado-E6)/CajasProm,0),0)</f>
@@ -32698,7 +32698,7 @@
       </c>
       <c r="G6" s="7">
         <f>ConteoTotal+C6-ROUND(D6*1,0)</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="H6">
         <f ca="1">IF(AND(G6&lt;MinimoSabado,Proyeccion!J6&gt;=FechaHoy),ROUNDUP((MinimoSabado-G6)/CajasProm,0),0)</f>
@@ -32706,7 +32706,7 @@
       </c>
       <c r="I6" s="7">
         <f>ConteoTotal+C6-ROUND(D6*1.1,0)</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="J6">
         <f ca="1">IF(AND(I6&lt;MinimoSabado,Proyeccion!J6&gt;=FechaHoy),ROUNDUP((MinimoSabado-I6)/CajasProm,0),0)</f>
@@ -32714,11 +32714,11 @@
       </c>
       <c r="K6" s="7">
         <f t="shared" ref="K6:K18" si="0">SUMIFS(CgCajas,CgSemanaP90,A6,CgCuenta,1)</f>
-        <v>980</v>
+        <v>0</v>
       </c>
       <c r="L6" s="7">
         <f>ConteoTotal+K6-D6</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="M6">
         <f ca="1">IF(AND(L6&lt;MinimoSabado,Proyeccion!J6&gt;=FechaHoy),ROUNDUP((MinimoSabado-L6)/CajasProm,0),0)</f>
@@ -32726,15 +32726,15 @@
       </c>
       <c r="N6" s="7">
         <f t="shared" ref="N6:N18" ca="1" si="1">G6-IF(A6&gt;=FechaHoy-WEEKDAY(FechaHoy,2)+8,3*CajasPY,0)</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="O6" s="7">
         <f t="shared" ref="O6:O18" ca="1" si="2">G6-IF(A6&gt;=FechaHoy-WEEKDAY(FechaHoy,2)+8,1000,0)</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
       <c r="P6" s="7">
         <f t="shared" ref="P6:P18" ca="1" si="3">G6-SUMIFS(CgCajas,CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+8),CgSemana,"&lt;="&amp;MIN(A6,FechaHoy-WEEKDAY(FechaHoy,2)+15))</f>
-        <v>27952</v>
+        <v>26972</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -32748,7 +32748,7 @@
       </c>
       <c r="C7" s="7">
         <f>Proyeccion!E7</f>
-        <v>10946</v>
+        <v>11926</v>
       </c>
       <c r="D7" s="7">
         <f>Proyeccion!F7</f>
@@ -32784,7 +32784,7 @@
       </c>
       <c r="L7" s="7">
         <f t="shared" ref="L7:L18" ca="1" si="7">(L6+M6*CajasProm)+K7-D7</f>
-        <v>18866</v>
+        <v>17886</v>
       </c>
       <c r="M7">
         <f ca="1">IF(AND(L7&lt;MinimoSabado,Proyeccion!J7&gt;=FechaHoy),ROUNDUP((MinimoSabado-L7)/CajasProm,0),0)</f>
@@ -32846,15 +32846,15 @@
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
-        <v>16924</v>
+        <v>15944</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>18790</v>
+        <v>16830</v>
       </c>
       <c r="M8">
         <f ca="1">IF(AND(L8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-L8)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
@@ -32912,15 +32912,15 @@
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
-        <v>15844</v>
+        <v>17804</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>21634</v>
+        <v>23634</v>
       </c>
       <c r="M9">
         <f ca="1">IF(AND(L9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-L9)/CajasProm,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
@@ -32982,11 +32982,11 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>18598</v>
+        <v>19598</v>
       </c>
       <c r="M10">
         <f ca="1">IF(AND(L10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-L10)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" ca="1" si="1"/>

</xml_diff>

<commit_message>
plan de compras: venta supuesta 18.000/semana desde el 05/10 (verano)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{167D7F55-B319-458B-A1CC-28D37EA6A334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0102A0E-9300-4D41-A032-F8B9C2C29FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -115,7 +115,7 @@
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 01/10/2026 12:39 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 01/10/2026 12:49 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -583,7 +583,7 @@
     <t>Gonzalo 27/09: se pide vender 16.000; Bolivia 1 carga, el resto PY y BR</t>
   </si>
   <si>
-    <t>SUPUESTO = semana anterior (confirmar)</t>
+    <t>SUPUESTO 18.000 (Gonzalo 01/10: "si sube es a 18 mil la venta, no mas"; verano)</t>
   </si>
   <si>
     <t>sin fila en ventas_plan: copia de la semana del 19/10 (SUPUESTO)</t>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="D7" s="7">
         <f>Demanda!H8</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E7" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="D8" s="7">
         <f>Demanda!H9</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E8" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D9" s="7">
         <f>Demanda!H10</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E9" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="D10" s="7">
         <f>Demanda!H11</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E10" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="D11" s="7">
         <f>Demanda!H12</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E11" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="D12" s="7">
         <f>Demanda!H13</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E12" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="D13" s="7">
         <f>Demanda!H14</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E13" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="D14" s="7">
         <f>Demanda!H15</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E14" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="D15" s="7">
         <f>Demanda!H16</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E15" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D16" s="7">
         <f>Demanda!H17</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E16" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="D17" s="7">
         <f>Demanda!H18</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E17" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="D18" s="7">
         <f>Demanda!H18</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E18" s="7" t="str">
         <f t="shared" si="0"/>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B9" s="25">
         <f ca="1">IFERROR(INDEX(PrACargar,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>303</v>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B10" s="24">
         <f ca="1">AVERAGEIFS(PrCobertura,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8.8275882352941188</v>
+        <v>8.3371666666666666</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>305</v>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="B12" s="25">
         <f ca="1">SUMIFS(PrACargar,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>309</v>
@@ -8523,11 +8523,11 @@
       </c>
       <c r="B52" s="7">
         <f ca="1">SSsugerido+ROUND(INDEX(DemVenta,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,DemSemana,0))/DiasVenta*DiasMadurar,0)</f>
-        <v>23119</v>
+        <v>24286</v>
       </c>
       <c r="E52" t="str">
         <f ca="1">"Contra el minimo de Gonzalo ("&amp;FIXED(MinimoSabado,0)&amp;"): "&amp;IF(MinSugerido&gt;MinimoSabado,"la formula pide "&amp;FIXED(MinSugerido-MinimoSabado,0)&amp;" cajas mas","la formula pide "&amp;FIXED(MinimoSabado-MinSugerido,0)&amp;" cajas menos")&amp;". El que manda en la planilla es el de la fila 5."</f>
-        <v>Contra el minimo de Gonzalo (25.000): la formula pide 1.881 cajas menos. El que manda en la planilla es el de la fila 5.</v>
+        <v>Contra el minimo de Gonzalo (25.000): la formula pide 714 cajas menos. El que manda en la planilla es el de la fila 5.</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="30">
@@ -8849,7 +8849,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="3"/>
@@ -8858,7 +8858,7 @@
       <c r="G8" s="8"/>
       <c r="H8" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I8" s="19">
         <v>0.61699999999999999</v>
@@ -8872,15 +8872,15 @@
       </c>
       <c r="L8" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M8" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N8" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O8" s="8"/>
       <c r="P8" s="20" t="str">
@@ -8908,7 +8908,7 @@
         <v>2</v>
       </c>
       <c r="E9" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="3"/>
@@ -8917,7 +8917,7 @@
       <c r="G9" s="8"/>
       <c r="H9" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I9" s="19">
         <v>0.61699999999999999</v>
@@ -8931,15 +8931,15 @@
       </c>
       <c r="L9" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M9" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N9" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="20" t="str">
@@ -8967,7 +8967,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="3"/>
@@ -8976,7 +8976,7 @@
       <c r="G10" s="8"/>
       <c r="H10" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I10" s="19">
         <v>0.61699999999999999</v>
@@ -8990,15 +8990,15 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M10" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O10" s="8"/>
       <c r="P10" s="20" t="str">
@@ -9026,7 +9026,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="3"/>
@@ -9035,7 +9035,7 @@
       <c r="G11" s="8"/>
       <c r="H11" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I11" s="19">
         <v>0.61699999999999999</v>
@@ -9049,15 +9049,15 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M11" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N11" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O11" s="8"/>
       <c r="P11" s="20" t="str">
@@ -9085,7 +9085,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F12" s="10">
         <f t="shared" si="3"/>
@@ -9094,7 +9094,7 @@
       <c r="G12" s="8"/>
       <c r="H12" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I12" s="19">
         <v>0.61699999999999999</v>
@@ -9108,15 +9108,15 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M12" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N12" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O12" s="8"/>
       <c r="P12" s="20" t="str">
@@ -9144,7 +9144,7 @@
         <v>2</v>
       </c>
       <c r="E13" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F13" s="10">
         <f t="shared" si="3"/>
@@ -9153,7 +9153,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I13" s="19">
         <v>0.61699999999999999</v>
@@ -9167,15 +9167,15 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M13" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N13" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O13" s="8"/>
       <c r="P13" s="20" t="str">
@@ -9203,7 +9203,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F14" s="10">
         <f t="shared" si="3"/>
@@ -9212,7 +9212,7 @@
       <c r="G14" s="8"/>
       <c r="H14" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I14" s="19">
         <v>0.61699999999999999</v>
@@ -9226,15 +9226,15 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M14" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N14" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O14" s="8"/>
       <c r="P14" s="20" t="str">
@@ -9262,7 +9262,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" si="3"/>
@@ -9271,7 +9271,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I15" s="19">
         <v>0.61699999999999999</v>
@@ -9285,15 +9285,15 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M15" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N15" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O15" s="8"/>
       <c r="P15" s="20" t="str">
@@ -9321,7 +9321,7 @@
         <v>5</v>
       </c>
       <c r="E16" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F16" s="10">
         <f t="shared" si="3"/>
@@ -9330,7 +9330,7 @@
       <c r="G16" s="8"/>
       <c r="H16" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I16" s="19">
         <v>0.61699999999999999</v>
@@ -9344,15 +9344,15 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M16" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N16" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O16" s="8"/>
       <c r="P16" s="20" t="str">
@@ -9380,7 +9380,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F17" s="10">
         <f t="shared" si="3"/>
@@ -9389,7 +9389,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I17" s="19">
         <v>0.61699999999999999</v>
@@ -9403,15 +9403,15 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M17" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N17" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O17" s="8"/>
       <c r="P17" s="20" t="str">
@@ -9439,7 +9439,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="8">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="F18" s="10">
         <f t="shared" si="3"/>
@@ -9448,7 +9448,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="12">
         <f t="shared" si="4"/>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="I18" s="19">
         <v>0.61699999999999999</v>
@@ -9462,15 +9462,15 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" si="6"/>
-        <v>10489</v>
+        <v>11106</v>
       </c>
       <c r="M18" s="7">
         <f t="shared" si="7"/>
-        <v>5304</v>
+        <v>5616</v>
       </c>
       <c r="N18" s="7">
         <f t="shared" si="8"/>
-        <v>1207</v>
+        <v>1278</v>
       </c>
       <c r="O18" s="8"/>
       <c r="P18" s="20" t="str">
@@ -30487,7 +30487,7 @@
       </c>
       <c r="M7" s="22">
         <f ca="1">IF(Demanda!H8=0,"",L7/(Demanda!H8/DiasVenta))</f>
-        <v>8.0816470588235294</v>
+        <v>7.6326666666666663</v>
       </c>
       <c r="N7" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30499,7 +30499,7 @@
       </c>
       <c r="P7" s="22">
         <f>IF(Demanda!L8=0,"",O7/(Demanda!L8/DiasVenta))</f>
-        <v>5.1419582419677754</v>
+        <v>4.8562938951917882</v>
       </c>
       <c r="Q7" s="7">
         <f>Q6+SUMIFS(CgCajas,CgSemana,A7,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M7,0)</f>
@@ -30507,7 +30507,7 @@
       </c>
       <c r="R7" s="22">
         <f>IF(Demanda!M8=0,"",Q7/(Demanda!M8/DiasVenta))</f>
-        <v>13.878959276018099</v>
+        <v>13.107905982905983</v>
       </c>
       <c r="S7" s="7">
         <f>S6+SUMIFS(CgCajas,CgSemana,A7,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N7,0)</f>
@@ -30515,7 +30515,7 @@
       </c>
       <c r="T7" s="22">
         <f>IF(Demanda!N8=0,"",S7/(Demanda!N8/DiasVenta))</f>
-        <v>8.1524440762220394</v>
+        <v>7.699530516431925</v>
       </c>
       <c r="U7" t="str">
         <f t="shared" si="9"/>
@@ -30545,11 +30545,11 @@
       </c>
       <c r="F8" s="7">
         <f>ROUND(Demanda!H8,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G8" s="7">
         <f t="shared" si="3"/>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="H8" s="7">
         <f ca="1">SUM($K$6:K7)*CajasProm</f>
@@ -30557,7 +30557,7 @@
       </c>
       <c r="I8" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="J8" s="21">
         <f t="shared" si="5"/>
@@ -30565,7 +30565,7 @@
       </c>
       <c r="K8" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30573,35 +30573,35 @@
       </c>
       <c r="M8" s="22">
         <f ca="1">IF(Demanda!H9=0,"",L8/(Demanda!H9/DiasVenta))</f>
-        <v>9.0938823529411756</v>
+        <v>8.5886666666666667</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 1</v>
+        <v>CARGAR 2</v>
       </c>
       <c r="O8" s="7">
         <f>O7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L8,0)</f>
-        <v>12468</v>
+        <v>11851</v>
       </c>
       <c r="P8" s="22">
         <f>IF(Demanda!L9=0,"",O8/(Demanda!L9/DiasVenta))</f>
-        <v>7.1320430927638476</v>
+        <v>6.4024851431658565</v>
       </c>
       <c r="Q8" s="7">
         <f>Q7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M8,0)</f>
-        <v>11865</v>
+        <v>11553</v>
       </c>
       <c r="R8" s="22">
         <f>IF(Demanda!M9=0,"",Q8/(Demanda!M9/DiasVenta))</f>
-        <v>13.421945701357465</v>
+        <v>12.342948717948717</v>
       </c>
       <c r="S8" s="7">
         <f>S7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N8,0)</f>
-        <v>433</v>
+        <v>362</v>
       </c>
       <c r="T8" s="22">
         <f>IF(Demanda!N9=0,"",S8/(Demanda!N9/DiasVenta))</f>
-        <v>2.152444076222038</v>
+        <v>1.699530516431925</v>
       </c>
       <c r="U8" t="str">
         <f t="shared" si="9"/>
@@ -30619,7 +30619,7 @@
       </c>
       <c r="C9" s="7">
         <f t="shared" si="10"/>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="1"/>
@@ -30631,19 +30631,19 @@
       </c>
       <c r="F9" s="7">
         <f>ROUND(Demanda!H9,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G9" s="7">
         <f t="shared" si="3"/>
-        <v>18684</v>
+        <v>16684</v>
       </c>
       <c r="H9" s="7">
         <f ca="1">SUM($K$6:K8)*CajasProm</f>
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="I9" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>19684</v>
+        <v>18684</v>
       </c>
       <c r="J9" s="21">
         <f t="shared" si="5"/>
@@ -30651,7 +30651,7 @@
       </c>
       <c r="K9" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30659,35 +30659,35 @@
       </c>
       <c r="M9" s="22">
         <f ca="1">IF(Demanda!H10=0,"",L9/(Demanda!H10/DiasVenta))</f>
-        <v>9.0649411764705885</v>
+        <v>8.5613333333333337</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 6</v>
+        <v>CARGAR 7</v>
       </c>
       <c r="O9" s="7">
         <f>O8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L9,0)</f>
-        <v>6947</v>
+        <v>5713</v>
       </c>
       <c r="P9" s="22">
         <f>IF(Demanda!L10=0,"",O9/(Demanda!L10/DiasVenta))</f>
-        <v>3.9738773953665745</v>
+        <v>3.0864397622906536</v>
       </c>
       <c r="Q9" s="7">
         <f>Q8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M9,0)</f>
-        <v>11461</v>
+        <v>10837</v>
       </c>
       <c r="R9" s="22">
         <f>IF(Demanda!M10=0,"",Q9/(Demanda!M10/DiasVenta))</f>
-        <v>12.964932126696832</v>
+        <v>11.577991452991453</v>
       </c>
       <c r="S9" s="7">
         <f>S8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N9,0)</f>
-        <v>276</v>
+        <v>134</v>
       </c>
       <c r="T9" s="22">
         <f>IF(Demanda!N10=0,"",S9/(Demanda!N10/DiasVenta))</f>
-        <v>1.371996685998343</v>
+        <v>0.62910798122065725</v>
       </c>
       <c r="U9" t="str">
         <f t="shared" si="9"/>
@@ -30705,7 +30705,7 @@
       </c>
       <c r="C10" s="7">
         <f t="shared" si="10"/>
-        <v>18684</v>
+        <v>16684</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
@@ -30717,19 +30717,19 @@
       </c>
       <c r="F10" s="7">
         <f>ROUND(Demanda!H10,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" si="3"/>
-        <v>15698</v>
+        <v>12698</v>
       </c>
       <c r="H10" s="7">
         <f ca="1">SUM($K$6:K9)*CajasProm</f>
-        <v>7000</v>
+        <v>9000</v>
       </c>
       <c r="I10" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>22698</v>
+        <v>21698</v>
       </c>
       <c r="J10" s="21">
         <f t="shared" si="5"/>
@@ -30737,7 +30737,7 @@
       </c>
       <c r="K10" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30745,35 +30745,35 @@
       </c>
       <c r="M10" s="22">
         <f ca="1">IF(Demanda!H11=0,"",L10/(Demanda!H11/DiasVenta))</f>
-        <v>9.0698823529411765</v>
+        <v>8.5660000000000007</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 3</v>
+        <v>CARGAR 4</v>
       </c>
       <c r="O10" s="7">
         <f>O9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L10,0)</f>
-        <v>4522</v>
+        <v>2671</v>
       </c>
       <c r="P10" s="22">
         <f>IF(Demanda!L11=0,"",O10/(Demanda!L11/DiasVenta))</f>
-        <v>2.586709886547812</v>
+        <v>1.4430037817396002</v>
       </c>
       <c r="Q10" s="7">
         <f>Q9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M10,0)</f>
-        <v>11057</v>
+        <v>10121</v>
       </c>
       <c r="R10" s="22">
         <f>IF(Demanda!M11=0,"",Q10/(Demanda!M11/DiasVenta))</f>
-        <v>12.5079185520362</v>
+        <v>10.813034188034187</v>
       </c>
       <c r="S10" s="7">
         <f>S9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N10,0)</f>
-        <v>119</v>
+        <v>-94</v>
       </c>
       <c r="T10" s="22">
         <f>IF(Demanda!N11=0,"",S10/(Demanda!N11/DiasVenta))</f>
-        <v>0.59154929577464788</v>
+        <v>-0.44131455399061031</v>
       </c>
       <c r="U10" t="str">
         <f t="shared" si="9"/>
@@ -30791,7 +30791,7 @@
       </c>
       <c r="C11" s="7">
         <f t="shared" si="10"/>
-        <v>15698</v>
+        <v>12698</v>
       </c>
       <c r="D11" s="7">
         <f t="shared" si="1"/>
@@ -30803,19 +30803,19 @@
       </c>
       <c r="F11" s="7">
         <f>ROUND(Demanda!H11,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G11" s="7">
         <f t="shared" si="3"/>
-        <v>7812</v>
+        <v>3812</v>
       </c>
       <c r="H11" s="7">
         <f ca="1">SUM($K$6:K10)*CajasProm</f>
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="I11" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>17812</v>
+        <v>16812</v>
       </c>
       <c r="J11" s="21">
         <f t="shared" si="5"/>
@@ -30823,7 +30823,7 @@
       </c>
       <c r="K11" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30831,35 +30831,35 @@
       </c>
       <c r="M11" s="22">
         <f ca="1">IF(Demanda!H12=0,"",L11/(Demanda!H12/DiasVenta))</f>
-        <v>9.1101176470588232</v>
+        <v>8.6039999999999992</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 8</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="O11" s="7">
         <f>O10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L11,0)</f>
-        <v>2097</v>
+        <v>-371</v>
       </c>
       <c r="P11" s="22">
         <f>IF(Demanda!L12=0,"",O11/(Demanda!L12/DiasVenta))</f>
-        <v>1.1995423777290495</v>
+        <v>-0.20043219881145327</v>
       </c>
       <c r="Q11" s="7">
         <f>Q10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M11,0)</f>
-        <v>5753</v>
+        <v>4505</v>
       </c>
       <c r="R11" s="22">
         <f>IF(Demanda!M12=0,"",Q11/(Demanda!M12/DiasVenta))</f>
-        <v>6.5079185520361991</v>
+        <v>4.8130341880341883</v>
       </c>
       <c r="S11" s="7">
         <f>S10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N11,0)</f>
-        <v>-38</v>
+        <v>-322</v>
       </c>
       <c r="T11" s="22">
         <f>IF(Demanda!N12=0,"",S11/(Demanda!N12/DiasVenta))</f>
-        <v>-0.18889809444904723</v>
+        <v>-1.511737089201878</v>
       </c>
       <c r="U11" t="str">
         <f t="shared" si="9"/>
@@ -30877,7 +30877,7 @@
       </c>
       <c r="C12" s="7">
         <f t="shared" si="10"/>
-        <v>7812</v>
+        <v>3812</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="1"/>
@@ -30889,19 +30889,19 @@
       </c>
       <c r="F12" s="7">
         <f>ROUND(Demanda!H12,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G12" s="7">
         <f t="shared" si="3"/>
-        <v>-1124</v>
+        <v>-6124</v>
       </c>
       <c r="H12" s="7">
         <f ca="1">SUM($K$6:K11)*CajasProm</f>
-        <v>18000</v>
+        <v>22000</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16876</v>
+        <v>15876</v>
       </c>
       <c r="J12" s="21">
         <f t="shared" si="5"/>
@@ -30909,7 +30909,7 @@
       </c>
       <c r="K12" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30917,35 +30917,35 @@
       </c>
       <c r="M12" s="22">
         <f ca="1">IF(Demanda!H13=0,"",L12/(Demanda!H13/DiasVenta))</f>
-        <v>9.1327058823529406</v>
+        <v>8.6253333333333337</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O12" s="7">
         <f>O11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L12,0)</f>
-        <v>-328</v>
+        <v>-3413</v>
       </c>
       <c r="P12" s="22">
         <f>IF(Demanda!L13=0,"",O12/(Demanda!L13/DiasVenta))</f>
-        <v>-0.18762513108971302</v>
+        <v>-1.8438681793625067</v>
       </c>
       <c r="Q12" s="7">
         <f>Q11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M12,0)</f>
-        <v>449</v>
+        <v>-1111</v>
       </c>
       <c r="R12" s="22">
         <f>IF(Demanda!M13=0,"",Q12/(Demanda!M13/DiasVenta))</f>
-        <v>0.50791855203619907</v>
+        <v>-1.186965811965812</v>
       </c>
       <c r="S12" s="7">
         <f>S11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N12,0)</f>
-        <v>-1245</v>
+        <v>-1600</v>
       </c>
       <c r="T12" s="22">
         <f>IF(Demanda!N13=0,"",S12/(Demanda!N13/DiasVenta))</f>
-        <v>-6.1888980944490477</v>
+        <v>-7.511737089201878</v>
       </c>
       <c r="U12" t="str">
         <f t="shared" si="9"/>
@@ -30963,7 +30963,7 @@
       </c>
       <c r="C13" s="7">
         <f t="shared" si="10"/>
-        <v>-1124</v>
+        <v>-6124</v>
       </c>
       <c r="D13" s="7">
         <f t="shared" si="1"/>
@@ -30975,19 +30975,19 @@
       </c>
       <c r="F13" s="7">
         <f>ROUND(Demanda!H13,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G13" s="7">
         <f t="shared" si="3"/>
-        <v>-10060</v>
+        <v>-16060</v>
       </c>
       <c r="H13" s="7">
         <f ca="1">SUM($K$6:K12)*CajasProm</f>
-        <v>27000</v>
+        <v>32000</v>
       </c>
       <c r="I13" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16940</v>
+        <v>15940</v>
       </c>
       <c r="J13" s="21">
         <f t="shared" si="5"/>
@@ -30995,7 +30995,7 @@
       </c>
       <c r="K13" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31003,35 +31003,35 @@
       </c>
       <c r="M13" s="22">
         <f ca="1">IF(Demanda!H14=0,"",L13/(Demanda!H14/DiasVenta))</f>
-        <v>9.1552941176470579</v>
+        <v>8.6466666666666665</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O13" s="7">
         <f>O12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L13,0)</f>
-        <v>-2753</v>
+        <v>-6455</v>
       </c>
       <c r="P13" s="22">
         <f>IF(Demanda!L14=0,"",O13/(Demanda!L14/DiasVenta))</f>
-        <v>-1.5747926399084755</v>
+        <v>-3.4873041599135601</v>
       </c>
       <c r="Q13" s="7">
         <f>Q12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M13,0)</f>
-        <v>-4855</v>
+        <v>-6727</v>
       </c>
       <c r="R13" s="22">
         <f>IF(Demanda!M14=0,"",Q13/(Demanda!M14/DiasVenta))</f>
-        <v>-5.4920814479638009</v>
+        <v>-7.1869658119658117</v>
       </c>
       <c r="S13" s="7">
         <f>S12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N13,0)</f>
-        <v>-2452</v>
+        <v>-2878</v>
       </c>
       <c r="T13" s="22">
         <f>IF(Demanda!N14=0,"",S13/(Demanda!N14/DiasVenta))</f>
-        <v>-12.188898094449048</v>
+        <v>-13.511737089201878</v>
       </c>
       <c r="U13" t="str">
         <f t="shared" si="9"/>
@@ -31049,7 +31049,7 @@
       </c>
       <c r="C14" s="7">
         <f t="shared" si="10"/>
-        <v>-10060</v>
+        <v>-16060</v>
       </c>
       <c r="D14" s="7">
         <f t="shared" si="1"/>
@@ -31061,19 +31061,19 @@
       </c>
       <c r="F14" s="7">
         <f>ROUND(Demanda!H14,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G14" s="7">
         <f t="shared" si="3"/>
-        <v>-18996</v>
+        <v>-25996</v>
       </c>
       <c r="H14" s="7">
         <f ca="1">SUM($K$6:K13)*CajasProm</f>
-        <v>36000</v>
+        <v>42000</v>
       </c>
       <c r="I14" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>17004</v>
+        <v>16004</v>
       </c>
       <c r="J14" s="21">
         <f t="shared" si="5"/>
@@ -31081,7 +31081,7 @@
       </c>
       <c r="K14" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31089,35 +31089,35 @@
       </c>
       <c r="M14" s="22">
         <f ca="1">IF(Demanda!H15=0,"",L14/(Demanda!H15/DiasVenta))</f>
-        <v>8.8249411764705883</v>
+        <v>8.3346666666666671</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 8</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="O14" s="7">
         <f>O13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L14,0)</f>
-        <v>-5178</v>
+        <v>-9497</v>
       </c>
       <c r="P14" s="22">
         <f>IF(Demanda!L15=0,"",O14/(Demanda!L15/DiasVenta))</f>
-        <v>-2.961960148727238</v>
+        <v>-5.1307401404646136</v>
       </c>
       <c r="Q14" s="7">
         <f>Q13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M14,0)</f>
-        <v>-10159</v>
+        <v>-12343</v>
       </c>
       <c r="R14" s="22">
         <f>IF(Demanda!M15=0,"",Q14/(Demanda!M15/DiasVenta))</f>
-        <v>-11.4920814479638</v>
+        <v>-13.186965811965813</v>
       </c>
       <c r="S14" s="7">
         <f>S13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N14,0)</f>
-        <v>-3659</v>
+        <v>-4156</v>
       </c>
       <c r="T14" s="22">
         <f>IF(Demanda!N15=0,"",S14/(Demanda!N15/DiasVenta))</f>
-        <v>-18.188898094449048</v>
+        <v>-19.511737089201876</v>
       </c>
       <c r="U14" t="str">
         <f t="shared" si="9"/>
@@ -31135,7 +31135,7 @@
       </c>
       <c r="C15" s="7">
         <f t="shared" si="10"/>
-        <v>-18996</v>
+        <v>-25996</v>
       </c>
       <c r="D15" s="7">
         <f t="shared" si="1"/>
@@ -31147,19 +31147,19 @@
       </c>
       <c r="F15" s="7">
         <f>ROUND(Demanda!H15,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G15" s="7">
         <f t="shared" si="3"/>
-        <v>-27932</v>
+        <v>-35932</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">SUM($K$6:K14)*CajasProm</f>
-        <v>44000</v>
+        <v>51000</v>
       </c>
       <c r="I15" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16068</v>
+        <v>15068</v>
       </c>
       <c r="J15" s="21">
         <f t="shared" si="5"/>
@@ -31167,7 +31167,7 @@
       </c>
       <c r="K15" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31175,35 +31175,35 @@
       </c>
       <c r="M15" s="22">
         <f ca="1">IF(Demanda!H16=0,"",L15/(Demanda!H16/DiasVenta))</f>
-        <v>8.8475294117647056</v>
+        <v>8.3559999999999999</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O15" s="7">
         <f>O14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L15,0)</f>
-        <v>-7603</v>
+        <v>-12539</v>
       </c>
       <c r="P15" s="22">
         <f>IF(Demanda!L16=0,"",O15/(Demanda!L16/DiasVenta))</f>
-        <v>-4.3491276575460001</v>
+        <v>-6.7741761210156675</v>
       </c>
       <c r="Q15" s="7">
         <f>Q14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M15,0)</f>
-        <v>-15463</v>
+        <v>-17959</v>
       </c>
       <c r="R15" s="22">
         <f>IF(Demanda!M16=0,"",Q15/(Demanda!M16/DiasVenta))</f>
-        <v>-17.492081447963802</v>
+        <v>-19.186965811965813</v>
       </c>
       <c r="S15" s="7">
         <f>S14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N15,0)</f>
-        <v>-4866</v>
+        <v>-5434</v>
       </c>
       <c r="T15" s="22">
         <f>IF(Demanda!N16=0,"",S15/(Demanda!N16/DiasVenta))</f>
-        <v>-24.188898094449048</v>
+        <v>-25.511737089201876</v>
       </c>
       <c r="U15" t="str">
         <f t="shared" si="9"/>
@@ -31221,7 +31221,7 @@
       </c>
       <c r="C16" s="7">
         <f t="shared" si="10"/>
-        <v>-27932</v>
+        <v>-35932</v>
       </c>
       <c r="D16" s="7">
         <f t="shared" si="1"/>
@@ -31233,19 +31233,19 @@
       </c>
       <c r="F16" s="7">
         <f>ROUND(Demanda!H16,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G16" s="7">
         <f t="shared" si="3"/>
-        <v>-36868</v>
+        <v>-45868</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">SUM($K$6:K15)*CajasProm</f>
-        <v>53000</v>
+        <v>61000</v>
       </c>
       <c r="I16" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16132</v>
+        <v>15132</v>
       </c>
       <c r="J16" s="21">
         <f t="shared" si="5"/>
@@ -31253,7 +31253,7 @@
       </c>
       <c r="K16" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31261,35 +31261,35 @@
       </c>
       <c r="M16" s="22">
         <f ca="1">IF(Demanda!H17=0,"",L16/(Demanda!H17/DiasVenta))</f>
-        <v>8.870117647058823</v>
+        <v>8.3773333333333326</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O16" s="7">
         <f>O15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L16,0)</f>
-        <v>-10028</v>
+        <v>-15581</v>
       </c>
       <c r="P16" s="22">
         <f>IF(Demanda!L17=0,"",O16/(Demanda!L17/DiasVenta))</f>
-        <v>-5.736295166364763</v>
+        <v>-8.4176121015667213</v>
       </c>
       <c r="Q16" s="7">
         <f>Q15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M16,0)</f>
-        <v>-20767</v>
+        <v>-23575</v>
       </c>
       <c r="R16" s="22">
         <f>IF(Demanda!M17=0,"",Q16/(Demanda!M17/DiasVenta))</f>
-        <v>-23.492081447963802</v>
+        <v>-25.186965811965813</v>
       </c>
       <c r="S16" s="7">
         <f>S15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N16,0)</f>
-        <v>-6073</v>
+        <v>-6712</v>
       </c>
       <c r="T16" s="22">
         <f>IF(Demanda!N17=0,"",S16/(Demanda!N17/DiasVenta))</f>
-        <v>-30.188898094449048</v>
+        <v>-31.511737089201876</v>
       </c>
       <c r="U16" t="str">
         <f t="shared" si="9"/>
@@ -31307,7 +31307,7 @@
       </c>
       <c r="C17" s="7">
         <f t="shared" si="10"/>
-        <v>-36868</v>
+        <v>-45868</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="1"/>
@@ -31319,19 +31319,19 @@
       </c>
       <c r="F17" s="7">
         <f>ROUND(Demanda!H17,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>-45804</v>
+        <v>-55804</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">SUM($K$6:K16)*CajasProm</f>
-        <v>62000</v>
+        <v>71000</v>
       </c>
       <c r="I17" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16196</v>
+        <v>15196</v>
       </c>
       <c r="J17" s="21">
         <f t="shared" si="5"/>
@@ -31339,7 +31339,7 @@
       </c>
       <c r="K17" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31347,35 +31347,35 @@
       </c>
       <c r="M17" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L17/(Demanda!H18/DiasVenta))</f>
-        <v>8.8927058823529403</v>
+        <v>8.3986666666666672</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O17" s="7">
         <f>O16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L17,0)</f>
-        <v>-12453</v>
+        <v>-18623</v>
       </c>
       <c r="P17" s="22">
         <f>IF(Demanda!L18=0,"",O17/(Demanda!L18/DiasVenta))</f>
-        <v>-7.1234626751835251</v>
+        <v>-10.061048082117773</v>
       </c>
       <c r="Q17" s="7">
         <f>Q16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M17,0)</f>
-        <v>-26071</v>
+        <v>-29191</v>
       </c>
       <c r="R17" s="22">
         <f>IF(Demanda!M18=0,"",Q17/(Demanda!M18/DiasVenta))</f>
-        <v>-29.492081447963802</v>
+        <v>-31.186965811965813</v>
       </c>
       <c r="S17" s="7">
         <f>S16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N17,0)</f>
-        <v>-7280</v>
+        <v>-7990</v>
       </c>
       <c r="T17" s="22">
         <f>IF(Demanda!N18=0,"",S17/(Demanda!N18/DiasVenta))</f>
-        <v>-36.188898094449051</v>
+        <v>-37.51173708920188</v>
       </c>
       <c r="U17" t="str">
         <f t="shared" si="9"/>
@@ -31393,7 +31393,7 @@
       </c>
       <c r="C18" s="7">
         <f t="shared" si="10"/>
-        <v>-45804</v>
+        <v>-55804</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="1"/>
@@ -31405,19 +31405,19 @@
       </c>
       <c r="F18" s="7">
         <f>ROUND(Demanda!H18,0)</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G18" s="7">
         <f t="shared" si="3"/>
-        <v>-54740</v>
+        <v>-65740</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">SUM($K$6:K17)*CajasProm</f>
-        <v>71000</v>
+        <v>81000</v>
       </c>
       <c r="I18" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16260</v>
+        <v>15260</v>
       </c>
       <c r="J18" s="21">
         <f t="shared" si="5"/>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="K18" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -31433,35 +31433,35 @@
       </c>
       <c r="M18" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L18/(Demanda!H18/DiasVenta))</f>
-        <v>8.9152941176470577</v>
+        <v>8.42</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O18" s="7">
         <f>O17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L18,0)</f>
-        <v>-14878</v>
+        <v>-21665</v>
       </c>
       <c r="P18" s="22">
         <f>IF(Demanda!L18=0,"",O18/(Demanda!L18/DiasVenta))</f>
-        <v>-8.510630184002288</v>
+        <v>-11.704484062668827</v>
       </c>
       <c r="Q18" s="7">
         <f>Q17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M18,0)</f>
-        <v>-31375</v>
+        <v>-34807</v>
       </c>
       <c r="R18" s="22">
         <f>IF(Demanda!M18=0,"",Q18/(Demanda!M18/DiasVenta))</f>
-        <v>-35.492081447963798</v>
+        <v>-37.186965811965813</v>
       </c>
       <c r="S18" s="7">
         <f>S17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N18,0)</f>
-        <v>-8487</v>
+        <v>-9268</v>
       </c>
       <c r="T18" s="22">
         <f>IF(Demanda!N18=0,"",S18/(Demanda!N18/DiasVenta))</f>
-        <v>-42.188898094449051</v>
+        <v>-43.51173708920188</v>
       </c>
       <c r="U18" t="str">
         <f t="shared" si="9"/>
@@ -31671,11 +31671,11 @@
       </c>
       <c r="B8" s="7">
         <f ca="1">IF(A8="","",Proyeccion!I8)</f>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="C8" s="3">
         <f ca="1">IF(A8="","",Proyeccion!K8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="str">
         <f ca="1">IF(A8="","","BR "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B8-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B8-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31691,15 +31691,15 @@
       </c>
       <c r="G8" s="22">
         <f ca="1">IF(A8="","",Proyeccion!M8)</f>
-        <v>9.0938823529411756</v>
+        <v>8.5886666666666667</v>
       </c>
       <c r="H8" t="str">
         <f ca="1">IF(A8="","",Proyeccion!N8)</f>
-        <v>CARGAR 1</v>
+        <v>CARGAR 2</v>
       </c>
       <c r="I8" t="str">
         <f ca="1">IF(A8="","","Sab "&amp;TEXT(A8,"dd/mm")&amp;": "&amp;FIXED(B8,0)&amp;" cajas - descargan "&amp;Proyeccion!D8&amp;" - vende "&amp;FIXED(Proyeccion!F8,0)&amp;IF(C8&gt;0," -&gt; cargar "&amp;C8&amp;" mas hasta el "&amp;TEXT(Proyeccion!J8,"dd/mm")&amp;" ("&amp;E8&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 10/10: 24.766 cajas - descargan 19 - vende 17.000 -&gt; cargar 1 mas hasta el 06/10 (Bolivia; BR hasta el 07/10)</v>
+        <v>Sab 10/10: 23.766 cajas - descargan 19 - vende 18.000 -&gt; cargar 2 mas hasta el 06/10 (Bolivia; BR hasta el 07/10)</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -31709,11 +31709,11 @@
       </c>
       <c r="B9" s="7">
         <f ca="1">IF(A9="","",Proyeccion!I9)</f>
-        <v>19684</v>
+        <v>18684</v>
       </c>
       <c r="C9" s="3">
         <f ca="1">IF(A9="","",Proyeccion!K9)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" t="str">
         <f ca="1">IF(A9="","","BR "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B9-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B9-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31729,15 +31729,15 @@
       </c>
       <c r="G9" s="22">
         <f ca="1">IF(A9="","",Proyeccion!M9)</f>
-        <v>9.0649411764705885</v>
+        <v>8.5613333333333337</v>
       </c>
       <c r="H9" t="str">
         <f ca="1">IF(A9="","",Proyeccion!N9)</f>
-        <v>CARGAR 6</v>
+        <v>CARGAR 7</v>
       </c>
       <c r="I9" t="str">
         <f ca="1">IF(A9="","","Sab "&amp;TEXT(A9,"dd/mm")&amp;": "&amp;FIXED(B9,0)&amp;" cajas - descargan "&amp;Proyeccion!D9&amp;" - vende "&amp;FIXED(Proyeccion!F9,0)&amp;IF(C9&gt;0," -&gt; cargar "&amp;C9&amp;" mas hasta el "&amp;TEXT(Proyeccion!J9,"dd/mm")&amp;" ("&amp;E9&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 17/10: 19.684 cajas - descargan 11 - vende 17.000 -&gt; cargar 6 mas hasta el 13/10 (Bolivia; BR hasta el 14/10)</v>
+        <v>Sab 17/10: 18.684 cajas - descargan 11 - vende 18.000 -&gt; cargar 7 mas hasta el 13/10 (Bolivia; BR hasta el 14/10)</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -31747,11 +31747,11 @@
       </c>
       <c r="B10" s="7">
         <f ca="1">IF(A10="","",Proyeccion!I10)</f>
-        <v>22698</v>
+        <v>21698</v>
       </c>
       <c r="C10" s="3">
         <f ca="1">IF(A10="","",Proyeccion!K10)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="str">
         <f ca="1">IF(A10="","","BR "&amp;TEXT(Proyeccion!B10-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B10-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B10-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31767,15 +31767,15 @@
       </c>
       <c r="G10" s="22">
         <f ca="1">IF(A10="","",Proyeccion!M10)</f>
-        <v>9.0698823529411765</v>
+        <v>8.5660000000000007</v>
       </c>
       <c r="H10" t="str">
         <f ca="1">IF(A10="","",Proyeccion!N10)</f>
-        <v>CARGAR 3</v>
+        <v>CARGAR 4</v>
       </c>
       <c r="I10" t="str">
         <f ca="1">IF(A10="","","Sab "&amp;TEXT(A10,"dd/mm")&amp;": "&amp;FIXED(B10,0)&amp;" cajas - descargan "&amp;Proyeccion!D10&amp;" - vende "&amp;FIXED(Proyeccion!F10,0)&amp;IF(C10&gt;0," -&gt; cargar "&amp;C10&amp;" mas hasta el "&amp;TEXT(Proyeccion!J10,"dd/mm")&amp;" ("&amp;E10&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B10-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 24/10: 22.698 cajas - descargan 14 - vende 17.000 -&gt; cargar 3 mas hasta el 20/10 (Bolivia; BR hasta el 21/10)</v>
+        <v>Sab 24/10: 21.698 cajas - descargan 14 - vende 18.000 -&gt; cargar 4 mas hasta el 20/10 (Bolivia; BR hasta el 21/10)</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -31785,11 +31785,11 @@
       </c>
       <c r="B11" s="7">
         <f ca="1">IF(A11="","",Proyeccion!I11)</f>
-        <v>17812</v>
+        <v>16812</v>
       </c>
       <c r="C11" s="3">
         <f ca="1">IF(A11="","",Proyeccion!K11)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" t="str">
         <f ca="1">IF(A11="","","BR "&amp;TEXT(Proyeccion!B11-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B11-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B11-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31805,15 +31805,15 @@
       </c>
       <c r="G11" s="22">
         <f ca="1">IF(A11="","",Proyeccion!M11)</f>
-        <v>9.1101176470588232</v>
+        <v>8.6039999999999992</v>
       </c>
       <c r="H11" t="str">
         <f ca="1">IF(A11="","",Proyeccion!N11)</f>
-        <v>CARGAR 8</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="I11" t="str">
         <f ca="1">IF(A11="","","Sab "&amp;TEXT(A11,"dd/mm")&amp;": "&amp;FIXED(B11,0)&amp;" cajas - descargan "&amp;Proyeccion!D11&amp;" - vende "&amp;FIXED(Proyeccion!F11,0)&amp;IF(C11&gt;0," -&gt; cargar "&amp;C11&amp;" mas hasta el "&amp;TEXT(Proyeccion!J11,"dd/mm")&amp;" ("&amp;E11&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B11-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 31/10: 17.812 cajas - descargan 9 - vende 17.000 -&gt; cargar 8 mas hasta el 27/10 (Bolivia; BR hasta el 28/10)</v>
+        <v>Sab 31/10: 16.812 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 27/10 (Bolivia; BR hasta el 28/10)</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -31823,11 +31823,11 @@
       </c>
       <c r="B12" s="7">
         <f ca="1">IF(A12="","",Proyeccion!I12)</f>
-        <v>16876</v>
+        <v>15876</v>
       </c>
       <c r="C12" s="3">
         <f ca="1">IF(A12="","",Proyeccion!K12)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" t="str">
         <f ca="1">IF(A12="","","BR "&amp;TEXT(Proyeccion!B12-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B12-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B12-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31843,15 +31843,15 @@
       </c>
       <c r="G12" s="22">
         <f ca="1">IF(A12="","",Proyeccion!M12)</f>
-        <v>9.1327058823529406</v>
+        <v>8.6253333333333337</v>
       </c>
       <c r="H12" t="str">
         <f ca="1">IF(A12="","",Proyeccion!N12)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I12" t="str">
         <f ca="1">IF(A12="","","Sab "&amp;TEXT(A12,"dd/mm")&amp;": "&amp;FIXED(B12,0)&amp;" cajas - descargan "&amp;Proyeccion!D12&amp;" - vende "&amp;FIXED(Proyeccion!F12,0)&amp;IF(C12&gt;0," -&gt; cargar "&amp;C12&amp;" mas hasta el "&amp;TEXT(Proyeccion!J12,"dd/mm")&amp;" ("&amp;E12&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B12-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 07/11: 16.876 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
+        <v>Sab 07/11: 15.876 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -31861,11 +31861,11 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IF(A13="","",Proyeccion!I13)</f>
-        <v>16940</v>
+        <v>15940</v>
       </c>
       <c r="C13" s="3">
         <f ca="1">IF(A13="","",Proyeccion!K13)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(A13="","","BR "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B13-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B13-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31881,15 +31881,15 @@
       </c>
       <c r="G13" s="22">
         <f ca="1">IF(A13="","",Proyeccion!M13)</f>
-        <v>9.1552941176470579</v>
+        <v>8.6466666666666665</v>
       </c>
       <c r="H13" t="str">
         <f ca="1">IF(A13="","",Proyeccion!N13)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I13" t="str">
         <f ca="1">IF(A13="","","Sab "&amp;TEXT(A13,"dd/mm")&amp;": "&amp;FIXED(B13,0)&amp;" cajas - descargan "&amp;Proyeccion!D13&amp;" - vende "&amp;FIXED(Proyeccion!F13,0)&amp;IF(C13&gt;0," -&gt; cargar "&amp;C13&amp;" mas hasta el "&amp;TEXT(Proyeccion!J13,"dd/mm")&amp;" ("&amp;E13&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 14/11: 16.940 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
+        <v>Sab 14/11: 15.940 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -31899,11 +31899,11 @@
       </c>
       <c r="B14" s="7">
         <f ca="1">IF(A14="","",Proyeccion!I14)</f>
-        <v>17004</v>
+        <v>16004</v>
       </c>
       <c r="C14" s="3">
         <f ca="1">IF(A14="","",Proyeccion!K14)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" t="str">
         <f ca="1">IF(A14="","","BR "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B14-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B14-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31919,15 +31919,15 @@
       </c>
       <c r="G14" s="22">
         <f ca="1">IF(A14="","",Proyeccion!M14)</f>
-        <v>8.8249411764705883</v>
+        <v>8.3346666666666671</v>
       </c>
       <c r="H14" t="str">
         <f ca="1">IF(A14="","",Proyeccion!N14)</f>
-        <v>CARGAR 8</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="I14" t="str">
         <f ca="1">IF(A14="","","Sab "&amp;TEXT(A14,"dd/mm")&amp;": "&amp;FIXED(B14,0)&amp;" cajas - descargan "&amp;Proyeccion!D14&amp;" - vende "&amp;FIXED(Proyeccion!F14,0)&amp;IF(C14&gt;0," -&gt; cargar "&amp;C14&amp;" mas hasta el "&amp;TEXT(Proyeccion!J14,"dd/mm")&amp;" ("&amp;E14&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 21/11: 17.004 cajas - descargan 8 - vende 17.000 -&gt; cargar 8 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
+        <v>Sab 21/11: 16.004 cajas - descargan 8 - vende 18.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -31937,11 +31937,11 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(A15="","",Proyeccion!I15)</f>
-        <v>16068</v>
+        <v>15068</v>
       </c>
       <c r="C15" s="3">
         <f ca="1">IF(A15="","",Proyeccion!K15)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D15" t="str">
         <f ca="1">IF(A15="","","BR "&amp;TEXT(Proyeccion!B15-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B15-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B15-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31957,15 +31957,15 @@
       </c>
       <c r="G15" s="22">
         <f ca="1">IF(A15="","",Proyeccion!M15)</f>
-        <v>8.8475294117647056</v>
+        <v>8.3559999999999999</v>
       </c>
       <c r="H15" t="str">
         <f ca="1">IF(A15="","",Proyeccion!N15)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I15" t="str">
         <f ca="1">IF(A15="","","Sab "&amp;TEXT(A15,"dd/mm")&amp;": "&amp;FIXED(B15,0)&amp;" cajas - descargan "&amp;Proyeccion!D15&amp;" - vende "&amp;FIXED(Proyeccion!F15,0)&amp;IF(C15&gt;0," -&gt; cargar "&amp;C15&amp;" mas hasta el "&amp;TEXT(Proyeccion!J15,"dd/mm")&amp;" ("&amp;E15&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B15-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 28/11: 16.068 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
+        <v>Sab 28/11: 15.068 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -31975,11 +31975,11 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(A16="","",Proyeccion!I16)</f>
-        <v>16132</v>
+        <v>15132</v>
       </c>
       <c r="C16" s="3">
         <f ca="1">IF(A16="","",Proyeccion!K16)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" t="str">
         <f ca="1">IF(A16="","","BR "&amp;TEXT(Proyeccion!B16-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B16-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B16-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31995,15 +31995,15 @@
       </c>
       <c r="G16" s="22">
         <f ca="1">IF(A16="","",Proyeccion!M16)</f>
-        <v>8.870117647058823</v>
+        <v>8.3773333333333326</v>
       </c>
       <c r="H16" t="str">
         <f ca="1">IF(A16="","",Proyeccion!N16)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I16" t="str">
         <f ca="1">IF(A16="","","Sab "&amp;TEXT(A16,"dd/mm")&amp;": "&amp;FIXED(B16,0)&amp;" cajas - descargan "&amp;Proyeccion!D16&amp;" - vende "&amp;FIXED(Proyeccion!F16,0)&amp;IF(C16&gt;0," -&gt; cargar "&amp;C16&amp;" mas hasta el "&amp;TEXT(Proyeccion!J16,"dd/mm")&amp;" ("&amp;E16&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B16-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 05/12: 16.132 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
+        <v>Sab 05/12: 15.132 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -32013,11 +32013,11 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(A17="","",Proyeccion!I17)</f>
-        <v>16196</v>
+        <v>15196</v>
       </c>
       <c r="C17" s="3">
         <f ca="1">IF(A17="","",Proyeccion!K17)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D17" t="str">
         <f ca="1">IF(A17="","","BR "&amp;TEXT(Proyeccion!B17-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B17-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B17-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -32033,15 +32033,15 @@
       </c>
       <c r="G17" s="22">
         <f ca="1">IF(A17="","",Proyeccion!M17)</f>
-        <v>8.8927058823529403</v>
+        <v>8.3986666666666672</v>
       </c>
       <c r="H17" t="str">
         <f ca="1">IF(A17="","",Proyeccion!N17)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I17" t="str">
         <f ca="1">IF(A17="","","Sab "&amp;TEXT(A17,"dd/mm")&amp;": "&amp;FIXED(B17,0)&amp;" cajas - descargan "&amp;Proyeccion!D17&amp;" - vende "&amp;FIXED(Proyeccion!F17,0)&amp;IF(C17&gt;0," -&gt; cargar "&amp;C17&amp;" mas hasta el "&amp;TEXT(Proyeccion!J17,"dd/mm")&amp;" ("&amp;E17&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B17-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 12/12: 16.196 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
+        <v>Sab 12/12: 15.196 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -32051,11 +32051,11 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(A18="","",Proyeccion!I18)</f>
-        <v>16260</v>
+        <v>15260</v>
       </c>
       <c r="C18" s="3">
         <f ca="1">IF(A18="","",Proyeccion!K18)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D18" t="str">
         <f ca="1">IF(A18="","","BR "&amp;TEXT(Proyeccion!B18-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B18-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B18-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -32071,15 +32071,15 @@
       </c>
       <c r="G18" s="22">
         <f ca="1">IF(A18="","",Proyeccion!M18)</f>
-        <v>8.9152941176470577</v>
+        <v>8.42</v>
       </c>
       <c r="H18" t="str">
         <f ca="1">IF(A18="","",Proyeccion!N18)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I18" t="str">
         <f ca="1">IF(A18="","","Sab "&amp;TEXT(A18,"dd/mm")&amp;": "&amp;FIXED(B18,0)&amp;" cajas - descargan "&amp;Proyeccion!D18&amp;" - vende "&amp;FIXED(Proyeccion!F18,0)&amp;IF(C18&gt;0," -&gt; cargar "&amp;C18&amp;" mas hasta el "&amp;TEXT(Proyeccion!J18,"dd/mm")&amp;" ("&amp;E18&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B18-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 19/12: 16.260 cajas - descargan 8 - vende 17.000 -&gt; cargar 9 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
+        <v>Sab 19/12: 15.260 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="33.950000000000003" customHeight="1">
@@ -32197,7 +32197,7 @@
       </c>
       <c r="C6" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+0),PrSemana,0)),"")</f>
-        <v>5.1419582419677754</v>
+        <v>4.8562938951917882</v>
       </c>
       <c r="D6" t="str">
         <f ca="1">IF(B6="","",IF(B6&lt;0,"FALTA",IF(C6&lt;2,"CRITICO",IF(C6&lt;CoberturaObjetivo,"JUSTO",IF(C6&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32218,7 +32218,7 @@
       </c>
       <c r="C7" s="22">
         <f ca="1">IFERROR(INDEX(PrPYd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+0),PrSemana,0)),"")</f>
-        <v>13.878959276018099</v>
+        <v>13.107905982905983</v>
       </c>
       <c r="D7" t="str">
         <f ca="1">IF(B7="","",IF(B7&lt;0,"FALTA",IF(C7&lt;2,"CRITICO",IF(C7&lt;CoberturaObjetivo,"JUSTO",IF(C7&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32239,7 +32239,7 @@
       </c>
       <c r="C8" s="22">
         <f ca="1">IFERROR(INDEX(PrBOd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+0),PrSemana,0)),"")</f>
-        <v>8.1524440762220394</v>
+        <v>7.699530516431925</v>
       </c>
       <c r="D8" t="str">
         <f ca="1">IF(B8="","",IF(B8&lt;0,"FALTA",IF(C8&lt;2,"CRITICO",IF(C8&lt;CoberturaObjetivo,"JUSTO",IF(C8&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32260,7 +32260,7 @@
       </c>
       <c r="C9" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+0),PrSemana,0)),"")</f>
-        <v>8.0816470588235294</v>
+        <v>7.6326666666666663</v>
       </c>
       <c r="D9" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+0),PrSemana,0)),"")</f>
@@ -32304,19 +32304,19 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>12468</v>
+        <v>11851</v>
       </c>
       <c r="C13" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>7.1320430927638476</v>
+        <v>6.4024851431658565</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(B13="","",IF(B13&lt;0,"FALTA",IF(C13&lt;2,"CRITICO",IF(C13&lt;CoberturaObjetivo,"JUSTO",IF(C13&gt;VidaVerde,"EXCESO","OK")))))</f>
-        <v>OK</v>
+        <v>JUSTO</v>
       </c>
       <c r="E13" t="str">
         <f ca="1">IF(D13="FALTA","se queda sin fruta: cargar ya",IF(D13="CRITICO","cargar esta semana, sin falta",IF(D13="JUSTO","priorizar este origen en los pedidos",IF(D13="EXCESO","frenar cargas: riesgo de merma",""))))</f>
-        <v/>
+        <v>priorizar este origen en los pedidos</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -32325,11 +32325,11 @@
       </c>
       <c r="B14" s="7">
         <f ca="1">IFERROR(INDEX(PrPY,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>11865</v>
+        <v>11553</v>
       </c>
       <c r="C14" s="22">
         <f ca="1">IFERROR(INDEX(PrPYd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>13.421945701357465</v>
+        <v>12.342948717948717</v>
       </c>
       <c r="D14" t="str">
         <f ca="1">IF(B14="","",IF(B14&lt;0,"FALTA",IF(C14&lt;2,"CRITICO",IF(C14&lt;CoberturaObjetivo,"JUSTO",IF(C14&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32346,19 +32346,19 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IFERROR(INDEX(PrBO,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>433</v>
+        <v>362</v>
       </c>
       <c r="C15" s="22">
         <f ca="1">IFERROR(INDEX(PrBOd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>2.152444076222038</v>
+        <v>1.699530516431925</v>
       </c>
       <c r="D15" t="str">
         <f ca="1">IF(B15="","",IF(B15&lt;0,"FALTA",IF(C15&lt;2,"CRITICO",IF(C15&lt;CoberturaObjetivo,"JUSTO",IF(C15&gt;VidaVerde,"EXCESO","OK")))))</f>
-        <v>JUSTO</v>
+        <v>CRITICO</v>
       </c>
       <c r="E15" t="str">
         <f ca="1">IF(D15="FALTA","se queda sin fruta: cargar ya",IF(D15="CRITICO","cargar esta semana, sin falta",IF(D15="JUSTO","priorizar este origen en los pedidos",IF(D15="EXCESO","frenar cargas: riesgo de merma",""))))</f>
-        <v>priorizar este origen en los pedidos</v>
+        <v>cargar esta semana, sin falta</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -32367,19 +32367,19 @@
       </c>
       <c r="B16" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="C16" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>9.0938823529411756</v>
+        <v>8.5886666666666667</v>
       </c>
       <c r="D16" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>CARGAR 1</v>
+        <v>CARGAR 2</v>
       </c>
       <c r="E16" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 1 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
+        <v>cargar 2 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -32415,11 +32415,11 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>6947</v>
+        <v>5713</v>
       </c>
       <c r="C20" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>3.9738773953665745</v>
+        <v>3.0864397622906536</v>
       </c>
       <c r="D20" t="str">
         <f ca="1">IF(B20="","",IF(B20&lt;0,"FALTA",IF(C20&lt;2,"CRITICO",IF(C20&lt;CoberturaObjetivo,"JUSTO",IF(C20&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32436,11 +32436,11 @@
       </c>
       <c r="B21" s="7">
         <f ca="1">IFERROR(INDEX(PrPY,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>11461</v>
+        <v>10837</v>
       </c>
       <c r="C21" s="22">
         <f ca="1">IFERROR(INDEX(PrPYd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>12.964932126696832</v>
+        <v>11.577991452991453</v>
       </c>
       <c r="D21" t="str">
         <f ca="1">IF(B21="","",IF(B21&lt;0,"FALTA",IF(C21&lt;2,"CRITICO",IF(C21&lt;CoberturaObjetivo,"JUSTO",IF(C21&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32457,11 +32457,11 @@
       </c>
       <c r="B22" s="7">
         <f ca="1">IFERROR(INDEX(PrBO,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>276</v>
+        <v>134</v>
       </c>
       <c r="C22" s="22">
         <f ca="1">IFERROR(INDEX(PrBOd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>1.371996685998343</v>
+        <v>0.62910798122065725</v>
       </c>
       <c r="D22" t="str">
         <f ca="1">IF(B22="","",IF(B22&lt;0,"FALTA",IF(C22&lt;2,"CRITICO",IF(C22&lt;CoberturaObjetivo,"JUSTO",IF(C22&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32478,19 +32478,19 @@
       </c>
       <c r="B23" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>19684</v>
+        <v>18684</v>
       </c>
       <c r="C23" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>9.0649411764705885</v>
+        <v>8.5613333333333337</v>
       </c>
       <c r="D23" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>CARGAR 6</v>
+        <v>CARGAR 7</v>
       </c>
       <c r="E23" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 6 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
+        <v>cargar 7 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30">
@@ -32545,7 +32545,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.830 (plan: 24.766).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 15.830 (plan: 23.766).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32866,11 +32866,11 @@
       </c>
       <c r="D8" s="7">
         <f>Proyeccion!F8</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>28066</v>
+        <v>27166</v>
       </c>
       <c r="F8">
         <f ca="1">IF(AND(E8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-E8)/CajasProm,0),0)</f>
@@ -32878,19 +32878,19 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>24766</v>
+        <v>23766</v>
       </c>
       <c r="H8">
         <f ca="1">IF(AND(G8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-G8)/CajasProm,0),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>21466</v>
+        <v>20366</v>
       </c>
       <c r="J8">
         <f ca="1">IF(AND(I8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-I8)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
@@ -32898,23 +32898,23 @@
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16830</v>
+        <v>15830</v>
       </c>
       <c r="M8">
         <f ca="1">IF(AND(L8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-L8)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>21826</v>
+        <v>20826</v>
       </c>
       <c r="O8" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>23766</v>
+        <v>22766</v>
       </c>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>24766</v>
+        <v>23766</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -32932,31 +32932,31 @@
       </c>
       <c r="D9" s="7">
         <f>Proyeccion!F9</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>23684</v>
+        <v>21884</v>
       </c>
       <c r="F9">
         <f ca="1">IF(AND(E9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-E9)/CajasProm,0),0)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G9" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>19684</v>
+        <v>18684</v>
       </c>
       <c r="H9">
         <f ca="1">IF(AND(G9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-G9)/CajasProm,0),0)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I9" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>17684</v>
+        <v>16484</v>
       </c>
       <c r="J9">
         <f ca="1">IF(AND(I9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-I9)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
@@ -32964,7 +32964,7 @@
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>27684</v>
+        <v>26684</v>
       </c>
       <c r="M9">
         <f ca="1">IF(AND(L9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-L9)/CajasProm,0),0)</f>
@@ -32972,15 +32972,15 @@
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>16744</v>
+        <v>15744</v>
       </c>
       <c r="O9" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>18684</v>
+        <v>17684</v>
       </c>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>18634</v>
+        <v>17634</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -32998,31 +32998,31 @@
       </c>
       <c r="D10" s="7">
         <f>Proyeccion!F10</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>24398</v>
+        <v>23698</v>
       </c>
       <c r="F10">
         <f ca="1">IF(AND(E10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-E10)/CajasProm,0),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>22698</v>
+        <v>21698</v>
       </c>
       <c r="H10">
         <f ca="1">IF(AND(G10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-G10)/CajasProm,0),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>20998</v>
+        <v>19698</v>
       </c>
       <c r="J10">
         <f ca="1">IF(AND(I10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-I10)/CajasProm,0),0)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="7">
         <f t="shared" si="0"/>
@@ -33030,23 +33030,23 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>24698</v>
+        <v>22698</v>
       </c>
       <c r="M10">
         <f ca="1">IF(AND(L10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-L10)/CajasProm,0),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>19758</v>
+        <v>18758</v>
       </c>
       <c r="O10" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>21698</v>
+        <v>20698</v>
       </c>
       <c r="P10" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>21648</v>
+        <v>20648</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -33064,31 +33064,31 @@
       </c>
       <c r="D11" s="7">
         <f>Proyeccion!F11</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>19212</v>
+        <v>18612</v>
       </c>
       <c r="F11">
         <f ca="1">IF(AND(E11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-E11)/CajasProm,0),0)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G11" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>17812</v>
+        <v>16812</v>
       </c>
       <c r="H11">
         <f ca="1">IF(AND(G11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-G11)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I11" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>16412</v>
+        <v>15012</v>
       </c>
       <c r="J11">
         <f ca="1">IF(AND(I11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-I11)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" si="0"/>
@@ -33096,23 +33096,23 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>17812</v>
+        <v>16812</v>
       </c>
       <c r="M11">
         <f ca="1">IF(AND(L11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-L11)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N11" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>14872</v>
+        <v>13872</v>
       </c>
       <c r="O11" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>16812</v>
+        <v>15812</v>
       </c>
       <c r="P11" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>16762</v>
+        <v>15762</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -33130,11 +33130,11 @@
       </c>
       <c r="D12" s="7">
         <f>Proyeccion!F12</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E12" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17976</v>
+        <v>17476</v>
       </c>
       <c r="F12">
         <f ca="1">IF(AND(E12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-E12)/CajasProm,0),0)</f>
@@ -33142,19 +33142,19 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16876</v>
+        <v>15876</v>
       </c>
       <c r="H12">
         <f ca="1">IF(AND(G12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-G12)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I12" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14776</v>
+        <v>13276</v>
       </c>
       <c r="J12">
         <f ca="1">IF(AND(I12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-I12)/CajasProm,0),0)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="0"/>
@@ -33162,23 +33162,23 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16876</v>
+        <v>15876</v>
       </c>
       <c r="M12">
         <f ca="1">IF(AND(L12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-L12)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N12" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13936</v>
+        <v>12936</v>
       </c>
       <c r="O12" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15876</v>
+        <v>14876</v>
       </c>
       <c r="P12" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15826</v>
+        <v>14826</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -33196,31 +33196,31 @@
       </c>
       <c r="D13" s="7">
         <f>Proyeccion!F13</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18740</v>
+        <v>17340</v>
       </c>
       <c r="F13">
         <f ca="1">IF(AND(E13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-E13)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G13" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16940</v>
+        <v>15940</v>
       </c>
       <c r="H13">
         <f ca="1">IF(AND(G13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-G13)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I13" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>15140</v>
+        <v>13540</v>
       </c>
       <c r="J13">
         <f ca="1">IF(AND(I13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-I13)/CajasProm,0),0)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="0"/>
@@ -33228,23 +33228,23 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16940</v>
+        <v>15940</v>
       </c>
       <c r="M13">
         <f ca="1">IF(AND(L13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-L13)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N13" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>14000</v>
+        <v>13000</v>
       </c>
       <c r="O13" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15940</v>
+        <v>14940</v>
       </c>
       <c r="P13" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15890</v>
+        <v>14890</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -33262,31 +33262,31 @@
       </c>
       <c r="D14" s="7">
         <f>Proyeccion!F14</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18504</v>
+        <v>17204</v>
       </c>
       <c r="F14">
         <f ca="1">IF(AND(E14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-E14)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G14" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>17004</v>
+        <v>16004</v>
       </c>
       <c r="H14">
         <f ca="1">IF(AND(G14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-G14)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I14" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14504</v>
+        <v>13804</v>
       </c>
       <c r="J14">
         <f ca="1">IF(AND(I14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-I14)/CajasProm,0),0)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="0"/>
@@ -33294,23 +33294,23 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>17004</v>
+        <v>16004</v>
       </c>
       <c r="M14">
         <f ca="1">IF(AND(L14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-L14)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N14" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>14064</v>
+        <v>13064</v>
       </c>
       <c r="O14" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>16004</v>
+        <v>15004</v>
       </c>
       <c r="P14" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15954</v>
+        <v>14954</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -33328,27 +33328,27 @@
       </c>
       <c r="D15" s="7">
         <f>Proyeccion!F15</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18268</v>
+        <v>17068</v>
       </c>
       <c r="F15">
         <f ca="1">IF(AND(E15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-E15)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16068</v>
+        <v>15068</v>
       </c>
       <c r="H15">
         <f ca="1">IF(AND(G15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-G15)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I15" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14868</v>
+        <v>14068</v>
       </c>
       <c r="J15">
         <f ca="1">IF(AND(I15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-I15)/CajasProm,0),0)</f>
@@ -33360,23 +33360,23 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16068</v>
+        <v>15068</v>
       </c>
       <c r="M15">
         <f ca="1">IF(AND(L15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-L15)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N15" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13128</v>
+        <v>12128</v>
       </c>
       <c r="O15" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15068</v>
+        <v>14068</v>
       </c>
       <c r="P15" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15018</v>
+        <v>14018</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -33394,31 +33394,31 @@
       </c>
       <c r="D16" s="7">
         <f>Proyeccion!F16</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18032</v>
+        <v>16932</v>
       </c>
       <c r="F16">
         <f ca="1">IF(AND(E16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-E16)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G16" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16132</v>
+        <v>15132</v>
       </c>
       <c r="H16">
         <f ca="1">IF(AND(G16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-G16)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I16" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>15232</v>
+        <v>13332</v>
       </c>
       <c r="J16">
         <f ca="1">IF(AND(I16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-I16)/CajasProm,0),0)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="0"/>
@@ -33426,23 +33426,23 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16132</v>
+        <v>15132</v>
       </c>
       <c r="M16">
         <f ca="1">IF(AND(L16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-L16)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N16" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13192</v>
+        <v>12192</v>
       </c>
       <c r="O16" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15132</v>
+        <v>14132</v>
       </c>
       <c r="P16" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15082</v>
+        <v>14082</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -33460,7 +33460,7 @@
       </c>
       <c r="D17" s="7">
         <f>Proyeccion!F17</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" ca="1" si="4"/>
@@ -33472,19 +33472,19 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16196</v>
+        <v>15196</v>
       </c>
       <c r="H17">
         <f ca="1">IF(AND(G17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-G17)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I17" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14596</v>
+        <v>13596</v>
       </c>
       <c r="J17">
         <f ca="1">IF(AND(I17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-I17)/CajasProm,0),0)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="0"/>
@@ -33492,23 +33492,23 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16196</v>
+        <v>15196</v>
       </c>
       <c r="M17">
         <f ca="1">IF(AND(L17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-L17)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N17" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13256</v>
+        <v>12256</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15196</v>
+        <v>14196</v>
       </c>
       <c r="P17" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15146</v>
+        <v>14146</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -33526,31 +33526,31 @@
       </c>
       <c r="D18" s="7">
         <f>Proyeccion!F18</f>
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18560</v>
+        <v>17660</v>
       </c>
       <c r="F18">
         <f ca="1">IF(AND(E18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-E18)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G18" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16260</v>
+        <v>15260</v>
       </c>
       <c r="H18">
         <f ca="1">IF(AND(G18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-G18)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I18" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14960</v>
+        <v>13860</v>
       </c>
       <c r="J18">
         <f ca="1">IF(AND(I18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-I18)/CajasProm,0),0)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="0"/>
@@ -33558,23 +33558,23 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16260</v>
+        <v>15260</v>
       </c>
       <c r="M18">
         <f ca="1">IF(AND(L18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-L18)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N18" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13320</v>
+        <v>12320</v>
       </c>
       <c r="O18" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15260</v>
+        <v>14260</v>
       </c>
       <c r="P18" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15210</v>
+        <v>14210</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="63.95" customHeight="1">

</xml_diff>

<commit_message>
plan de compras: Bolivia 1 camion por semana siempre, tambien en la semana en curso
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0102A0E-9300-4D41-A032-F8B9C2C29FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935BD00B-2EF7-4EC9-9B16-04B00CF42E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,12 +110,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="681">
   <si>
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 01/10/2026 12:49 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 01/10/2026 12:52 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -727,6 +727,15 @@
     <t>nota 25/09: Milciades 1, nota completa 25/09: lunes confirmado</t>
   </si>
   <si>
+    <t>Bolivia (supuesto)</t>
+  </si>
+  <si>
+    <t>Supuesto</t>
+  </si>
+  <si>
+    <t>supuesto: 1 camion BO por semana, descarga el lunes (Gonzalo 01/10)</t>
+  </si>
+  <si>
     <t>Ivo zimer</t>
   </si>
   <si>
@@ -785,15 +794,6 @@
   </si>
   <si>
     <t>nota 30/09: Milciades 2, lunes</t>
-  </si>
-  <si>
-    <t>Bolivia (supuesto)</t>
-  </si>
-  <si>
-    <t>Supuesto</t>
-  </si>
-  <si>
-    <t>supuesto: 1 camion BO por semana, descarga el lunes (Gonzalo 01/10)</t>
   </si>
   <si>
     <t>nota 30/09: tersa; transportista supuesto = semana anterior</t>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>18868</v>
+        <v>19918</v>
       </c>
       <c r="D8" s="7">
         <f>Demanda!H9</f>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="H8" s="7">
         <f ca="1">Proyeccion!L8</f>
-        <v>25766</v>
+        <v>25816</v>
       </c>
       <c r="I8" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="H9" s="7">
         <f ca="1">Proyeccion!L9</f>
-        <v>25684</v>
+        <v>25734</v>
       </c>
       <c r="I9" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H10" s="7">
         <f ca="1">Proyeccion!L10</f>
-        <v>25698</v>
+        <v>25748</v>
       </c>
       <c r="I10" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="H11" s="7">
         <f ca="1">Proyeccion!L11</f>
-        <v>25812</v>
+        <v>25862</v>
       </c>
       <c r="I11" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="H12" s="7">
         <f ca="1">Proyeccion!L12</f>
-        <v>25876</v>
+        <v>25926</v>
       </c>
       <c r="I12" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4306,7 +4306,7 @@
       </c>
       <c r="H13" s="7">
         <f ca="1">Proyeccion!L13</f>
-        <v>25940</v>
+        <v>25990</v>
       </c>
       <c r="I13" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="H14" s="7">
         <f ca="1">Proyeccion!L14</f>
-        <v>25004</v>
+        <v>25054</v>
       </c>
       <c r="I14" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="H15" s="7">
         <f ca="1">Proyeccion!L15</f>
-        <v>25068</v>
+        <v>25118</v>
       </c>
       <c r="I15" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="H16" s="7">
         <f ca="1">Proyeccion!L16</f>
-        <v>25132</v>
+        <v>25182</v>
       </c>
       <c r="I16" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="H17" s="7">
         <f ca="1">Proyeccion!L17</f>
-        <v>25196</v>
+        <v>25246</v>
       </c>
       <c r="I17" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="H18" s="7">
         <f ca="1">Proyeccion!L18</f>
-        <v>25260</v>
+        <v>25310</v>
       </c>
       <c r="I18" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B9" s="25">
         <f ca="1">IFERROR(INDEX(PrACargar,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>303</v>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B10" s="24">
         <f ca="1">AVERAGEIFS(PrCobertura,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8.3371666666666666</v>
+        <v>8.3496666666666659</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>305</v>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="B12" s="25">
         <f ca="1">SUMIFS(PrACargar,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>309</v>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="B19" s="24">
         <f ca="1">AVERAGEIFS(PrCamiones,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>14</v>
+        <v>14.25</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>322</v>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="B20" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BR",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.59175250331981477</v>
+        <v>0.58080879244751304</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>324</v>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="B21" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"PY",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.35172092021677492</v>
+        <v>0.34521628857263631</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>3</v>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B22" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>5.6526576463410257E-2</v>
+        <v>7.3974918979850646E-2</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>3</v>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B23" s="12">
         <f ca="1">SUMIFS(CgCosto,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>405019.83999999979</v>
+        <v>416359.83999999973</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>328</v>
@@ -4853,7 +4853,7 @@
       </c>
       <c r="B24" s="25">
         <f>COUNTIFS(CgEstado,"Supuesto*",CgCuenta,1)</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>330</v>
@@ -5149,7 +5149,7 @@
         <v>197</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D5">
         <v>12</v>
@@ -5216,7 +5216,7 @@
         <v>401</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D6">
         <v>12</v>
@@ -5283,7 +5283,7 @@
         <v>196</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D7">
         <v>10</v>
@@ -5350,7 +5350,7 @@
         <v>411</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D8">
         <v>7</v>
@@ -5417,7 +5417,7 @@
         <v>416</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D9">
         <v>6</v>
@@ -5481,10 +5481,10 @@
         <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D10">
         <v>5</v>
@@ -5551,7 +5551,7 @@
         <v>424</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -5612,7 +5612,7 @@
         <v>427</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D12">
         <v>3</v>
@@ -6409,7 +6409,7 @@
         <v>1008</v>
       </c>
       <c r="K25" s="33" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="L25" s="33"/>
       <c r="M25" s="35">
@@ -7498,7 +7498,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="3" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>627</v>
@@ -10610,36 +10610,36 @@
         <v>mar</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>205</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>206</v>
+        <v>3</v>
       </c>
       <c r="G12" s="8">
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="H12" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="J12" s="6"/>
       <c r="K12">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L12" s="5">
         <f t="shared" si="4"/>
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="M12" s="5">
         <f t="shared" si="5"/>
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="N12">
         <f t="shared" si="6"/>
@@ -10647,18 +10647,18 @@
       </c>
       <c r="O12" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>10.8</v>
       </c>
       <c r="P12" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>11340</v>
       </c>
       <c r="Q12" s="9" t="s">
         <v>207</v>
       </c>
       <c r="R12" s="5">
         <f t="shared" si="9"/>
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="S12" s="5">
         <f t="shared" si="10"/>
@@ -10666,7 +10666,7 @@
       </c>
       <c r="T12" s="7">
         <f t="shared" ca="1" si="11"/>
-        <v>1008</v>
+        <v>0</v>
       </c>
       <c r="U12" t="str">
         <f t="shared" si="12"/>
@@ -10686,20 +10686,20 @@
         <v>mar</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>3</v>
+        <v>209</v>
       </c>
       <c r="G13" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H13" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>199</v>
@@ -10707,11 +10707,11 @@
       <c r="J13" s="6"/>
       <c r="K13">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="5">
         <f t="shared" si="4"/>
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="M13" s="5">
         <f t="shared" si="5"/>
@@ -10723,18 +10723,18 @@
       </c>
       <c r="O13" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P13" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q13" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="R13" s="5">
         <f t="shared" si="9"/>
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="S13" s="5">
         <f t="shared" si="10"/>
@@ -10742,7 +10742,7 @@
       </c>
       <c r="T13" s="7">
         <f t="shared" ca="1" si="11"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="U13" t="str">
         <f t="shared" si="12"/>
@@ -10755,27 +10755,27 @@
         <v>10</v>
       </c>
       <c r="B14" s="6">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
-        <v>mié</v>
+        <v>mar</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>210</v>
+        <v>3</v>
       </c>
       <c r="G14" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H14" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>199</v>
@@ -10783,7 +10783,7 @@
       <c r="J14" s="6"/>
       <c r="K14">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L14" s="5">
         <f t="shared" si="4"/>
@@ -10799,18 +10799,18 @@
       </c>
       <c r="O14" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P14" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q14" s="9" t="s">
         <v>211</v>
       </c>
       <c r="R14" s="5">
         <f t="shared" si="9"/>
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="S14" s="5">
         <f t="shared" si="10"/>
@@ -10818,7 +10818,7 @@
       </c>
       <c r="T14" s="7">
         <f t="shared" ca="1" si="11"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="U14" t="str">
         <f t="shared" si="12"/>
@@ -10882,7 +10882,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="R15" s="5">
         <f t="shared" si="9"/>
@@ -10917,10 +10917,10 @@
         <v>58</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G16" s="8">
         <v>1008</v>
@@ -10958,7 +10958,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q16" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="R16" s="5">
         <f t="shared" si="9"/>
@@ -10983,20 +10983,20 @@
         <v>13</v>
       </c>
       <c r="B17" s="6">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>mié</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G17" s="8">
         <v>1008</v>
@@ -11015,11 +11015,11 @@
       </c>
       <c r="L17" s="5">
         <f t="shared" si="4"/>
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="M17" s="5">
         <f t="shared" si="5"/>
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="N17">
         <f t="shared" si="6"/>
@@ -11034,11 +11034,11 @@
         <v>7146.72</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="R17" s="5">
         <f t="shared" si="9"/>
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="S17" s="5">
         <f t="shared" si="10"/>
@@ -11046,7 +11046,7 @@
       </c>
       <c r="T17" s="7">
         <f t="shared" ca="1" si="11"/>
-        <v>0</v>
+        <v>1008</v>
       </c>
       <c r="U17" t="str">
         <f t="shared" si="12"/>
@@ -11069,17 +11069,17 @@
         <v>58</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="G18" s="8">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="H18" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I18" s="9" t="s">
         <v>199</v>
@@ -11107,10 +11107,10 @@
       </c>
       <c r="P18" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>7146.72</v>
       </c>
       <c r="Q18" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R18" s="5">
         <f t="shared" si="9"/>
@@ -11145,17 +11145,17 @@
         <v>58</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="G19" s="8">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="H19" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I19" s="9" t="s">
         <v>199</v>
@@ -11183,10 +11183,10 @@
       </c>
       <c r="P19" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6636.24</v>
       </c>
       <c r="Q19" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R19" s="5">
         <f t="shared" si="9"/>
@@ -11221,10 +11221,10 @@
         <v>58</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G20" s="8">
         <v>1008</v>
@@ -11262,7 +11262,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q20" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R20" s="5">
         <f t="shared" si="9"/>
@@ -11297,10 +11297,10 @@
         <v>58</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G21" s="8">
         <v>1008</v>
@@ -11338,7 +11338,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q21" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R21" s="5">
         <f t="shared" si="9"/>
@@ -11373,10 +11373,10 @@
         <v>58</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G22" s="8">
         <v>1008</v>
@@ -11414,7 +11414,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R22" s="5">
         <f t="shared" si="9"/>
@@ -11449,10 +11449,10 @@
         <v>58</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G23" s="8">
         <v>1008</v>
@@ -11490,7 +11490,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q23" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R23" s="5">
         <f t="shared" si="9"/>
@@ -11525,10 +11525,10 @@
         <v>58</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G24" s="8">
         <v>1008</v>
@@ -11566,7 +11566,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q24" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="R24" s="5">
         <f t="shared" si="9"/>
@@ -11591,27 +11591,27 @@
         <v>21</v>
       </c>
       <c r="B25" s="6">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>vie</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>190</v>
+        <v>217</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>3</v>
+        <v>213</v>
       </c>
       <c r="G25" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H25" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I25" s="9" t="s">
         <v>199</v>
@@ -11619,11 +11619,11 @@
       <c r="J25" s="6"/>
       <c r="K25">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L25" s="5">
         <f t="shared" si="4"/>
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="M25" s="5">
         <f t="shared" si="5"/>
@@ -11635,18 +11635,18 @@
       </c>
       <c r="O25" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P25" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q25" s="9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="R25" s="5">
         <f t="shared" si="9"/>
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="S25" s="5">
         <f t="shared" si="10"/>
@@ -11677,7 +11677,7 @@
         <v>59</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>3</v>
@@ -11718,7 +11718,7 @@
         <v>6860</v>
       </c>
       <c r="Q26" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="R26" s="5">
         <f t="shared" si="9"/>
@@ -11753,7 +11753,7 @@
         <v>59</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>3</v>
@@ -11794,7 +11794,7 @@
         <v>6860</v>
       </c>
       <c r="Q27" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="R27" s="5">
         <f t="shared" si="9"/>
@@ -11819,43 +11819,43 @@
         <v>24</v>
       </c>
       <c r="B28" s="6">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>lun</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G28" s="8">
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="H28" s="7">
         <f t="shared" si="2"/>
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>226</v>
+        <v>199</v>
       </c>
       <c r="J28" s="6"/>
       <c r="K28">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L28" s="5">
         <f t="shared" si="4"/>
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="M28" s="5">
         <f t="shared" si="5"/>
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="N28">
         <f t="shared" si="6"/>
@@ -11863,22 +11863,22 @@
       </c>
       <c r="O28" s="10">
         <f t="shared" si="7"/>
-        <v>10.8</v>
+        <v>7</v>
       </c>
       <c r="P28" s="7">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>6860</v>
       </c>
       <c r="Q28" s="9" t="s">
         <v>227</v>
       </c>
       <c r="R28" s="5">
         <f t="shared" si="9"/>
-        <v>46309</v>
+        <v>46305</v>
       </c>
       <c r="S28" s="5">
         <f t="shared" si="10"/>
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="T28" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -11902,36 +11902,36 @@
         <v>mar</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>213</v>
+        <v>3</v>
       </c>
       <c r="G29" s="8">
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="H29" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="J29" s="6"/>
       <c r="K29">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L29" s="5">
         <f t="shared" si="4"/>
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="M29" s="5">
         <f t="shared" si="5"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="N29">
         <f t="shared" si="6"/>
@@ -11939,18 +11939,18 @@
       </c>
       <c r="O29" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>10.8</v>
       </c>
       <c r="P29" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>11340</v>
       </c>
       <c r="Q29" s="9" t="s">
-        <v>228</v>
+        <v>207</v>
       </c>
       <c r="R29" s="5">
         <f t="shared" si="9"/>
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="S29" s="5">
         <f t="shared" si="10"/>
@@ -11981,10 +11981,10 @@
         <v>58</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G30" s="8">
         <v>1008</v>
@@ -12022,7 +12022,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q30" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="R30" s="5">
         <f t="shared" si="9"/>
@@ -12057,10 +12057,10 @@
         <v>58</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G31" s="8">
         <v>1008</v>
@@ -12098,7 +12098,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q31" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="R31" s="5">
         <f t="shared" si="9"/>
@@ -12130,20 +12130,20 @@
         <v>mar</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>3</v>
+        <v>213</v>
       </c>
       <c r="G32" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H32" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I32" s="9" t="s">
         <v>199</v>
@@ -12151,11 +12151,11 @@
       <c r="J32" s="6"/>
       <c r="K32">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L32" s="5">
         <f t="shared" si="4"/>
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="M32" s="5">
         <f t="shared" si="5"/>
@@ -12167,18 +12167,18 @@
       </c>
       <c r="O32" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P32" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q32" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="R32" s="5">
         <f t="shared" si="9"/>
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S32" s="5">
         <f t="shared" si="10"/>
@@ -12209,7 +12209,7 @@
         <v>59</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>3</v>
@@ -12250,7 +12250,7 @@
         <v>6860</v>
       </c>
       <c r="Q33" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="R33" s="5">
         <f t="shared" si="9"/>
@@ -12275,27 +12275,27 @@
         <v>30</v>
       </c>
       <c r="B34" s="6">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="1"/>
-        <v>mié</v>
+        <v>mar</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>210</v>
+        <v>3</v>
       </c>
       <c r="G34" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H34" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I34" s="9" t="s">
         <v>199</v>
@@ -12303,7 +12303,7 @@
       <c r="J34" s="6"/>
       <c r="K34">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L34" s="5">
         <f t="shared" si="4"/>
@@ -12319,18 +12319,18 @@
       </c>
       <c r="O34" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P34" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q34" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="R34" s="5">
         <f t="shared" si="9"/>
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="S34" s="5">
         <f t="shared" si="10"/>
@@ -12361,17 +12361,17 @@
         <v>58</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="G35" s="8">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="H35" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I35" s="9" t="s">
         <v>199</v>
@@ -12399,10 +12399,10 @@
       </c>
       <c r="P35" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>7146.72</v>
       </c>
       <c r="Q35" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R35" s="5">
         <f t="shared" si="9"/>
@@ -12437,17 +12437,17 @@
         <v>58</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="G36" s="8">
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="H36" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>936</v>
       </c>
       <c r="I36" s="9" t="s">
         <v>199</v>
@@ -12475,10 +12475,10 @@
       </c>
       <c r="P36" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6636.24</v>
       </c>
       <c r="Q36" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="R36" s="5">
         <f t="shared" si="9"/>
@@ -12503,20 +12503,20 @@
         <v>33</v>
       </c>
       <c r="B37" s="6">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>mié</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G37" s="8">
         <v>1008</v>
@@ -12535,11 +12535,11 @@
       </c>
       <c r="L37" s="5">
         <f t="shared" si="4"/>
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="M37" s="5">
         <f t="shared" si="5"/>
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="N37">
         <f t="shared" si="6"/>
@@ -12554,11 +12554,11 @@
         <v>7146.72</v>
       </c>
       <c r="Q37" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="R37" s="5">
         <f t="shared" si="9"/>
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="S37" s="5">
         <f t="shared" si="10"/>
@@ -12589,10 +12589,10 @@
         <v>58</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G38" s="8">
         <v>1008</v>
@@ -12665,10 +12665,10 @@
         <v>58</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G39" s="8">
         <v>1008</v>
@@ -12741,10 +12741,10 @@
         <v>58</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="G40" s="8">
         <v>1008</v>
@@ -12807,27 +12807,27 @@
         <v>37</v>
       </c>
       <c r="B41" s="6">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="1"/>
-        <v>sáb</v>
+        <v>vie</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="G41" s="8">
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="H41" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>1008</v>
       </c>
       <c r="I41" s="9" t="s">
         <v>199</v>
@@ -12839,7 +12839,7 @@
       </c>
       <c r="L41" s="5">
         <f t="shared" si="4"/>
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="M41" s="5">
         <f t="shared" si="5"/>
@@ -12855,14 +12855,14 @@
       </c>
       <c r="P41" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>7146.72</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R41" s="5">
         <f t="shared" si="9"/>
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="S41" s="5">
         <f t="shared" si="10"/>
@@ -12883,39 +12883,39 @@
         <v>38</v>
       </c>
       <c r="B42" s="6">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>sáb</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>3</v>
+        <v>221</v>
       </c>
       <c r="G42" s="8">
-        <v>980</v>
+        <v>936</v>
       </c>
       <c r="H42" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>936</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>226</v>
+        <v>199</v>
       </c>
       <c r="J42" s="6"/>
       <c r="K42">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L42" s="5">
         <f t="shared" si="4"/>
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="M42" s="5">
         <f t="shared" si="5"/>
@@ -12927,18 +12927,18 @@
       </c>
       <c r="O42" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P42" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>6636.24</v>
       </c>
       <c r="Q42" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="R42" s="5">
         <f t="shared" si="9"/>
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="S42" s="5">
         <f t="shared" si="10"/>
@@ -12982,7 +12982,7 @@
         <v>980</v>
       </c>
       <c r="I43" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J43" s="6"/>
       <c r="K43">
@@ -13058,7 +13058,7 @@
         <v>980</v>
       </c>
       <c r="I44" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J44" s="6"/>
       <c r="K44">
@@ -13134,7 +13134,7 @@
         <v>980</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J45" s="6"/>
       <c r="K45">
@@ -13210,7 +13210,7 @@
         <v>980</v>
       </c>
       <c r="I46" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46">
@@ -13263,43 +13263,43 @@
         <v>43</v>
       </c>
       <c r="B47" s="6">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>lun</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G47" s="8">
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="H47" s="7">
         <f t="shared" si="2"/>
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L47" s="5">
         <f t="shared" si="4"/>
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="M47" s="5">
         <f t="shared" si="5"/>
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="N47">
         <f t="shared" si="6"/>
@@ -13307,22 +13307,22 @@
       </c>
       <c r="O47" s="10">
         <f t="shared" si="7"/>
-        <v>10.8</v>
+        <v>7</v>
       </c>
       <c r="P47" s="7">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>6860</v>
       </c>
       <c r="Q47" s="9" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="R47" s="5">
         <f t="shared" si="9"/>
-        <v>46316</v>
+        <v>46312</v>
       </c>
       <c r="S47" s="5">
         <f t="shared" si="10"/>
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="T47" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -13339,35 +13339,35 @@
         <v>44</v>
       </c>
       <c r="B48" s="6">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>mar</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>238</v>
+        <v>205</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G48" s="8">
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="H48" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="J48" s="6"/>
       <c r="K48">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L48" s="5">
         <f t="shared" si="4"/>
@@ -13383,18 +13383,18 @@
       </c>
       <c r="O48" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>10.8</v>
       </c>
       <c r="P48" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>11340</v>
       </c>
       <c r="Q48" s="9" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="R48" s="5">
         <f t="shared" si="9"/>
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="S48" s="5">
         <f t="shared" si="10"/>
@@ -13947,39 +13947,39 @@
         <v>52</v>
       </c>
       <c r="B56" s="6">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>vie</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G56" s="8">
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="H56" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1008</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="J56" s="6"/>
       <c r="K56">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L56" s="5">
         <f t="shared" si="4"/>
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="M56" s="5">
         <f t="shared" si="5"/>
@@ -13991,18 +13991,18 @@
       </c>
       <c r="O56" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>7.09</v>
       </c>
       <c r="P56" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>7146.72</v>
       </c>
       <c r="Q56" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="R56" s="5">
         <f t="shared" si="9"/>
-        <v>46319</v>
+        <v>46317</v>
       </c>
       <c r="S56" s="5">
         <f t="shared" si="10"/>
@@ -14046,7 +14046,7 @@
         <v>980</v>
       </c>
       <c r="I57" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J57" s="6"/>
       <c r="K57">
@@ -14122,7 +14122,7 @@
         <v>980</v>
       </c>
       <c r="I58" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58">
@@ -14198,7 +14198,7 @@
         <v>980</v>
       </c>
       <c r="I59" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59">
@@ -14274,7 +14274,7 @@
         <v>980</v>
       </c>
       <c r="I60" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J60" s="6"/>
       <c r="K60">
@@ -14327,43 +14327,43 @@
         <v>57</v>
       </c>
       <c r="B61" s="6">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>lun</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G61" s="8">
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="H61" s="7">
         <f t="shared" si="2"/>
-        <v>1050</v>
+        <v>980</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="J61" s="6"/>
       <c r="K61">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L61" s="5">
         <f t="shared" si="4"/>
-        <v>46321</v>
+        <v>46318</v>
       </c>
       <c r="M61" s="5">
         <f t="shared" si="5"/>
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="N61">
         <f t="shared" si="6"/>
@@ -14371,22 +14371,22 @@
       </c>
       <c r="O61" s="10">
         <f t="shared" si="7"/>
-        <v>10.8</v>
+        <v>7</v>
       </c>
       <c r="P61" s="7">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>6860</v>
       </c>
       <c r="Q61" s="9" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="R61" s="5">
         <f t="shared" si="9"/>
-        <v>46323</v>
+        <v>46319</v>
       </c>
       <c r="S61" s="5">
         <f t="shared" si="10"/>
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="T61" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -14403,35 +14403,35 @@
         <v>58</v>
       </c>
       <c r="B62" s="6">
-        <v>46318</v>
+        <v>46315</v>
       </c>
       <c r="C62" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>mar</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>238</v>
+        <v>205</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G62" s="8">
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="H62" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>1050</v>
       </c>
       <c r="I62" s="9" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L62" s="5">
         <f t="shared" si="4"/>
@@ -14447,18 +14447,18 @@
       </c>
       <c r="O62" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>10.8</v>
       </c>
       <c r="P62" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>11340</v>
       </c>
       <c r="Q62" s="9" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="R62" s="5">
         <f t="shared" si="9"/>
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="S62" s="5">
         <f t="shared" si="10"/>
@@ -15011,7 +15011,7 @@
         <v>66</v>
       </c>
       <c r="B70" s="6">
-        <v>46325</v>
+        <v>46318</v>
       </c>
       <c r="C70" t="str">
         <f t="shared" si="14"/>
@@ -15043,11 +15043,11 @@
       </c>
       <c r="L70" s="5">
         <f t="shared" si="17"/>
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="M70" s="5">
         <f t="shared" si="18"/>
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="N70">
         <f t="shared" si="19"/>
@@ -15066,11 +15066,11 @@
       </c>
       <c r="R70" s="5">
         <f t="shared" si="22"/>
-        <v>46331</v>
+        <v>46324</v>
       </c>
       <c r="S70" s="5">
         <f t="shared" si="23"/>
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="T70" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -15619,7 +15619,7 @@
         <v>74</v>
       </c>
       <c r="B78" s="6">
-        <v>46332</v>
+        <v>46325</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="14"/>
@@ -15651,11 +15651,11 @@
       </c>
       <c r="L78" s="5">
         <f t="shared" si="17"/>
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="M78" s="5">
         <f t="shared" si="18"/>
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="N78">
         <f t="shared" si="19"/>
@@ -15674,11 +15674,11 @@
       </c>
       <c r="R78" s="5">
         <f t="shared" si="22"/>
-        <v>46338</v>
+        <v>46331</v>
       </c>
       <c r="S78" s="5">
         <f t="shared" si="23"/>
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="T78" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -16227,7 +16227,7 @@
         <v>82</v>
       </c>
       <c r="B86" s="6">
-        <v>46339</v>
+        <v>46332</v>
       </c>
       <c r="C86" t="str">
         <f t="shared" si="14"/>
@@ -16259,11 +16259,11 @@
       </c>
       <c r="L86" s="5">
         <f t="shared" si="17"/>
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="M86" s="5">
         <f t="shared" si="18"/>
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="N86">
         <f t="shared" si="19"/>
@@ -16282,11 +16282,11 @@
       </c>
       <c r="R86" s="5">
         <f t="shared" si="22"/>
-        <v>46345</v>
+        <v>46338</v>
       </c>
       <c r="S86" s="5">
         <f t="shared" si="23"/>
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="T86" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -16835,7 +16835,7 @@
         <v>90</v>
       </c>
       <c r="B94" s="6">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="C94" t="str">
         <f t="shared" si="14"/>
@@ -16867,11 +16867,11 @@
       </c>
       <c r="L94" s="5">
         <f t="shared" si="17"/>
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="M94" s="5">
         <f t="shared" si="18"/>
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="N94">
         <f t="shared" si="19"/>
@@ -16890,11 +16890,11 @@
       </c>
       <c r="R94" s="5">
         <f t="shared" si="22"/>
-        <v>46352</v>
+        <v>46345</v>
       </c>
       <c r="S94" s="5">
         <f t="shared" si="23"/>
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="T94" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -17443,7 +17443,7 @@
         <v>98</v>
       </c>
       <c r="B102" s="6">
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="14"/>
@@ -17475,11 +17475,11 @@
       </c>
       <c r="L102" s="5">
         <f t="shared" si="17"/>
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="M102" s="5">
         <f t="shared" si="18"/>
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="N102">
         <f t="shared" si="19"/>
@@ -17498,11 +17498,11 @@
       </c>
       <c r="R102" s="5">
         <f t="shared" si="22"/>
-        <v>46359</v>
+        <v>46352</v>
       </c>
       <c r="S102" s="5">
         <f t="shared" si="23"/>
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="T102" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -18051,7 +18051,7 @@
         <v>106</v>
       </c>
       <c r="B110" s="6">
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="14"/>
@@ -18083,11 +18083,11 @@
       </c>
       <c r="L110" s="5">
         <f t="shared" si="17"/>
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="M110" s="5">
         <f t="shared" si="18"/>
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="N110">
         <f t="shared" si="19"/>
@@ -18106,11 +18106,11 @@
       </c>
       <c r="R110" s="5">
         <f t="shared" si="22"/>
-        <v>46366</v>
+        <v>46359</v>
       </c>
       <c r="S110" s="5">
         <f t="shared" si="23"/>
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="T110" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -18659,7 +18659,7 @@
         <v>114</v>
       </c>
       <c r="B118" s="6">
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="14"/>
@@ -18691,11 +18691,11 @@
       </c>
       <c r="L118" s="5">
         <f t="shared" si="17"/>
-        <v>46370</v>
+        <v>46363</v>
       </c>
       <c r="M118" s="5">
         <f t="shared" si="18"/>
-        <v>46370</v>
+        <v>46363</v>
       </c>
       <c r="N118">
         <f t="shared" si="19"/>
@@ -18714,11 +18714,11 @@
       </c>
       <c r="R118" s="5">
         <f t="shared" si="22"/>
-        <v>46373</v>
+        <v>46366</v>
       </c>
       <c r="S118" s="5">
         <f t="shared" si="23"/>
-        <v>46370</v>
+        <v>46363</v>
       </c>
       <c r="T118" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19267,7 +19267,7 @@
         <v>122</v>
       </c>
       <c r="B126" s="6">
-        <v>46374</v>
+        <v>46367</v>
       </c>
       <c r="C126" t="str">
         <f t="shared" si="14"/>
@@ -19299,11 +19299,11 @@
       </c>
       <c r="L126" s="5">
         <f t="shared" si="17"/>
-        <v>46377</v>
+        <v>46370</v>
       </c>
       <c r="M126" s="5">
         <f t="shared" si="18"/>
-        <v>46377</v>
+        <v>46370</v>
       </c>
       <c r="N126">
         <f t="shared" si="19"/>
@@ -19322,11 +19322,11 @@
       </c>
       <c r="R126" s="5">
         <f t="shared" si="22"/>
-        <v>46380</v>
+        <v>46373</v>
       </c>
       <c r="S126" s="5">
         <f t="shared" si="23"/>
-        <v>46377</v>
+        <v>46370</v>
       </c>
       <c r="T126" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19870,61 +19870,75 @@
       </c>
     </row>
     <row r="134" spans="1:21">
-      <c r="A134" t="str">
+      <c r="A134">
         <f t="shared" si="26"/>
-        <v/>
-      </c>
-      <c r="B134" s="6"/>
+        <v>130</v>
+      </c>
+      <c r="B134" s="6">
+        <v>46374</v>
+      </c>
       <c r="C134" t="str">
         <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="D134" s="9"/>
-      <c r="E134" s="9"/>
-      <c r="F134" s="9"/>
-      <c r="G134" s="8"/>
-      <c r="H134" s="7" t="str">
+        <v>vie</v>
+      </c>
+      <c r="D134" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E134" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="F134" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G134" s="8">
+        <v>1008</v>
+      </c>
+      <c r="H134" s="7">
         <f t="shared" si="28"/>
-        <v/>
-      </c>
-      <c r="I134" s="9"/>
+        <v>1008</v>
+      </c>
+      <c r="I134" s="9" t="s">
+        <v>239</v>
+      </c>
       <c r="J134" s="6"/>
-      <c r="K134" t="str">
+      <c r="K134">
         <f t="shared" si="29"/>
-        <v/>
-      </c>
-      <c r="L134" s="5" t="str">
+        <v>3</v>
+      </c>
+      <c r="L134" s="5">
         <f t="shared" si="30"/>
-        <v/>
-      </c>
-      <c r="M134" s="5" t="str">
+        <v>46377</v>
+      </c>
+      <c r="M134" s="5">
         <f t="shared" si="31"/>
-        <v/>
-      </c>
-      <c r="N134" t="str">
+        <v>46377</v>
+      </c>
+      <c r="N134">
         <f t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="O134" s="10" t="str">
+        <v>1</v>
+      </c>
+      <c r="O134" s="10">
         <f t="shared" si="33"/>
-        <v/>
-      </c>
-      <c r="P134" s="7" t="str">
+        <v>7.09</v>
+      </c>
+      <c r="P134" s="7">
         <f t="shared" si="34"/>
-        <v/>
-      </c>
-      <c r="Q134" s="9"/>
-      <c r="R134" s="5" t="str">
+        <v>7146.72</v>
+      </c>
+      <c r="Q134" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="R134" s="5">
         <f t="shared" si="35"/>
-        <v/>
-      </c>
-      <c r="S134" s="5" t="str">
+        <v>46380</v>
+      </c>
+      <c r="S134" s="5">
         <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="T134" s="7" t="str">
-        <f t="shared" si="37"/>
-        <v/>
+        <v>46377</v>
+      </c>
+      <c r="T134" s="7">
+        <f t="shared" ca="1" si="37"/>
+        <v>0</v>
       </c>
       <c r="U134" t="str">
         <f t="shared" si="38"/>
@@ -30537,11 +30551,11 @@
       </c>
       <c r="D8" s="7">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="2"/>
-        <v>18868</v>
+        <v>19918</v>
       </c>
       <c r="F8" s="7">
         <f>ROUND(Demanda!H8,0)</f>
@@ -30549,7 +30563,7 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" si="3"/>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="H8" s="7">
         <f ca="1">SUM($K$6:K7)*CajasProm</f>
@@ -30557,7 +30571,7 @@
       </c>
       <c r="I8" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="J8" s="21">
         <f t="shared" si="5"/>
@@ -30565,19 +30579,19 @@
       </c>
       <c r="K8" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25766</v>
+        <v>25816</v>
       </c>
       <c r="M8" s="22">
         <f ca="1">IF(Demanda!H9=0,"",L8/(Demanda!H9/DiasVenta))</f>
-        <v>8.5886666666666667</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 2</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="O8" s="7">
         <f>O7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L8,0)</f>
@@ -30597,15 +30611,15 @@
       </c>
       <c r="S8" s="7">
         <f>S7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N8,0)</f>
-        <v>362</v>
+        <v>1412</v>
       </c>
       <c r="T8" s="22">
         <f>IF(Demanda!N9=0,"",S8/(Demanda!N9/DiasVenta))</f>
-        <v>1.699530516431925</v>
+        <v>6.629107981220657</v>
       </c>
       <c r="U8" t="str">
         <f t="shared" si="9"/>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -30619,7 +30633,7 @@
       </c>
       <c r="C9" s="7">
         <f t="shared" si="10"/>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="1"/>
@@ -30635,15 +30649,15 @@
       </c>
       <c r="G9" s="7">
         <f t="shared" si="3"/>
-        <v>16684</v>
+        <v>17734</v>
       </c>
       <c r="H9" s="7">
         <f ca="1">SUM($K$6:K8)*CajasProm</f>
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>18684</v>
+        <v>18734</v>
       </c>
       <c r="J9" s="21">
         <f t="shared" si="5"/>
@@ -30655,11 +30669,11 @@
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25684</v>
+        <v>25734</v>
       </c>
       <c r="M9" s="22">
         <f ca="1">IF(Demanda!H10=0,"",L9/(Demanda!H10/DiasVenta))</f>
-        <v>8.5613333333333337</v>
+        <v>8.5779999999999994</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30683,15 +30697,15 @@
       </c>
       <c r="S9" s="7">
         <f>S8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N9,0)</f>
-        <v>134</v>
+        <v>1184</v>
       </c>
       <c r="T9" s="22">
         <f>IF(Demanda!N10=0,"",S9/(Demanda!N10/DiasVenta))</f>
-        <v>0.62910798122065725</v>
+        <v>5.55868544600939</v>
       </c>
       <c r="U9" t="str">
         <f t="shared" si="9"/>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
     </row>
     <row r="10" spans="1:21">
@@ -30705,7 +30719,7 @@
       </c>
       <c r="C10" s="7">
         <f t="shared" si="10"/>
-        <v>16684</v>
+        <v>17734</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
@@ -30721,15 +30735,15 @@
       </c>
       <c r="G10" s="7">
         <f t="shared" si="3"/>
-        <v>12698</v>
+        <v>13748</v>
       </c>
       <c r="H10" s="7">
         <f ca="1">SUM($K$6:K9)*CajasProm</f>
-        <v>9000</v>
+        <v>8000</v>
       </c>
       <c r="I10" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>21698</v>
+        <v>21748</v>
       </c>
       <c r="J10" s="21">
         <f t="shared" si="5"/>
@@ -30741,11 +30755,11 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25698</v>
+        <v>25748</v>
       </c>
       <c r="M10" s="22">
         <f ca="1">IF(Demanda!H11=0,"",L10/(Demanda!H11/DiasVenta))</f>
-        <v>8.5660000000000007</v>
+        <v>8.5826666666666664</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30769,15 +30783,15 @@
       </c>
       <c r="S10" s="7">
         <f>S9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N10,0)</f>
-        <v>-94</v>
+        <v>956</v>
       </c>
       <c r="T10" s="22">
         <f>IF(Demanda!N11=0,"",S10/(Demanda!N11/DiasVenta))</f>
-        <v>-0.44131455399061031</v>
+        <v>4.488262910798122</v>
       </c>
       <c r="U10" t="str">
         <f t="shared" si="9"/>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
     </row>
     <row r="11" spans="1:21">
@@ -30791,7 +30805,7 @@
       </c>
       <c r="C11" s="7">
         <f t="shared" si="10"/>
-        <v>12698</v>
+        <v>13748</v>
       </c>
       <c r="D11" s="7">
         <f t="shared" si="1"/>
@@ -30807,15 +30821,15 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" si="3"/>
-        <v>3812</v>
+        <v>4862</v>
       </c>
       <c r="H11" s="7">
         <f ca="1">SUM($K$6:K10)*CajasProm</f>
-        <v>13000</v>
+        <v>12000</v>
       </c>
       <c r="I11" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16812</v>
+        <v>16862</v>
       </c>
       <c r="J11" s="21">
         <f t="shared" si="5"/>
@@ -30827,11 +30841,11 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25812</v>
+        <v>25862</v>
       </c>
       <c r="M11" s="22">
         <f ca="1">IF(Demanda!H12=0,"",L11/(Demanda!H12/DiasVenta))</f>
-        <v>8.6039999999999992</v>
+        <v>8.6206666666666667</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30855,15 +30869,15 @@
       </c>
       <c r="S11" s="7">
         <f>S10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N11,0)</f>
-        <v>-322</v>
+        <v>728</v>
       </c>
       <c r="T11" s="22">
         <f>IF(Demanda!N12=0,"",S11/(Demanda!N12/DiasVenta))</f>
-        <v>-1.511737089201878</v>
+        <v>3.4178403755868545</v>
       </c>
       <c r="U11" t="str">
         <f t="shared" si="9"/>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
     </row>
     <row r="12" spans="1:21">
@@ -30877,7 +30891,7 @@
       </c>
       <c r="C12" s="7">
         <f t="shared" si="10"/>
-        <v>3812</v>
+        <v>4862</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="1"/>
@@ -30893,15 +30907,15 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" si="3"/>
-        <v>-6124</v>
+        <v>-5074</v>
       </c>
       <c r="H12" s="7">
         <f ca="1">SUM($K$6:K11)*CajasProm</f>
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15876</v>
+        <v>15926</v>
       </c>
       <c r="J12" s="21">
         <f t="shared" si="5"/>
@@ -30913,11 +30927,11 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25876</v>
+        <v>25926</v>
       </c>
       <c r="M12" s="22">
         <f ca="1">IF(Demanda!H13=0,"",L12/(Demanda!H13/DiasVenta))</f>
-        <v>8.6253333333333337</v>
+        <v>8.6419999999999995</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30941,11 +30955,11 @@
       </c>
       <c r="S12" s="7">
         <f>S11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N12,0)</f>
-        <v>-1600</v>
+        <v>-550</v>
       </c>
       <c r="T12" s="22">
         <f>IF(Demanda!N13=0,"",S12/(Demanda!N13/DiasVenta))</f>
-        <v>-7.511737089201878</v>
+        <v>-2.5821596244131455</v>
       </c>
       <c r="U12" t="str">
         <f t="shared" si="9"/>
@@ -30963,7 +30977,7 @@
       </c>
       <c r="C13" s="7">
         <f t="shared" si="10"/>
-        <v>-6124</v>
+        <v>-5074</v>
       </c>
       <c r="D13" s="7">
         <f t="shared" si="1"/>
@@ -30979,15 +30993,15 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" si="3"/>
-        <v>-16060</v>
+        <v>-15010</v>
       </c>
       <c r="H13" s="7">
         <f ca="1">SUM($K$6:K12)*CajasProm</f>
-        <v>32000</v>
+        <v>31000</v>
       </c>
       <c r="I13" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15940</v>
+        <v>15990</v>
       </c>
       <c r="J13" s="21">
         <f t="shared" si="5"/>
@@ -30999,11 +31013,11 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25940</v>
+        <v>25990</v>
       </c>
       <c r="M13" s="22">
         <f ca="1">IF(Demanda!H14=0,"",L13/(Demanda!H14/DiasVenta))</f>
-        <v>8.6466666666666665</v>
+        <v>8.663333333333334</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31027,11 +31041,11 @@
       </c>
       <c r="S13" s="7">
         <f>S12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N13,0)</f>
-        <v>-2878</v>
+        <v>-1828</v>
       </c>
       <c r="T13" s="22">
         <f>IF(Demanda!N14=0,"",S13/(Demanda!N14/DiasVenta))</f>
-        <v>-13.511737089201878</v>
+        <v>-8.5821596244131459</v>
       </c>
       <c r="U13" t="str">
         <f t="shared" si="9"/>
@@ -31049,7 +31063,7 @@
       </c>
       <c r="C14" s="7">
         <f t="shared" si="10"/>
-        <v>-16060</v>
+        <v>-15010</v>
       </c>
       <c r="D14" s="7">
         <f t="shared" si="1"/>
@@ -31065,15 +31079,15 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" si="3"/>
-        <v>-25996</v>
+        <v>-24946</v>
       </c>
       <c r="H14" s="7">
         <f ca="1">SUM($K$6:K13)*CajasProm</f>
-        <v>42000</v>
+        <v>41000</v>
       </c>
       <c r="I14" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16004</v>
+        <v>16054</v>
       </c>
       <c r="J14" s="21">
         <f t="shared" si="5"/>
@@ -31085,11 +31099,11 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25004</v>
+        <v>25054</v>
       </c>
       <c r="M14" s="22">
         <f ca="1">IF(Demanda!H15=0,"",L14/(Demanda!H15/DiasVenta))</f>
-        <v>8.3346666666666671</v>
+        <v>8.3513333333333328</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31113,11 +31127,11 @@
       </c>
       <c r="S14" s="7">
         <f>S13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N14,0)</f>
-        <v>-4156</v>
+        <v>-3106</v>
       </c>
       <c r="T14" s="22">
         <f>IF(Demanda!N15=0,"",S14/(Demanda!N15/DiasVenta))</f>
-        <v>-19.511737089201876</v>
+        <v>-14.582159624413146</v>
       </c>
       <c r="U14" t="str">
         <f t="shared" si="9"/>
@@ -31135,7 +31149,7 @@
       </c>
       <c r="C15" s="7">
         <f t="shared" si="10"/>
-        <v>-25996</v>
+        <v>-24946</v>
       </c>
       <c r="D15" s="7">
         <f t="shared" si="1"/>
@@ -31151,15 +31165,15 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" si="3"/>
-        <v>-35932</v>
+        <v>-34882</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">SUM($K$6:K14)*CajasProm</f>
-        <v>51000</v>
+        <v>50000</v>
       </c>
       <c r="I15" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15068</v>
+        <v>15118</v>
       </c>
       <c r="J15" s="21">
         <f t="shared" si="5"/>
@@ -31171,11 +31185,11 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25068</v>
+        <v>25118</v>
       </c>
       <c r="M15" s="22">
         <f ca="1">IF(Demanda!H16=0,"",L15/(Demanda!H16/DiasVenta))</f>
-        <v>8.3559999999999999</v>
+        <v>8.3726666666666674</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31199,11 +31213,11 @@
       </c>
       <c r="S15" s="7">
         <f>S14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N15,0)</f>
-        <v>-5434</v>
+        <v>-4384</v>
       </c>
       <c r="T15" s="22">
         <f>IF(Demanda!N16=0,"",S15/(Demanda!N16/DiasVenta))</f>
-        <v>-25.511737089201876</v>
+        <v>-20.582159624413144</v>
       </c>
       <c r="U15" t="str">
         <f t="shared" si="9"/>
@@ -31221,7 +31235,7 @@
       </c>
       <c r="C16" s="7">
         <f t="shared" si="10"/>
-        <v>-35932</v>
+        <v>-34882</v>
       </c>
       <c r="D16" s="7">
         <f t="shared" si="1"/>
@@ -31237,15 +31251,15 @@
       </c>
       <c r="G16" s="7">
         <f t="shared" si="3"/>
-        <v>-45868</v>
+        <v>-44818</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">SUM($K$6:K15)*CajasProm</f>
-        <v>61000</v>
+        <v>60000</v>
       </c>
       <c r="I16" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15132</v>
+        <v>15182</v>
       </c>
       <c r="J16" s="21">
         <f t="shared" si="5"/>
@@ -31257,11 +31271,11 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25132</v>
+        <v>25182</v>
       </c>
       <c r="M16" s="22">
         <f ca="1">IF(Demanda!H17=0,"",L16/(Demanda!H17/DiasVenta))</f>
-        <v>8.3773333333333326</v>
+        <v>8.3940000000000001</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31285,11 +31299,11 @@
       </c>
       <c r="S16" s="7">
         <f>S15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N16,0)</f>
-        <v>-6712</v>
+        <v>-5662</v>
       </c>
       <c r="T16" s="22">
         <f>IF(Demanda!N17=0,"",S16/(Demanda!N17/DiasVenta))</f>
-        <v>-31.511737089201876</v>
+        <v>-26.582159624413144</v>
       </c>
       <c r="U16" t="str">
         <f t="shared" si="9"/>
@@ -31307,7 +31321,7 @@
       </c>
       <c r="C17" s="7">
         <f t="shared" si="10"/>
-        <v>-45868</v>
+        <v>-44818</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="1"/>
@@ -31323,15 +31337,15 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>-55804</v>
+        <v>-54754</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">SUM($K$6:K16)*CajasProm</f>
-        <v>71000</v>
+        <v>70000</v>
       </c>
       <c r="I17" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15196</v>
+        <v>15246</v>
       </c>
       <c r="J17" s="21">
         <f t="shared" si="5"/>
@@ -31343,11 +31357,11 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25196</v>
+        <v>25246</v>
       </c>
       <c r="M17" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L17/(Demanda!H18/DiasVenta))</f>
-        <v>8.3986666666666672</v>
+        <v>8.4153333333333329</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31371,11 +31385,11 @@
       </c>
       <c r="S17" s="7">
         <f>S16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N17,0)</f>
-        <v>-7990</v>
+        <v>-6940</v>
       </c>
       <c r="T17" s="22">
         <f>IF(Demanda!N18=0,"",S17/(Demanda!N18/DiasVenta))</f>
-        <v>-37.51173708920188</v>
+        <v>-32.582159624413144</v>
       </c>
       <c r="U17" t="str">
         <f t="shared" si="9"/>
@@ -31393,7 +31407,7 @@
       </c>
       <c r="C18" s="7">
         <f t="shared" si="10"/>
-        <v>-55804</v>
+        <v>-54754</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="1"/>
@@ -31409,15 +31423,15 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" si="3"/>
-        <v>-65740</v>
+        <v>-64690</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">SUM($K$6:K17)*CajasProm</f>
-        <v>81000</v>
+        <v>80000</v>
       </c>
       <c r="I18" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15260</v>
+        <v>15310</v>
       </c>
       <c r="J18" s="21">
         <f t="shared" si="5"/>
@@ -31429,11 +31443,11 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25260</v>
+        <v>25310</v>
       </c>
       <c r="M18" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L18/(Demanda!H18/DiasVenta))</f>
-        <v>8.42</v>
+        <v>8.4366666666666674</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31457,11 +31471,11 @@
       </c>
       <c r="S18" s="7">
         <f>S17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"BO")-ROUND(Demanda!N18,0)</f>
-        <v>-9268</v>
+        <v>-8218</v>
       </c>
       <c r="T18" s="22">
         <f>IF(Demanda!N18=0,"",S18/(Demanda!N18/DiasVenta))</f>
-        <v>-43.51173708920188</v>
+        <v>-38.582159624413144</v>
       </c>
       <c r="U18" t="str">
         <f t="shared" si="9"/>
@@ -31671,11 +31685,11 @@
       </c>
       <c r="B8" s="7">
         <f ca="1">IF(A8="","",Proyeccion!I8)</f>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="C8" s="3">
         <f ca="1">IF(A8="","",Proyeccion!K8)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="str">
         <f ca="1">IF(A8="","","BR "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B8-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B8-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31683,7 +31697,7 @@
       </c>
       <c r="E8" t="str">
         <f ca="1">IF(A8="","",IF(C8&gt;0,Proyeccion!U8,"-"))</f>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
       <c r="F8" t="str">
         <f ca="1">IF(A8="","","PY mie "&amp;TEXT(Proyeccion!A8-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A8-4,"dd/mm"))</f>
@@ -31691,15 +31705,15 @@
       </c>
       <c r="G8" s="22">
         <f ca="1">IF(A8="","",Proyeccion!M8)</f>
-        <v>8.5886666666666667</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="H8" t="str">
         <f ca="1">IF(A8="","",Proyeccion!N8)</f>
-        <v>CARGAR 2</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="I8" t="str">
         <f ca="1">IF(A8="","","Sab "&amp;TEXT(A8,"dd/mm")&amp;": "&amp;FIXED(B8,0)&amp;" cajas - descargan "&amp;Proyeccion!D8&amp;" - vende "&amp;FIXED(Proyeccion!F8,0)&amp;IF(C8&gt;0," -&gt; cargar "&amp;C8&amp;" mas hasta el "&amp;TEXT(Proyeccion!J8,"dd/mm")&amp;" ("&amp;E8&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 10/10: 23.766 cajas - descargan 19 - vende 18.000 -&gt; cargar 2 mas hasta el 06/10 (Bolivia; BR hasta el 07/10)</v>
+        <v>Sab 10/10: 24.816 cajas - descargan 20 - vende 18.000 -&gt; cargar 1 mas hasta el 06/10 (Brasil; BR hasta el 07/10)</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -31709,7 +31723,7 @@
       </c>
       <c r="B9" s="7">
         <f ca="1">IF(A9="","",Proyeccion!I9)</f>
-        <v>18684</v>
+        <v>18734</v>
       </c>
       <c r="C9" s="3">
         <f ca="1">IF(A9="","",Proyeccion!K9)</f>
@@ -31721,7 +31735,7 @@
       </c>
       <c r="E9" t="str">
         <f ca="1">IF(A9="","",IF(C9&gt;0,Proyeccion!U9,"-"))</f>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
       <c r="F9" t="str">
         <f ca="1">IF(A9="","","PY mie "&amp;TEXT(Proyeccion!A9-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A9-4,"dd/mm"))</f>
@@ -31729,7 +31743,7 @@
       </c>
       <c r="G9" s="22">
         <f ca="1">IF(A9="","",Proyeccion!M9)</f>
-        <v>8.5613333333333337</v>
+        <v>8.5779999999999994</v>
       </c>
       <c r="H9" t="str">
         <f ca="1">IF(A9="","",Proyeccion!N9)</f>
@@ -31737,7 +31751,7 @@
       </c>
       <c r="I9" t="str">
         <f ca="1">IF(A9="","","Sab "&amp;TEXT(A9,"dd/mm")&amp;": "&amp;FIXED(B9,0)&amp;" cajas - descargan "&amp;Proyeccion!D9&amp;" - vende "&amp;FIXED(Proyeccion!F9,0)&amp;IF(C9&gt;0," -&gt; cargar "&amp;C9&amp;" mas hasta el "&amp;TEXT(Proyeccion!J9,"dd/mm")&amp;" ("&amp;E9&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 17/10: 18.684 cajas - descargan 11 - vende 18.000 -&gt; cargar 7 mas hasta el 13/10 (Bolivia; BR hasta el 14/10)</v>
+        <v>Sab 17/10: 18.734 cajas - descargan 11 - vende 18.000 -&gt; cargar 7 mas hasta el 13/10 (Brasil; BR hasta el 14/10)</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -31747,7 +31761,7 @@
       </c>
       <c r="B10" s="7">
         <f ca="1">IF(A10="","",Proyeccion!I10)</f>
-        <v>21698</v>
+        <v>21748</v>
       </c>
       <c r="C10" s="3">
         <f ca="1">IF(A10="","",Proyeccion!K10)</f>
@@ -31759,7 +31773,7 @@
       </c>
       <c r="E10" t="str">
         <f ca="1">IF(A10="","",IF(C10&gt;0,Proyeccion!U10,"-"))</f>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
       <c r="F10" t="str">
         <f ca="1">IF(A10="","","PY mie "&amp;TEXT(Proyeccion!A10-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A10-4,"dd/mm"))</f>
@@ -31767,7 +31781,7 @@
       </c>
       <c r="G10" s="22">
         <f ca="1">IF(A10="","",Proyeccion!M10)</f>
-        <v>8.5660000000000007</v>
+        <v>8.5826666666666664</v>
       </c>
       <c r="H10" t="str">
         <f ca="1">IF(A10="","",Proyeccion!N10)</f>
@@ -31775,7 +31789,7 @@
       </c>
       <c r="I10" t="str">
         <f ca="1">IF(A10="","","Sab "&amp;TEXT(A10,"dd/mm")&amp;": "&amp;FIXED(B10,0)&amp;" cajas - descargan "&amp;Proyeccion!D10&amp;" - vende "&amp;FIXED(Proyeccion!F10,0)&amp;IF(C10&gt;0," -&gt; cargar "&amp;C10&amp;" mas hasta el "&amp;TEXT(Proyeccion!J10,"dd/mm")&amp;" ("&amp;E10&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B10-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 24/10: 21.698 cajas - descargan 14 - vende 18.000 -&gt; cargar 4 mas hasta el 20/10 (Bolivia; BR hasta el 21/10)</v>
+        <v>Sab 24/10: 21.748 cajas - descargan 14 - vende 18.000 -&gt; cargar 4 mas hasta el 20/10 (Brasil; BR hasta el 21/10)</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -31785,7 +31799,7 @@
       </c>
       <c r="B11" s="7">
         <f ca="1">IF(A11="","",Proyeccion!I11)</f>
-        <v>16812</v>
+        <v>16862</v>
       </c>
       <c r="C11" s="3">
         <f ca="1">IF(A11="","",Proyeccion!K11)</f>
@@ -31797,7 +31811,7 @@
       </c>
       <c r="E11" t="str">
         <f ca="1">IF(A11="","",IF(C11&gt;0,Proyeccion!U11,"-"))</f>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
       <c r="F11" t="str">
         <f ca="1">IF(A11="","","PY mie "&amp;TEXT(Proyeccion!A11-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A11-4,"dd/mm"))</f>
@@ -31805,7 +31819,7 @@
       </c>
       <c r="G11" s="22">
         <f ca="1">IF(A11="","",Proyeccion!M11)</f>
-        <v>8.6039999999999992</v>
+        <v>8.6206666666666667</v>
       </c>
       <c r="H11" t="str">
         <f ca="1">IF(A11="","",Proyeccion!N11)</f>
@@ -31813,7 +31827,7 @@
       </c>
       <c r="I11" t="str">
         <f ca="1">IF(A11="","","Sab "&amp;TEXT(A11,"dd/mm")&amp;": "&amp;FIXED(B11,0)&amp;" cajas - descargan "&amp;Proyeccion!D11&amp;" - vende "&amp;FIXED(Proyeccion!F11,0)&amp;IF(C11&gt;0," -&gt; cargar "&amp;C11&amp;" mas hasta el "&amp;TEXT(Proyeccion!J11,"dd/mm")&amp;" ("&amp;E11&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B11-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 31/10: 16.812 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 27/10 (Bolivia; BR hasta el 28/10)</v>
+        <v>Sab 31/10: 16.862 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 27/10 (Brasil; BR hasta el 28/10)</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -31823,7 +31837,7 @@
       </c>
       <c r="B12" s="7">
         <f ca="1">IF(A12="","",Proyeccion!I12)</f>
-        <v>15876</v>
+        <v>15926</v>
       </c>
       <c r="C12" s="3">
         <f ca="1">IF(A12="","",Proyeccion!K12)</f>
@@ -31843,7 +31857,7 @@
       </c>
       <c r="G12" s="22">
         <f ca="1">IF(A12="","",Proyeccion!M12)</f>
-        <v>8.6253333333333337</v>
+        <v>8.6419999999999995</v>
       </c>
       <c r="H12" t="str">
         <f ca="1">IF(A12="","",Proyeccion!N12)</f>
@@ -31851,7 +31865,7 @@
       </c>
       <c r="I12" t="str">
         <f ca="1">IF(A12="","","Sab "&amp;TEXT(A12,"dd/mm")&amp;": "&amp;FIXED(B12,0)&amp;" cajas - descargan "&amp;Proyeccion!D12&amp;" - vende "&amp;FIXED(Proyeccion!F12,0)&amp;IF(C12&gt;0," -&gt; cargar "&amp;C12&amp;" mas hasta el "&amp;TEXT(Proyeccion!J12,"dd/mm")&amp;" ("&amp;E12&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B12-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 07/11: 15.876 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
+        <v>Sab 07/11: 15.926 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -31861,7 +31875,7 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IF(A13="","",Proyeccion!I13)</f>
-        <v>15940</v>
+        <v>15990</v>
       </c>
       <c r="C13" s="3">
         <f ca="1">IF(A13="","",Proyeccion!K13)</f>
@@ -31881,7 +31895,7 @@
       </c>
       <c r="G13" s="22">
         <f ca="1">IF(A13="","",Proyeccion!M13)</f>
-        <v>8.6466666666666665</v>
+        <v>8.663333333333334</v>
       </c>
       <c r="H13" t="str">
         <f ca="1">IF(A13="","",Proyeccion!N13)</f>
@@ -31889,7 +31903,7 @@
       </c>
       <c r="I13" t="str">
         <f ca="1">IF(A13="","","Sab "&amp;TEXT(A13,"dd/mm")&amp;": "&amp;FIXED(B13,0)&amp;" cajas - descargan "&amp;Proyeccion!D13&amp;" - vende "&amp;FIXED(Proyeccion!F13,0)&amp;IF(C13&gt;0," -&gt; cargar "&amp;C13&amp;" mas hasta el "&amp;TEXT(Proyeccion!J13,"dd/mm")&amp;" ("&amp;E13&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 14/11: 15.940 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
+        <v>Sab 14/11: 15.990 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -31899,7 +31913,7 @@
       </c>
       <c r="B14" s="7">
         <f ca="1">IF(A14="","",Proyeccion!I14)</f>
-        <v>16004</v>
+        <v>16054</v>
       </c>
       <c r="C14" s="3">
         <f ca="1">IF(A14="","",Proyeccion!K14)</f>
@@ -31919,7 +31933,7 @@
       </c>
       <c r="G14" s="22">
         <f ca="1">IF(A14="","",Proyeccion!M14)</f>
-        <v>8.3346666666666671</v>
+        <v>8.3513333333333328</v>
       </c>
       <c r="H14" t="str">
         <f ca="1">IF(A14="","",Proyeccion!N14)</f>
@@ -31927,7 +31941,7 @@
       </c>
       <c r="I14" t="str">
         <f ca="1">IF(A14="","","Sab "&amp;TEXT(A14,"dd/mm")&amp;": "&amp;FIXED(B14,0)&amp;" cajas - descargan "&amp;Proyeccion!D14&amp;" - vende "&amp;FIXED(Proyeccion!F14,0)&amp;IF(C14&gt;0," -&gt; cargar "&amp;C14&amp;" mas hasta el "&amp;TEXT(Proyeccion!J14,"dd/mm")&amp;" ("&amp;E14&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 21/11: 16.004 cajas - descargan 8 - vende 18.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
+        <v>Sab 21/11: 16.054 cajas - descargan 8 - vende 18.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -31937,7 +31951,7 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(A15="","",Proyeccion!I15)</f>
-        <v>15068</v>
+        <v>15118</v>
       </c>
       <c r="C15" s="3">
         <f ca="1">IF(A15="","",Proyeccion!K15)</f>
@@ -31957,7 +31971,7 @@
       </c>
       <c r="G15" s="22">
         <f ca="1">IF(A15="","",Proyeccion!M15)</f>
-        <v>8.3559999999999999</v>
+        <v>8.3726666666666674</v>
       </c>
       <c r="H15" t="str">
         <f ca="1">IF(A15="","",Proyeccion!N15)</f>
@@ -31965,7 +31979,7 @@
       </c>
       <c r="I15" t="str">
         <f ca="1">IF(A15="","","Sab "&amp;TEXT(A15,"dd/mm")&amp;": "&amp;FIXED(B15,0)&amp;" cajas - descargan "&amp;Proyeccion!D15&amp;" - vende "&amp;FIXED(Proyeccion!F15,0)&amp;IF(C15&gt;0," -&gt; cargar "&amp;C15&amp;" mas hasta el "&amp;TEXT(Proyeccion!J15,"dd/mm")&amp;" ("&amp;E15&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B15-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 28/11: 15.068 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
+        <v>Sab 28/11: 15.118 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -31975,7 +31989,7 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(A16="","",Proyeccion!I16)</f>
-        <v>15132</v>
+        <v>15182</v>
       </c>
       <c r="C16" s="3">
         <f ca="1">IF(A16="","",Proyeccion!K16)</f>
@@ -31995,7 +32009,7 @@
       </c>
       <c r="G16" s="22">
         <f ca="1">IF(A16="","",Proyeccion!M16)</f>
-        <v>8.3773333333333326</v>
+        <v>8.3940000000000001</v>
       </c>
       <c r="H16" t="str">
         <f ca="1">IF(A16="","",Proyeccion!N16)</f>
@@ -32003,7 +32017,7 @@
       </c>
       <c r="I16" t="str">
         <f ca="1">IF(A16="","","Sab "&amp;TEXT(A16,"dd/mm")&amp;": "&amp;FIXED(B16,0)&amp;" cajas - descargan "&amp;Proyeccion!D16&amp;" - vende "&amp;FIXED(Proyeccion!F16,0)&amp;IF(C16&gt;0," -&gt; cargar "&amp;C16&amp;" mas hasta el "&amp;TEXT(Proyeccion!J16,"dd/mm")&amp;" ("&amp;E16&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B16-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 05/12: 15.132 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
+        <v>Sab 05/12: 15.182 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -32013,7 +32027,7 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(A17="","",Proyeccion!I17)</f>
-        <v>15196</v>
+        <v>15246</v>
       </c>
       <c r="C17" s="3">
         <f ca="1">IF(A17="","",Proyeccion!K17)</f>
@@ -32033,7 +32047,7 @@
       </c>
       <c r="G17" s="22">
         <f ca="1">IF(A17="","",Proyeccion!M17)</f>
-        <v>8.3986666666666672</v>
+        <v>8.4153333333333329</v>
       </c>
       <c r="H17" t="str">
         <f ca="1">IF(A17="","",Proyeccion!N17)</f>
@@ -32041,7 +32055,7 @@
       </c>
       <c r="I17" t="str">
         <f ca="1">IF(A17="","","Sab "&amp;TEXT(A17,"dd/mm")&amp;": "&amp;FIXED(B17,0)&amp;" cajas - descargan "&amp;Proyeccion!D17&amp;" - vende "&amp;FIXED(Proyeccion!F17,0)&amp;IF(C17&gt;0," -&gt; cargar "&amp;C17&amp;" mas hasta el "&amp;TEXT(Proyeccion!J17,"dd/mm")&amp;" ("&amp;E17&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B17-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 12/12: 15.196 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
+        <v>Sab 12/12: 15.246 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -32051,7 +32065,7 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(A18="","",Proyeccion!I18)</f>
-        <v>15260</v>
+        <v>15310</v>
       </c>
       <c r="C18" s="3">
         <f ca="1">IF(A18="","",Proyeccion!K18)</f>
@@ -32071,7 +32085,7 @@
       </c>
       <c r="G18" s="22">
         <f ca="1">IF(A18="","",Proyeccion!M18)</f>
-        <v>8.42</v>
+        <v>8.4366666666666674</v>
       </c>
       <c r="H18" t="str">
         <f ca="1">IF(A18="","",Proyeccion!N18)</f>
@@ -32079,7 +32093,7 @@
       </c>
       <c r="I18" t="str">
         <f ca="1">IF(A18="","","Sab "&amp;TEXT(A18,"dd/mm")&amp;": "&amp;FIXED(B18,0)&amp;" cajas - descargan "&amp;Proyeccion!D18&amp;" - vende "&amp;FIXED(Proyeccion!F18,0)&amp;IF(C18&gt;0," -&gt; cargar "&amp;C18&amp;" mas hasta el "&amp;TEXT(Proyeccion!J18,"dd/mm")&amp;" ("&amp;E18&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B18-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 19/12: 15.260 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
+        <v>Sab 19/12: 15.310 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="33.950000000000003" customHeight="1">
@@ -32346,19 +32360,19 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IFERROR(INDEX(PrBO,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>362</v>
+        <v>1412</v>
       </c>
       <c r="C15" s="22">
         <f ca="1">IFERROR(INDEX(PrBOd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>1.699530516431925</v>
+        <v>6.629107981220657</v>
       </c>
       <c r="D15" t="str">
         <f ca="1">IF(B15="","",IF(B15&lt;0,"FALTA",IF(C15&lt;2,"CRITICO",IF(C15&lt;CoberturaObjetivo,"JUSTO",IF(C15&gt;VidaVerde,"EXCESO","OK")))))</f>
-        <v>CRITICO</v>
+        <v>JUSTO</v>
       </c>
       <c r="E15" t="str">
         <f ca="1">IF(D15="FALTA","se queda sin fruta: cargar ya",IF(D15="CRITICO","cargar esta semana, sin falta",IF(D15="JUSTO","priorizar este origen en los pedidos",IF(D15="EXCESO","frenar cargas: riesgo de merma",""))))</f>
-        <v>cargar esta semana, sin falta</v>
+        <v>priorizar este origen en los pedidos</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -32367,19 +32381,19 @@
       </c>
       <c r="B16" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="C16" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>8.5886666666666667</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="D16" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>CARGAR 2</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="E16" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 2 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
+        <v>cargar 1 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -32457,19 +32471,19 @@
       </c>
       <c r="B22" s="7">
         <f ca="1">IFERROR(INDEX(PrBO,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>134</v>
+        <v>1184</v>
       </c>
       <c r="C22" s="22">
         <f ca="1">IFERROR(INDEX(PrBOd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>0.62910798122065725</v>
+        <v>5.55868544600939</v>
       </c>
       <c r="D22" t="str">
         <f ca="1">IF(B22="","",IF(B22&lt;0,"FALTA",IF(C22&lt;2,"CRITICO",IF(C22&lt;CoberturaObjetivo,"JUSTO",IF(C22&gt;VidaVerde,"EXCESO","OK")))))</f>
-        <v>CRITICO</v>
+        <v>JUSTO</v>
       </c>
       <c r="E22" t="str">
         <f ca="1">IF(D22="FALTA","se queda sin fruta: cargar ya",IF(D22="CRITICO","cargar esta semana, sin falta",IF(D22="JUSTO","priorizar este origen en los pedidos",IF(D22="EXCESO","frenar cargas: riesgo de merma",""))))</f>
-        <v>cargar esta semana, sin falta</v>
+        <v>priorizar este origen en los pedidos</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -32478,11 +32492,11 @@
       </c>
       <c r="B23" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>18684</v>
+        <v>18734</v>
       </c>
       <c r="C23" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>8.5613333333333337</v>
+        <v>8.5779999999999994</v>
       </c>
       <c r="D23" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
@@ -32505,7 +32519,7 @@
     <row r="26" spans="1:5">
       <c r="A26" s="45" t="str">
         <f ca="1">IF(COUNTIFS(CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1))=0,"Bolivia: no hay ningun camion en camino ni dictado. Tarda 6 dias: para que entre el sabado que viene tiene que cargar antes del "&amp;TEXT(FechaHoy-WEEKDAY(FechaHoy,2)+1+12-LagBO,"ddd dd/mm"),"Bolivia: "&amp;COUNTIFS(CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1))&amp;" camion(es) en el plan")</f>
-        <v>Bolivia: 4 camion(es) en el plan</v>
+        <v>Bolivia: 5 camion(es) en el plan</v>
       </c>
       <c r="B26" s="46"/>
       <c r="C26" s="46"/>
@@ -32515,7 +32529,7 @@
     <row r="27" spans="1:5">
       <c r="A27" s="45" t="str">
         <f ca="1">"Paraguay: "&amp;COUNTIFS(CgEstado,"Supuesto",CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+14))&amp;" camiones SUPUESTOS en las proximas 2 semanas (todavia no dictados). El plan es firme cuando se dictan."</f>
-        <v>Paraguay: 0 camiones SUPUESTOS en las proximas 2 semanas (todavia no dictados). El plan es firme cuando se dictan.</v>
+        <v>Paraguay: 1 camiones SUPUESTOS en las proximas 2 semanas (todavia no dictados). El plan es firme cuando se dictan.</v>
       </c>
       <c r="B27" s="46"/>
       <c r="C27" s="46"/>
@@ -32545,7 +32559,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 15.830 (plan: 23.766).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.880 (plan: 24.816).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32862,7 +32876,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>18868</v>
+        <v>19918</v>
       </c>
       <c r="D8" s="7">
         <f>Proyeccion!F8</f>
@@ -32870,7 +32884,7 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>27166</v>
+        <v>28216</v>
       </c>
       <c r="F8">
         <f ca="1">IF(AND(E8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-E8)/CajasProm,0),0)</f>
@@ -32878,39 +32892,39 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>23766</v>
+        <v>24816</v>
       </c>
       <c r="H8">
         <f ca="1">IF(AND(G8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-G8)/CajasProm,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>20366</v>
+        <v>21416</v>
       </c>
       <c r="J8">
         <f ca="1">IF(AND(I8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-I8)/CajasProm,0),0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
-        <v>15944</v>
+        <v>16994</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15830</v>
+        <v>16880</v>
       </c>
       <c r="M8">
         <f ca="1">IF(AND(L8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-L8)/CajasProm,0),0)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>20826</v>
+        <v>21876</v>
       </c>
       <c r="O8" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>22766</v>
+        <v>23816</v>
       </c>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="3"/>
@@ -32936,15 +32950,15 @@
       </c>
       <c r="E9" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>21884</v>
+        <v>22934</v>
       </c>
       <c r="F9">
         <f ca="1">IF(AND(E9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-E9)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>18684</v>
+        <v>18734</v>
       </c>
       <c r="H9">
         <f ca="1">IF(AND(G9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-G9)/CajasProm,0),0)</f>
@@ -32952,7 +32966,7 @@
       </c>
       <c r="I9" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>16484</v>
+        <v>16534</v>
       </c>
       <c r="J9">
         <f ca="1">IF(AND(I9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-I9)/CajasProm,0),0)</f>
@@ -32964,7 +32978,7 @@
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>26684</v>
+        <v>26734</v>
       </c>
       <c r="M9">
         <f ca="1">IF(AND(L9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-L9)/CajasProm,0),0)</f>
@@ -32972,15 +32986,15 @@
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>15744</v>
+        <v>15794</v>
       </c>
       <c r="O9" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>17684</v>
+        <v>17734</v>
       </c>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>17634</v>
+        <v>16634</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -33002,7 +33016,7 @@
       </c>
       <c r="E10" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>23698</v>
+        <v>23748</v>
       </c>
       <c r="F10">
         <f ca="1">IF(AND(E10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-E10)/CajasProm,0),0)</f>
@@ -33010,7 +33024,7 @@
       </c>
       <c r="G10" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>21698</v>
+        <v>21748</v>
       </c>
       <c r="H10">
         <f ca="1">IF(AND(G10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-G10)/CajasProm,0),0)</f>
@@ -33018,7 +33032,7 @@
       </c>
       <c r="I10" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>19698</v>
+        <v>19748</v>
       </c>
       <c r="J10">
         <f ca="1">IF(AND(I10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-I10)/CajasProm,0),0)</f>
@@ -33030,7 +33044,7 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22698</v>
+        <v>22748</v>
       </c>
       <c r="M10">
         <f ca="1">IF(AND(L10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-L10)/CajasProm,0),0)</f>
@@ -33038,15 +33052,15 @@
       </c>
       <c r="N10" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>18758</v>
+        <v>18808</v>
       </c>
       <c r="O10" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>20698</v>
+        <v>20748</v>
       </c>
       <c r="P10" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>20648</v>
+        <v>19648</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -33068,7 +33082,7 @@
       </c>
       <c r="E11" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18612</v>
+        <v>18662</v>
       </c>
       <c r="F11">
         <f ca="1">IF(AND(E11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-E11)/CajasProm,0),0)</f>
@@ -33076,7 +33090,7 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16812</v>
+        <v>16862</v>
       </c>
       <c r="H11">
         <f ca="1">IF(AND(G11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-G11)/CajasProm,0),0)</f>
@@ -33084,7 +33098,7 @@
       </c>
       <c r="I11" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>15012</v>
+        <v>15062</v>
       </c>
       <c r="J11">
         <f ca="1">IF(AND(I11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-I11)/CajasProm,0),0)</f>
@@ -33096,7 +33110,7 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16812</v>
+        <v>16862</v>
       </c>
       <c r="M11">
         <f ca="1">IF(AND(L11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-L11)/CajasProm,0),0)</f>
@@ -33104,15 +33118,15 @@
       </c>
       <c r="N11" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13872</v>
+        <v>13922</v>
       </c>
       <c r="O11" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15812</v>
+        <v>15862</v>
       </c>
       <c r="P11" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>15762</v>
+        <v>14762</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -33134,7 +33148,7 @@
       </c>
       <c r="E12" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17476</v>
+        <v>17526</v>
       </c>
       <c r="F12">
         <f ca="1">IF(AND(E12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-E12)/CajasProm,0),0)</f>
@@ -33142,7 +33156,7 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15876</v>
+        <v>15926</v>
       </c>
       <c r="H12">
         <f ca="1">IF(AND(G12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-G12)/CajasProm,0),0)</f>
@@ -33150,7 +33164,7 @@
       </c>
       <c r="I12" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13276</v>
+        <v>13326</v>
       </c>
       <c r="J12">
         <f ca="1">IF(AND(I12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-I12)/CajasProm,0),0)</f>
@@ -33162,7 +33176,7 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15876</v>
+        <v>15926</v>
       </c>
       <c r="M12">
         <f ca="1">IF(AND(L12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-L12)/CajasProm,0),0)</f>
@@ -33170,15 +33184,15 @@
       </c>
       <c r="N12" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12936</v>
+        <v>12986</v>
       </c>
       <c r="O12" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14876</v>
+        <v>14926</v>
       </c>
       <c r="P12" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14826</v>
+        <v>13826</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -33200,7 +33214,7 @@
       </c>
       <c r="E13" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17340</v>
+        <v>17390</v>
       </c>
       <c r="F13">
         <f ca="1">IF(AND(E13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-E13)/CajasProm,0),0)</f>
@@ -33208,7 +33222,7 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15940</v>
+        <v>15990</v>
       </c>
       <c r="H13">
         <f ca="1">IF(AND(G13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-G13)/CajasProm,0),0)</f>
@@ -33216,7 +33230,7 @@
       </c>
       <c r="I13" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13540</v>
+        <v>13590</v>
       </c>
       <c r="J13">
         <f ca="1">IF(AND(I13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-I13)/CajasProm,0),0)</f>
@@ -33228,7 +33242,7 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15940</v>
+        <v>15990</v>
       </c>
       <c r="M13">
         <f ca="1">IF(AND(L13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-L13)/CajasProm,0),0)</f>
@@ -33236,15 +33250,15 @@
       </c>
       <c r="N13" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13000</v>
+        <v>13050</v>
       </c>
       <c r="O13" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14940</v>
+        <v>14990</v>
       </c>
       <c r="P13" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14890</v>
+        <v>13890</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -33266,7 +33280,7 @@
       </c>
       <c r="E14" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17204</v>
+        <v>17254</v>
       </c>
       <c r="F14">
         <f ca="1">IF(AND(E14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-E14)/CajasProm,0),0)</f>
@@ -33274,7 +33288,7 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16004</v>
+        <v>16054</v>
       </c>
       <c r="H14">
         <f ca="1">IF(AND(G14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-G14)/CajasProm,0),0)</f>
@@ -33282,7 +33296,7 @@
       </c>
       <c r="I14" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13804</v>
+        <v>13854</v>
       </c>
       <c r="J14">
         <f ca="1">IF(AND(I14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-I14)/CajasProm,0),0)</f>
@@ -33294,7 +33308,7 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16004</v>
+        <v>16054</v>
       </c>
       <c r="M14">
         <f ca="1">IF(AND(L14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-L14)/CajasProm,0),0)</f>
@@ -33302,15 +33316,15 @@
       </c>
       <c r="N14" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13064</v>
+        <v>13114</v>
       </c>
       <c r="O14" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15004</v>
+        <v>15054</v>
       </c>
       <c r="P14" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14954</v>
+        <v>13954</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -33332,7 +33346,7 @@
       </c>
       <c r="E15" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17068</v>
+        <v>17118</v>
       </c>
       <c r="F15">
         <f ca="1">IF(AND(E15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-E15)/CajasProm,0),0)</f>
@@ -33340,7 +33354,7 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15068</v>
+        <v>15118</v>
       </c>
       <c r="H15">
         <f ca="1">IF(AND(G15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-G15)/CajasProm,0),0)</f>
@@ -33348,7 +33362,7 @@
       </c>
       <c r="I15" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14068</v>
+        <v>14118</v>
       </c>
       <c r="J15">
         <f ca="1">IF(AND(I15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-I15)/CajasProm,0),0)</f>
@@ -33360,7 +33374,7 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15068</v>
+        <v>15118</v>
       </c>
       <c r="M15">
         <f ca="1">IF(AND(L15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-L15)/CajasProm,0),0)</f>
@@ -33368,15 +33382,15 @@
       </c>
       <c r="N15" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12128</v>
+        <v>12178</v>
       </c>
       <c r="O15" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14068</v>
+        <v>14118</v>
       </c>
       <c r="P15" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14018</v>
+        <v>13018</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -33398,7 +33412,7 @@
       </c>
       <c r="E16" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>16932</v>
+        <v>16982</v>
       </c>
       <c r="F16">
         <f ca="1">IF(AND(E16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-E16)/CajasProm,0),0)</f>
@@ -33406,7 +33420,7 @@
       </c>
       <c r="G16" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15132</v>
+        <v>15182</v>
       </c>
       <c r="H16">
         <f ca="1">IF(AND(G16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-G16)/CajasProm,0),0)</f>
@@ -33414,7 +33428,7 @@
       </c>
       <c r="I16" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13332</v>
+        <v>13382</v>
       </c>
       <c r="J16">
         <f ca="1">IF(AND(I16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-I16)/CajasProm,0),0)</f>
@@ -33426,7 +33440,7 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15132</v>
+        <v>15182</v>
       </c>
       <c r="M16">
         <f ca="1">IF(AND(L16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-L16)/CajasProm,0),0)</f>
@@ -33434,15 +33448,15 @@
       </c>
       <c r="N16" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12192</v>
+        <v>12242</v>
       </c>
       <c r="O16" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14132</v>
+        <v>14182</v>
       </c>
       <c r="P16" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14082</v>
+        <v>13082</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -33464,7 +33478,7 @@
       </c>
       <c r="E17" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17796</v>
+        <v>17846</v>
       </c>
       <c r="F17">
         <f ca="1">IF(AND(E17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-E17)/CajasProm,0),0)</f>
@@ -33472,7 +33486,7 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15196</v>
+        <v>15246</v>
       </c>
       <c r="H17">
         <f ca="1">IF(AND(G17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-G17)/CajasProm,0),0)</f>
@@ -33480,7 +33494,7 @@
       </c>
       <c r="I17" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13596</v>
+        <v>13646</v>
       </c>
       <c r="J17">
         <f ca="1">IF(AND(I17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-I17)/CajasProm,0),0)</f>
@@ -33492,7 +33506,7 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15196</v>
+        <v>15246</v>
       </c>
       <c r="M17">
         <f ca="1">IF(AND(L17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-L17)/CajasProm,0),0)</f>
@@ -33500,15 +33514,15 @@
       </c>
       <c r="N17" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12256</v>
+        <v>12306</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14196</v>
+        <v>14246</v>
       </c>
       <c r="P17" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14146</v>
+        <v>13146</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -33530,7 +33544,7 @@
       </c>
       <c r="E18" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17660</v>
+        <v>17710</v>
       </c>
       <c r="F18">
         <f ca="1">IF(AND(E18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-E18)/CajasProm,0),0)</f>
@@ -33538,7 +33552,7 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15260</v>
+        <v>15310</v>
       </c>
       <c r="H18">
         <f ca="1">IF(AND(G18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-G18)/CajasProm,0),0)</f>
@@ -33546,7 +33560,7 @@
       </c>
       <c r="I18" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13860</v>
+        <v>13910</v>
       </c>
       <c r="J18">
         <f ca="1">IF(AND(I18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-I18)/CajasProm,0),0)</f>
@@ -33558,7 +33572,7 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15260</v>
+        <v>15310</v>
       </c>
       <c r="M18">
         <f ca="1">IF(AND(L18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-L18)/CajasProm,0),0)</f>
@@ -33566,15 +33580,15 @@
       </c>
       <c r="N18" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12320</v>
+        <v>12370</v>
       </c>
       <c r="O18" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14260</v>
+        <v>14310</v>
       </c>
       <c r="P18" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14210</v>
+        <v>13210</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="63.95" customHeight="1">

</xml_diff>

<commit_message>
plan de compras: semana 05-10/10 v3 (Cassio solo mie, Gilson mie)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935BD00B-2EF7-4EC9-9B16-04B00CF42E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F346E5D6-36FE-4E2A-ABFB-9222F388B35D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,12 +110,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="681">
   <si>
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 01/10/2026 12:52 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 01/10/2026 18:41 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -814,10 +814,10 @@
     <t>nota 01/10: cuarta (antes martes, sacada el 30/09); transportista supuesto</t>
   </si>
   <si>
+    <t>nota 01/10 (v3): cuarta (antes sexta); transportista supuesto = semana anterior</t>
+  </si>
+  <si>
     <t>nota 30/09: sexta; transportista supuesto = semana anterior</t>
-  </si>
-  <si>
-    <t>nota 30/09: sabado (descarga martes 13, suma a la semana siguiente); transportista supuesto = semana anterior</t>
   </si>
   <si>
     <t>Paraguay (supuesto)</t>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>19918</v>
+        <v>20926</v>
       </c>
       <c r="D8" s="7">
         <f>Demanda!H9</f>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="H8" s="7">
         <f ca="1">Proyeccion!L8</f>
-        <v>25816</v>
+        <v>25824</v>
       </c>
       <c r="I8" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="C9" s="7">
         <f>Proyeccion!E9</f>
-        <v>10918</v>
+        <v>8974</v>
       </c>
       <c r="D9" s="7">
         <f>Demanda!H10</f>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="H9" s="7">
         <f ca="1">Proyeccion!L9</f>
-        <v>25734</v>
+        <v>25798</v>
       </c>
       <c r="I9" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H10" s="7">
         <f ca="1">Proyeccion!L10</f>
-        <v>25748</v>
+        <v>25812</v>
       </c>
       <c r="I10" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="H11" s="7">
         <f ca="1">Proyeccion!L11</f>
-        <v>25862</v>
+        <v>25926</v>
       </c>
       <c r="I11" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="H12" s="7">
         <f ca="1">Proyeccion!L12</f>
-        <v>25926</v>
+        <v>25990</v>
       </c>
       <c r="I12" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4306,7 +4306,7 @@
       </c>
       <c r="H13" s="7">
         <f ca="1">Proyeccion!L13</f>
-        <v>25990</v>
+        <v>25054</v>
       </c>
       <c r="I13" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="H14" s="7">
         <f ca="1">Proyeccion!L14</f>
-        <v>25054</v>
+        <v>25118</v>
       </c>
       <c r="I14" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="H15" s="7">
         <f ca="1">Proyeccion!L15</f>
-        <v>25118</v>
+        <v>25182</v>
       </c>
       <c r="I15" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="H16" s="7">
         <f ca="1">Proyeccion!L16</f>
-        <v>25182</v>
+        <v>25246</v>
       </c>
       <c r="I16" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="H17" s="7">
         <f ca="1">Proyeccion!L17</f>
-        <v>25246</v>
+        <v>25310</v>
       </c>
       <c r="I17" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="H18" s="7">
         <f ca="1">Proyeccion!L18</f>
-        <v>25310</v>
+        <v>25374</v>
       </c>
       <c r="I18" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B9" s="25">
         <f ca="1">IFERROR(INDEX(PrACargar,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>303</v>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B10" s="24">
         <f ca="1">AVERAGEIFS(PrCobertura,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8.3496666666666659</v>
+        <v>8.3610000000000007</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>305</v>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B11" s="25">
         <f ca="1">COUNTIFS(PrACargar,"&gt;0",PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>307</v>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="B12" s="25">
         <f ca="1">SUMIFS(PrACargar,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>309</v>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="B19" s="24">
         <f ca="1">AVERAGEIFS(PrCamiones,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>14.25</v>
+        <v>14</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>322</v>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="B20" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BR",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.58080879244751304</v>
+        <v>0.57378223495702008</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>324</v>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="B21" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"PY",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>0.34521628857263631</v>
+        <v>0.35100286532951291</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>3</v>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B22" s="27">
         <f ca="1">IFERROR(SUMIFS(CgCajas,CgOrigen,"BO",CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))/SUMIFS(CgCajas,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28)),0)</f>
-        <v>7.3974918979850646E-2</v>
+        <v>7.5214899713467051E-2</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>3</v>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B23" s="12">
         <f ca="1">SUMIFS(CgCosto,CgCuenta,1,CgSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),CgSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>416359.83999999973</v>
+        <v>409723.59999999974</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>328</v>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="B27" s="25">
         <f>COUNTIFS(CgEstado,"Dictado",CgCuenta,1)</f>
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>336</v>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="O10">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" t="s">
         <v>3</v>
@@ -12513,10 +12513,10 @@
         <v>58</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="G37" s="8">
         <v>1008</v>
@@ -12554,7 +12554,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q37" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="R37" s="5">
         <f t="shared" si="9"/>
@@ -12579,20 +12579,20 @@
         <v>34</v>
       </c>
       <c r="B38" s="6">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>mié</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="G38" s="8">
         <v>1008</v>
@@ -12611,11 +12611,11 @@
       </c>
       <c r="L38" s="5">
         <f t="shared" si="4"/>
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="M38" s="5">
         <f t="shared" si="5"/>
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="N38">
         <f t="shared" si="6"/>
@@ -12630,11 +12630,11 @@
         <v>7146.72</v>
       </c>
       <c r="Q38" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="R38" s="5">
         <f t="shared" si="9"/>
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="S38" s="5">
         <f t="shared" si="10"/>
@@ -12665,10 +12665,10 @@
         <v>58</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G39" s="8">
         <v>1008</v>
@@ -12706,7 +12706,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q39" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R39" s="5">
         <f t="shared" si="9"/>
@@ -12782,7 +12782,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q40" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R40" s="5">
         <f t="shared" si="9"/>
@@ -12858,7 +12858,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R41" s="5">
         <f t="shared" si="9"/>
@@ -12883,39 +12883,39 @@
         <v>38</v>
       </c>
       <c r="B42" s="6">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="1"/>
-        <v>sáb</v>
+        <v>lun</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>221</v>
+        <v>3</v>
       </c>
       <c r="G42" s="8">
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="H42" s="7">
         <f t="shared" si="2"/>
-        <v>936</v>
+        <v>980</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="J42" s="6"/>
       <c r="K42">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L42" s="5">
         <f t="shared" si="4"/>
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="M42" s="5">
         <f t="shared" si="5"/>
@@ -12927,18 +12927,18 @@
       </c>
       <c r="O42" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P42" s="7">
         <f t="shared" si="8"/>
-        <v>6636.24</v>
+        <v>6860</v>
       </c>
       <c r="Q42" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="R42" s="5">
         <f t="shared" si="9"/>
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="S42" s="5">
         <f t="shared" si="10"/>
@@ -13263,27 +13263,27 @@
         <v>43</v>
       </c>
       <c r="B47" s="6">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>mar</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G47" s="8">
-        <v>980</v>
+        <v>1050</v>
       </c>
       <c r="H47" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1050</v>
       </c>
       <c r="I47" s="9" t="s">
         <v>206</v>
@@ -13291,15 +13291,15 @@
       <c r="J47" s="6"/>
       <c r="K47">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L47" s="5">
         <f t="shared" si="4"/>
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="M47" s="5">
         <f t="shared" si="5"/>
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="N47">
         <f t="shared" si="6"/>
@@ -13307,22 +13307,22 @@
       </c>
       <c r="O47" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>10.8</v>
       </c>
       <c r="P47" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>11340</v>
       </c>
       <c r="Q47" s="9" t="s">
-        <v>237</v>
+        <v>207</v>
       </c>
       <c r="R47" s="5">
         <f t="shared" si="9"/>
-        <v>46312</v>
+        <v>46316</v>
       </c>
       <c r="S47" s="5">
         <f t="shared" si="10"/>
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="T47" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -13339,35 +13339,35 @@
         <v>44</v>
       </c>
       <c r="B48" s="6">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>vie</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>205</v>
+        <v>238</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G48" s="8">
-        <v>1050</v>
+        <v>1008</v>
       </c>
       <c r="H48" s="7">
         <f t="shared" si="2"/>
-        <v>1050</v>
+        <v>1008</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>206</v>
+        <v>239</v>
       </c>
       <c r="J48" s="6"/>
       <c r="K48">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L48" s="5">
         <f t="shared" si="4"/>
@@ -13383,18 +13383,18 @@
       </c>
       <c r="O48" s="10">
         <f t="shared" si="7"/>
-        <v>10.8</v>
+        <v>7.09</v>
       </c>
       <c r="P48" s="7">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>7146.72</v>
       </c>
       <c r="Q48" s="9" t="s">
-        <v>207</v>
+        <v>240</v>
       </c>
       <c r="R48" s="5">
         <f t="shared" si="9"/>
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="S48" s="5">
         <f t="shared" si="10"/>
@@ -13947,39 +13947,39 @@
         <v>52</v>
       </c>
       <c r="B56" s="6">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="1"/>
-        <v>vie</v>
+        <v>lun</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G56" s="8">
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="H56" s="7">
         <f t="shared" si="2"/>
-        <v>1008</v>
+        <v>980</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="J56" s="6"/>
       <c r="K56">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L56" s="5">
         <f t="shared" si="4"/>
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="M56" s="5">
         <f t="shared" si="5"/>
@@ -13991,18 +13991,18 @@
       </c>
       <c r="O56" s="10">
         <f t="shared" si="7"/>
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="P56" s="7">
         <f t="shared" si="8"/>
-        <v>7146.72</v>
+        <v>6860</v>
       </c>
       <c r="Q56" s="9" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="R56" s="5">
         <f t="shared" si="9"/>
-        <v>46317</v>
+        <v>46319</v>
       </c>
       <c r="S56" s="5">
         <f t="shared" si="10"/>
@@ -14327,27 +14327,27 @@
         <v>57</v>
       </c>
       <c r="B61" s="6">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="1"/>
-        <v>lun</v>
+        <v>mar</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G61" s="8">
-        <v>980</v>
+        <v>1050</v>
       </c>
       <c r="H61" s="7">
         <f t="shared" si="2"/>
-        <v>980</v>
+        <v>1050</v>
       </c>
       <c r="I61" s="9" t="s">
         <v>206</v>
@@ -14355,15 +14355,15 @@
       <c r="J61" s="6"/>
       <c r="K61">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L61" s="5">
         <f t="shared" si="4"/>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="M61" s="5">
         <f t="shared" si="5"/>
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="N61">
         <f t="shared" si="6"/>
@@ -14371,22 +14371,22 @@
       </c>
       <c r="O61" s="10">
         <f t="shared" si="7"/>
-        <v>7</v>
+        <v>10.8</v>
       </c>
       <c r="P61" s="7">
         <f t="shared" si="8"/>
-        <v>6860</v>
+        <v>11340</v>
       </c>
       <c r="Q61" s="9" t="s">
-        <v>237</v>
+        <v>207</v>
       </c>
       <c r="R61" s="5">
         <f t="shared" si="9"/>
-        <v>46319</v>
+        <v>46323</v>
       </c>
       <c r="S61" s="5">
         <f t="shared" si="10"/>
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="T61" s="7">
         <f t="shared" ca="1" si="11"/>
@@ -14403,35 +14403,35 @@
         <v>58</v>
       </c>
       <c r="B62" s="6">
-        <v>46315</v>
+        <v>46318</v>
       </c>
       <c r="C62" t="str">
         <f t="shared" si="1"/>
-        <v>mar</v>
+        <v>vie</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>205</v>
+        <v>238</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G62" s="8">
-        <v>1050</v>
+        <v>1008</v>
       </c>
       <c r="H62" s="7">
         <f t="shared" si="2"/>
-        <v>1050</v>
+        <v>1008</v>
       </c>
       <c r="I62" s="9" t="s">
-        <v>206</v>
+        <v>239</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L62" s="5">
         <f t="shared" si="4"/>
@@ -14447,18 +14447,18 @@
       </c>
       <c r="O62" s="10">
         <f t="shared" si="7"/>
-        <v>10.8</v>
+        <v>7.09</v>
       </c>
       <c r="P62" s="7">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>7146.72</v>
       </c>
       <c r="Q62" s="9" t="s">
-        <v>207</v>
+        <v>240</v>
       </c>
       <c r="R62" s="5">
         <f t="shared" si="9"/>
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="S62" s="5">
         <f t="shared" si="10"/>
@@ -15011,7 +15011,7 @@
         <v>66</v>
       </c>
       <c r="B70" s="6">
-        <v>46318</v>
+        <v>46325</v>
       </c>
       <c r="C70" t="str">
         <f t="shared" si="14"/>
@@ -15043,11 +15043,11 @@
       </c>
       <c r="L70" s="5">
         <f t="shared" si="17"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="M70" s="5">
         <f t="shared" si="18"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="N70">
         <f t="shared" si="19"/>
@@ -15066,11 +15066,11 @@
       </c>
       <c r="R70" s="5">
         <f t="shared" si="22"/>
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="S70" s="5">
         <f t="shared" si="23"/>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="T70" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -15619,7 +15619,7 @@
         <v>74</v>
       </c>
       <c r="B78" s="6">
-        <v>46325</v>
+        <v>46332</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="14"/>
@@ -15651,11 +15651,11 @@
       </c>
       <c r="L78" s="5">
         <f t="shared" si="17"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="M78" s="5">
         <f t="shared" si="18"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="N78">
         <f t="shared" si="19"/>
@@ -15674,11 +15674,11 @@
       </c>
       <c r="R78" s="5">
         <f t="shared" si="22"/>
-        <v>46331</v>
+        <v>46338</v>
       </c>
       <c r="S78" s="5">
         <f t="shared" si="23"/>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="T78" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -16227,7 +16227,7 @@
         <v>82</v>
       </c>
       <c r="B86" s="6">
-        <v>46332</v>
+        <v>46339</v>
       </c>
       <c r="C86" t="str">
         <f t="shared" si="14"/>
@@ -16259,11 +16259,11 @@
       </c>
       <c r="L86" s="5">
         <f t="shared" si="17"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="M86" s="5">
         <f t="shared" si="18"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="N86">
         <f t="shared" si="19"/>
@@ -16282,11 +16282,11 @@
       </c>
       <c r="R86" s="5">
         <f t="shared" si="22"/>
-        <v>46338</v>
+        <v>46345</v>
       </c>
       <c r="S86" s="5">
         <f t="shared" si="23"/>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="T86" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -16835,7 +16835,7 @@
         <v>90</v>
       </c>
       <c r="B94" s="6">
-        <v>46339</v>
+        <v>46346</v>
       </c>
       <c r="C94" t="str">
         <f t="shared" si="14"/>
@@ -16867,11 +16867,11 @@
       </c>
       <c r="L94" s="5">
         <f t="shared" si="17"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="M94" s="5">
         <f t="shared" si="18"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="N94">
         <f t="shared" si="19"/>
@@ -16890,11 +16890,11 @@
       </c>
       <c r="R94" s="5">
         <f t="shared" si="22"/>
-        <v>46345</v>
+        <v>46352</v>
       </c>
       <c r="S94" s="5">
         <f t="shared" si="23"/>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="T94" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -17443,7 +17443,7 @@
         <v>98</v>
       </c>
       <c r="B102" s="6">
-        <v>46346</v>
+        <v>46353</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="14"/>
@@ -17475,11 +17475,11 @@
       </c>
       <c r="L102" s="5">
         <f t="shared" si="17"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="M102" s="5">
         <f t="shared" si="18"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="N102">
         <f t="shared" si="19"/>
@@ -17498,11 +17498,11 @@
       </c>
       <c r="R102" s="5">
         <f t="shared" si="22"/>
-        <v>46352</v>
+        <v>46359</v>
       </c>
       <c r="S102" s="5">
         <f t="shared" si="23"/>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="T102" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -18051,7 +18051,7 @@
         <v>106</v>
       </c>
       <c r="B110" s="6">
-        <v>46353</v>
+        <v>46360</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="14"/>
@@ -18083,11 +18083,11 @@
       </c>
       <c r="L110" s="5">
         <f t="shared" si="17"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="M110" s="5">
         <f t="shared" si="18"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="N110">
         <f t="shared" si="19"/>
@@ -18106,11 +18106,11 @@
       </c>
       <c r="R110" s="5">
         <f t="shared" si="22"/>
-        <v>46359</v>
+        <v>46366</v>
       </c>
       <c r="S110" s="5">
         <f t="shared" si="23"/>
-        <v>46356</v>
+        <v>46363</v>
       </c>
       <c r="T110" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -18659,7 +18659,7 @@
         <v>114</v>
       </c>
       <c r="B118" s="6">
-        <v>46360</v>
+        <v>46367</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="14"/>
@@ -18691,11 +18691,11 @@
       </c>
       <c r="L118" s="5">
         <f t="shared" si="17"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="M118" s="5">
         <f t="shared" si="18"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="N118">
         <f t="shared" si="19"/>
@@ -18714,11 +18714,11 @@
       </c>
       <c r="R118" s="5">
         <f t="shared" si="22"/>
-        <v>46366</v>
+        <v>46373</v>
       </c>
       <c r="S118" s="5">
         <f t="shared" si="23"/>
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="T118" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19267,7 +19267,7 @@
         <v>122</v>
       </c>
       <c r="B126" s="6">
-        <v>46367</v>
+        <v>46374</v>
       </c>
       <c r="C126" t="str">
         <f t="shared" si="14"/>
@@ -19299,11 +19299,11 @@
       </c>
       <c r="L126" s="5">
         <f t="shared" si="17"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="M126" s="5">
         <f t="shared" si="18"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="N126">
         <f t="shared" si="19"/>
@@ -19322,11 +19322,11 @@
       </c>
       <c r="R126" s="5">
         <f t="shared" si="22"/>
-        <v>46373</v>
+        <v>46380</v>
       </c>
       <c r="S126" s="5">
         <f t="shared" si="23"/>
-        <v>46370</v>
+        <v>46377</v>
       </c>
       <c r="T126" s="7">
         <f t="shared" ca="1" si="24"/>
@@ -19870,75 +19870,61 @@
       </c>
     </row>
     <row r="134" spans="1:21">
-      <c r="A134">
+      <c r="A134" t="str">
         <f t="shared" si="26"/>
-        <v>130</v>
-      </c>
-      <c r="B134" s="6">
-        <v>46374</v>
-      </c>
+        <v/>
+      </c>
+      <c r="B134" s="6"/>
       <c r="C134" t="str">
         <f t="shared" si="27"/>
-        <v>vie</v>
-      </c>
-      <c r="D134" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E134" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="F134" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G134" s="8">
-        <v>1008</v>
-      </c>
-      <c r="H134" s="7">
+        <v/>
+      </c>
+      <c r="D134" s="9"/>
+      <c r="E134" s="9"/>
+      <c r="F134" s="9"/>
+      <c r="G134" s="8"/>
+      <c r="H134" s="7" t="str">
         <f t="shared" si="28"/>
-        <v>1008</v>
-      </c>
-      <c r="I134" s="9" t="s">
-        <v>239</v>
-      </c>
+        <v/>
+      </c>
+      <c r="I134" s="9"/>
       <c r="J134" s="6"/>
-      <c r="K134">
+      <c r="K134" t="str">
         <f t="shared" si="29"/>
-        <v>3</v>
-      </c>
-      <c r="L134" s="5">
+        <v/>
+      </c>
+      <c r="L134" s="5" t="str">
         <f t="shared" si="30"/>
-        <v>46377</v>
-      </c>
-      <c r="M134" s="5">
+        <v/>
+      </c>
+      <c r="M134" s="5" t="str">
         <f t="shared" si="31"/>
-        <v>46377</v>
-      </c>
-      <c r="N134">
+        <v/>
+      </c>
+      <c r="N134" t="str">
         <f t="shared" si="32"/>
-        <v>1</v>
-      </c>
-      <c r="O134" s="10">
+        <v/>
+      </c>
+      <c r="O134" s="10" t="str">
         <f t="shared" si="33"/>
-        <v>7.09</v>
-      </c>
-      <c r="P134" s="7">
+        <v/>
+      </c>
+      <c r="P134" s="7" t="str">
         <f t="shared" si="34"/>
-        <v>7146.72</v>
-      </c>
-      <c r="Q134" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="R134" s="5">
+        <v/>
+      </c>
+      <c r="Q134" s="9"/>
+      <c r="R134" s="5" t="str">
         <f t="shared" si="35"/>
-        <v>46380</v>
-      </c>
-      <c r="S134" s="5">
+        <v/>
+      </c>
+      <c r="S134" s="5" t="str">
         <f t="shared" si="36"/>
-        <v>46377</v>
-      </c>
-      <c r="T134" s="7">
-        <f t="shared" ca="1" si="37"/>
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="T134" s="7" t="str">
+        <f t="shared" si="37"/>
+        <v/>
       </c>
       <c r="U134" t="str">
         <f t="shared" si="38"/>
@@ -30551,11 +30537,11 @@
       </c>
       <c r="D8" s="7">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="2"/>
-        <v>19918</v>
+        <v>20926</v>
       </c>
       <c r="F8" s="7">
         <f>ROUND(Demanda!H8,0)</f>
@@ -30563,7 +30549,7 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" si="3"/>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="H8" s="7">
         <f ca="1">SUM($K$6:K7)*CajasProm</f>
@@ -30571,7 +30557,7 @@
       </c>
       <c r="I8" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="J8" s="21">
         <f t="shared" si="5"/>
@@ -30579,27 +30565,27 @@
       </c>
       <c r="K8" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25816</v>
+        <v>25824</v>
       </c>
       <c r="M8" s="22">
         <f ca="1">IF(Demanda!H9=0,"",L8/(Demanda!H9/DiasVenta))</f>
-        <v>8.6053333333333342</v>
+        <v>8.6080000000000005</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 1</v>
+        <v>OK</v>
       </c>
       <c r="O8" s="7">
         <f>O7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L8,0)</f>
-        <v>11851</v>
+        <v>12859</v>
       </c>
       <c r="P8" s="22">
         <f>IF(Demanda!L9=0,"",O8/(Demanda!L9/DiasVenta))</f>
-        <v>6.4024851431658565</v>
+        <v>6.9470556455969747</v>
       </c>
       <c r="Q8" s="7">
         <f>Q7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M8,0)</f>
@@ -30619,7 +30605,7 @@
       </c>
       <c r="U8" t="str">
         <f t="shared" si="9"/>
-        <v>Brasil</v>
+        <v>Bolivia</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -30633,15 +30619,15 @@
       </c>
       <c r="C9" s="7">
         <f t="shared" si="10"/>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" si="2"/>
-        <v>10918</v>
+        <v>8974</v>
       </c>
       <c r="F9" s="7">
         <f>ROUND(Demanda!H9,0)</f>
@@ -30649,15 +30635,15 @@
       </c>
       <c r="G9" s="7">
         <f t="shared" si="3"/>
-        <v>17734</v>
+        <v>16798</v>
       </c>
       <c r="H9" s="7">
         <f ca="1">SUM($K$6:K8)*CajasProm</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I9" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>18734</v>
+        <v>16798</v>
       </c>
       <c r="J9" s="21">
         <f t="shared" si="5"/>
@@ -30665,27 +30651,27 @@
       </c>
       <c r="K9" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25734</v>
+        <v>25798</v>
       </c>
       <c r="M9" s="22">
         <f ca="1">IF(Demanda!H10=0,"",L9/(Demanda!H10/DiasVenta))</f>
-        <v>8.5779999999999994</v>
+        <v>8.5993333333333339</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 7</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="O9" s="7">
         <f>O8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L9,0)</f>
-        <v>5713</v>
+        <v>4777</v>
       </c>
       <c r="P9" s="22">
         <f>IF(Demanda!L10=0,"",O9/(Demanda!L10/DiasVenta))</f>
-        <v>3.0864397622906536</v>
+        <v>2.5807671528903295</v>
       </c>
       <c r="Q9" s="7">
         <f>Q8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M9,0)</f>
@@ -30719,7 +30705,7 @@
       </c>
       <c r="C10" s="7">
         <f t="shared" si="10"/>
-        <v>17734</v>
+        <v>16798</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
@@ -30735,15 +30721,15 @@
       </c>
       <c r="G10" s="7">
         <f t="shared" si="3"/>
-        <v>13748</v>
+        <v>12812</v>
       </c>
       <c r="H10" s="7">
         <f ca="1">SUM($K$6:K9)*CajasProm</f>
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="I10" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>21748</v>
+        <v>21812</v>
       </c>
       <c r="J10" s="21">
         <f t="shared" si="5"/>
@@ -30755,11 +30741,11 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25748</v>
+        <v>25812</v>
       </c>
       <c r="M10" s="22">
         <f ca="1">IF(Demanda!H11=0,"",L10/(Demanda!H11/DiasVenta))</f>
-        <v>8.5826666666666664</v>
+        <v>8.6039999999999992</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30767,11 +30753,11 @@
       </c>
       <c r="O10" s="7">
         <f>O9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L10,0)</f>
-        <v>2671</v>
+        <v>1735</v>
       </c>
       <c r="P10" s="22">
         <f>IF(Demanda!L11=0,"",O10/(Demanda!L11/DiasVenta))</f>
-        <v>1.4430037817396002</v>
+        <v>0.9373311723392761</v>
       </c>
       <c r="Q10" s="7">
         <f>Q9+SUMIFS(CgCajas,CgSemana,A10,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M10,0)</f>
@@ -30805,7 +30791,7 @@
       </c>
       <c r="C11" s="7">
         <f t="shared" si="10"/>
-        <v>13748</v>
+        <v>12812</v>
       </c>
       <c r="D11" s="7">
         <f t="shared" si="1"/>
@@ -30821,15 +30807,15 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" si="3"/>
-        <v>4862</v>
+        <v>3926</v>
       </c>
       <c r="H11" s="7">
         <f ca="1">SUM($K$6:K10)*CajasProm</f>
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="I11" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16862</v>
+        <v>16926</v>
       </c>
       <c r="J11" s="21">
         <f t="shared" si="5"/>
@@ -30841,11 +30827,11 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25862</v>
+        <v>25926</v>
       </c>
       <c r="M11" s="22">
         <f ca="1">IF(Demanda!H12=0,"",L11/(Demanda!H12/DiasVenta))</f>
-        <v>8.6206666666666667</v>
+        <v>8.6419999999999995</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30853,11 +30839,11 @@
       </c>
       <c r="O11" s="7">
         <f>O10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L11,0)</f>
-        <v>-371</v>
+        <v>-1307</v>
       </c>
       <c r="P11" s="22">
         <f>IF(Demanda!L12=0,"",O11/(Demanda!L12/DiasVenta))</f>
-        <v>-0.20043219881145327</v>
+        <v>-0.70610480821177746</v>
       </c>
       <c r="Q11" s="7">
         <f>Q10+SUMIFS(CgCajas,CgSemana,A11,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M11,0)</f>
@@ -30891,7 +30877,7 @@
       </c>
       <c r="C12" s="7">
         <f t="shared" si="10"/>
-        <v>4862</v>
+        <v>3926</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="1"/>
@@ -30907,15 +30893,15 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" si="3"/>
-        <v>-5074</v>
+        <v>-6010</v>
       </c>
       <c r="H12" s="7">
         <f ca="1">SUM($K$6:K11)*CajasProm</f>
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15926</v>
+        <v>15990</v>
       </c>
       <c r="J12" s="21">
         <f t="shared" si="5"/>
@@ -30927,11 +30913,11 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25926</v>
+        <v>25990</v>
       </c>
       <c r="M12" s="22">
         <f ca="1">IF(Demanda!H13=0,"",L12/(Demanda!H13/DiasVenta))</f>
-        <v>8.6419999999999995</v>
+        <v>8.663333333333334</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -30939,11 +30925,11 @@
       </c>
       <c r="O12" s="7">
         <f>O11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L12,0)</f>
-        <v>-3413</v>
+        <v>-4349</v>
       </c>
       <c r="P12" s="22">
         <f>IF(Demanda!L13=0,"",O12/(Demanda!L13/DiasVenta))</f>
-        <v>-1.8438681793625067</v>
+        <v>-2.3495407887628308</v>
       </c>
       <c r="Q12" s="7">
         <f>Q11+SUMIFS(CgCajas,CgSemana,A12,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M12,0)</f>
@@ -30977,7 +30963,7 @@
       </c>
       <c r="C13" s="7">
         <f t="shared" si="10"/>
-        <v>-5074</v>
+        <v>-6010</v>
       </c>
       <c r="D13" s="7">
         <f t="shared" si="1"/>
@@ -30993,15 +30979,15 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" si="3"/>
-        <v>-15010</v>
+        <v>-15946</v>
       </c>
       <c r="H13" s="7">
         <f ca="1">SUM($K$6:K12)*CajasProm</f>
-        <v>31000</v>
+        <v>32000</v>
       </c>
       <c r="I13" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15990</v>
+        <v>16054</v>
       </c>
       <c r="J13" s="21">
         <f t="shared" si="5"/>
@@ -31009,27 +30995,27 @@
       </c>
       <c r="K13" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25990</v>
+        <v>25054</v>
       </c>
       <c r="M13" s="22">
         <f ca="1">IF(Demanda!H14=0,"",L13/(Demanda!H14/DiasVenta))</f>
-        <v>8.663333333333334</v>
+        <v>8.3513333333333328</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 10</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="O13" s="7">
         <f>O12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L13,0)</f>
-        <v>-6455</v>
+        <v>-7391</v>
       </c>
       <c r="P13" s="22">
         <f>IF(Demanda!L14=0,"",O13/(Demanda!L14/DiasVenta))</f>
-        <v>-3.4873041599135601</v>
+        <v>-3.9929767693138842</v>
       </c>
       <c r="Q13" s="7">
         <f>Q12+SUMIFS(CgCajas,CgSemana,A13,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M13,0)</f>
@@ -31063,7 +31049,7 @@
       </c>
       <c r="C14" s="7">
         <f t="shared" si="10"/>
-        <v>-15010</v>
+        <v>-15946</v>
       </c>
       <c r="D14" s="7">
         <f t="shared" si="1"/>
@@ -31079,7 +31065,7 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" si="3"/>
-        <v>-24946</v>
+        <v>-25882</v>
       </c>
       <c r="H14" s="7">
         <f ca="1">SUM($K$6:K13)*CajasProm</f>
@@ -31087,7 +31073,7 @@
       </c>
       <c r="I14" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16054</v>
+        <v>15118</v>
       </c>
       <c r="J14" s="21">
         <f t="shared" si="5"/>
@@ -31095,27 +31081,27 @@
       </c>
       <c r="K14" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25054</v>
+        <v>25118</v>
       </c>
       <c r="M14" s="22">
         <f ca="1">IF(Demanda!H15=0,"",L14/(Demanda!H15/DiasVenta))</f>
-        <v>8.3513333333333328</v>
+        <v>8.3726666666666674</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="O14" s="7">
         <f>O13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L14,0)</f>
-        <v>-9497</v>
+        <v>-10433</v>
       </c>
       <c r="P14" s="22">
         <f>IF(Demanda!L15=0,"",O14/(Demanda!L15/DiasVenta))</f>
-        <v>-5.1307401404646136</v>
+        <v>-5.6364127498649381</v>
       </c>
       <c r="Q14" s="7">
         <f>Q13+SUMIFS(CgCajas,CgSemana,A14,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M14,0)</f>
@@ -31149,7 +31135,7 @@
       </c>
       <c r="C15" s="7">
         <f t="shared" si="10"/>
-        <v>-24946</v>
+        <v>-25882</v>
       </c>
       <c r="D15" s="7">
         <f t="shared" si="1"/>
@@ -31165,15 +31151,15 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" si="3"/>
-        <v>-34882</v>
+        <v>-35818</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">SUM($K$6:K14)*CajasProm</f>
-        <v>50000</v>
+        <v>51000</v>
       </c>
       <c r="I15" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15118</v>
+        <v>15182</v>
       </c>
       <c r="J15" s="21">
         <f t="shared" si="5"/>
@@ -31185,11 +31171,11 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25118</v>
+        <v>25182</v>
       </c>
       <c r="M15" s="22">
         <f ca="1">IF(Demanda!H16=0,"",L15/(Demanda!H16/DiasVenta))</f>
-        <v>8.3726666666666674</v>
+        <v>8.3940000000000001</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31197,11 +31183,11 @@
       </c>
       <c r="O15" s="7">
         <f>O14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L15,0)</f>
-        <v>-12539</v>
+        <v>-13475</v>
       </c>
       <c r="P15" s="22">
         <f>IF(Demanda!L16=0,"",O15/(Demanda!L16/DiasVenta))</f>
-        <v>-6.7741761210156675</v>
+        <v>-7.2798487304159911</v>
       </c>
       <c r="Q15" s="7">
         <f>Q14+SUMIFS(CgCajas,CgSemana,A15,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M15,0)</f>
@@ -31235,7 +31221,7 @@
       </c>
       <c r="C16" s="7">
         <f t="shared" si="10"/>
-        <v>-34882</v>
+        <v>-35818</v>
       </c>
       <c r="D16" s="7">
         <f t="shared" si="1"/>
@@ -31251,15 +31237,15 @@
       </c>
       <c r="G16" s="7">
         <f t="shared" si="3"/>
-        <v>-44818</v>
+        <v>-45754</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">SUM($K$6:K15)*CajasProm</f>
-        <v>60000</v>
+        <v>61000</v>
       </c>
       <c r="I16" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15182</v>
+        <v>15246</v>
       </c>
       <c r="J16" s="21">
         <f t="shared" si="5"/>
@@ -31271,11 +31257,11 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25182</v>
+        <v>25246</v>
       </c>
       <c r="M16" s="22">
         <f ca="1">IF(Demanda!H17=0,"",L16/(Demanda!H17/DiasVenta))</f>
-        <v>8.3940000000000001</v>
+        <v>8.4153333333333329</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31283,11 +31269,11 @@
       </c>
       <c r="O16" s="7">
         <f>O15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L16,0)</f>
-        <v>-15581</v>
+        <v>-16517</v>
       </c>
       <c r="P16" s="22">
         <f>IF(Demanda!L17=0,"",O16/(Demanda!L17/DiasVenta))</f>
-        <v>-8.4176121015667213</v>
+        <v>-8.9232847109670441</v>
       </c>
       <c r="Q16" s="7">
         <f>Q15+SUMIFS(CgCajas,CgSemana,A16,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M16,0)</f>
@@ -31321,7 +31307,7 @@
       </c>
       <c r="C17" s="7">
         <f t="shared" si="10"/>
-        <v>-44818</v>
+        <v>-45754</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="1"/>
@@ -31337,15 +31323,15 @@
       </c>
       <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>-54754</v>
+        <v>-55690</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">SUM($K$6:K16)*CajasProm</f>
-        <v>70000</v>
+        <v>71000</v>
       </c>
       <c r="I17" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15246</v>
+        <v>15310</v>
       </c>
       <c r="J17" s="21">
         <f t="shared" si="5"/>
@@ -31357,11 +31343,11 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25246</v>
+        <v>25310</v>
       </c>
       <c r="M17" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L17/(Demanda!H18/DiasVenta))</f>
-        <v>8.4153333333333329</v>
+        <v>8.4366666666666674</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31369,11 +31355,11 @@
       </c>
       <c r="O17" s="7">
         <f>O16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L17,0)</f>
-        <v>-18623</v>
+        <v>-19559</v>
       </c>
       <c r="P17" s="22">
         <f>IF(Demanda!L18=0,"",O17/(Demanda!L18/DiasVenta))</f>
-        <v>-10.061048082117773</v>
+        <v>-10.566720691518098</v>
       </c>
       <c r="Q17" s="7">
         <f>Q16+SUMIFS(CgCajas,CgSemana,A17,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M17,0)</f>
@@ -31407,7 +31393,7 @@
       </c>
       <c r="C18" s="7">
         <f t="shared" si="10"/>
-        <v>-54754</v>
+        <v>-55690</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="1"/>
@@ -31423,15 +31409,15 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" si="3"/>
-        <v>-64690</v>
+        <v>-65626</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">SUM($K$6:K17)*CajasProm</f>
-        <v>80000</v>
+        <v>81000</v>
       </c>
       <c r="I18" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>15310</v>
+        <v>15374</v>
       </c>
       <c r="J18" s="21">
         <f t="shared" si="5"/>
@@ -31443,11 +31429,11 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25310</v>
+        <v>25374</v>
       </c>
       <c r="M18" s="22">
         <f ca="1">IF(Demanda!H18=0,"",L18/(Demanda!H18/DiasVenta))</f>
-        <v>8.4366666666666674</v>
+        <v>8.4580000000000002</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -31455,11 +31441,11 @@
       </c>
       <c r="O18" s="7">
         <f>O17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L18,0)</f>
-        <v>-21665</v>
+        <v>-22601</v>
       </c>
       <c r="P18" s="22">
         <f>IF(Demanda!L18=0,"",O18/(Demanda!L18/DiasVenta))</f>
-        <v>-11.704484062668827</v>
+        <v>-12.210156672069152</v>
       </c>
       <c r="Q18" s="7">
         <f>Q17+SUMIFS(CgCajas,CgSemana,A18,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M18,0)</f>
@@ -31685,11 +31671,11 @@
       </c>
       <c r="B8" s="7">
         <f ca="1">IF(A8="","",Proyeccion!I8)</f>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="C8" s="3">
         <f ca="1">IF(A8="","",Proyeccion!K8)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="str">
         <f ca="1">IF(A8="","","BR "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B8-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B8-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31697,7 +31683,7 @@
       </c>
       <c r="E8" t="str">
         <f ca="1">IF(A8="","",IF(C8&gt;0,Proyeccion!U8,"-"))</f>
-        <v>Brasil</v>
+        <v>-</v>
       </c>
       <c r="F8" t="str">
         <f ca="1">IF(A8="","","PY mie "&amp;TEXT(Proyeccion!A8-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A8-4,"dd/mm"))</f>
@@ -31705,15 +31691,15 @@
       </c>
       <c r="G8" s="22">
         <f ca="1">IF(A8="","",Proyeccion!M8)</f>
-        <v>8.6053333333333342</v>
+        <v>8.6080000000000005</v>
       </c>
       <c r="H8" t="str">
         <f ca="1">IF(A8="","",Proyeccion!N8)</f>
-        <v>CARGAR 1</v>
+        <v>OK</v>
       </c>
       <c r="I8" t="str">
         <f ca="1">IF(A8="","","Sab "&amp;TEXT(A8,"dd/mm")&amp;": "&amp;FIXED(B8,0)&amp;" cajas - descargan "&amp;Proyeccion!D8&amp;" - vende "&amp;FIXED(Proyeccion!F8,0)&amp;IF(C8&gt;0," -&gt; cargar "&amp;C8&amp;" mas hasta el "&amp;TEXT(Proyeccion!J8,"dd/mm")&amp;" ("&amp;E8&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 10/10: 24.816 cajas - descargan 20 - vende 18.000 -&gt; cargar 1 mas hasta el 06/10 (Brasil; BR hasta el 07/10)</v>
+        <v>Sab 10/10: 25.824 cajas - descargan 21 - vende 18.000 -&gt; ok</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -31723,11 +31709,11 @@
       </c>
       <c r="B9" s="7">
         <f ca="1">IF(A9="","",Proyeccion!I9)</f>
-        <v>18734</v>
+        <v>16798</v>
       </c>
       <c r="C9" s="3">
         <f ca="1">IF(A9="","",Proyeccion!K9)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D9" t="str">
         <f ca="1">IF(A9="","","BR "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B9-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B9-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31743,15 +31729,15 @@
       </c>
       <c r="G9" s="22">
         <f ca="1">IF(A9="","",Proyeccion!M9)</f>
-        <v>8.5779999999999994</v>
+        <v>8.5993333333333339</v>
       </c>
       <c r="H9" t="str">
         <f ca="1">IF(A9="","",Proyeccion!N9)</f>
-        <v>CARGAR 7</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="I9" t="str">
         <f ca="1">IF(A9="","","Sab "&amp;TEXT(A9,"dd/mm")&amp;": "&amp;FIXED(B9,0)&amp;" cajas - descargan "&amp;Proyeccion!D9&amp;" - vende "&amp;FIXED(Proyeccion!F9,0)&amp;IF(C9&gt;0," -&gt; cargar "&amp;C9&amp;" mas hasta el "&amp;TEXT(Proyeccion!J9,"dd/mm")&amp;" ("&amp;E9&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 17/10: 18.734 cajas - descargan 11 - vende 18.000 -&gt; cargar 7 mas hasta el 13/10 (Brasil; BR hasta el 14/10)</v>
+        <v>Sab 17/10: 16.798 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 13/10 (Brasil; BR hasta el 14/10)</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -31761,7 +31747,7 @@
       </c>
       <c r="B10" s="7">
         <f ca="1">IF(A10="","",Proyeccion!I10)</f>
-        <v>21748</v>
+        <v>21812</v>
       </c>
       <c r="C10" s="3">
         <f ca="1">IF(A10="","",Proyeccion!K10)</f>
@@ -31781,7 +31767,7 @@
       </c>
       <c r="G10" s="22">
         <f ca="1">IF(A10="","",Proyeccion!M10)</f>
-        <v>8.5826666666666664</v>
+        <v>8.6039999999999992</v>
       </c>
       <c r="H10" t="str">
         <f ca="1">IF(A10="","",Proyeccion!N10)</f>
@@ -31789,7 +31775,7 @@
       </c>
       <c r="I10" t="str">
         <f ca="1">IF(A10="","","Sab "&amp;TEXT(A10,"dd/mm")&amp;": "&amp;FIXED(B10,0)&amp;" cajas - descargan "&amp;Proyeccion!D10&amp;" - vende "&amp;FIXED(Proyeccion!F10,0)&amp;IF(C10&gt;0," -&gt; cargar "&amp;C10&amp;" mas hasta el "&amp;TEXT(Proyeccion!J10,"dd/mm")&amp;" ("&amp;E10&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B10-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 24/10: 21.748 cajas - descargan 14 - vende 18.000 -&gt; cargar 4 mas hasta el 20/10 (Brasil; BR hasta el 21/10)</v>
+        <v>Sab 24/10: 21.812 cajas - descargan 14 - vende 18.000 -&gt; cargar 4 mas hasta el 20/10 (Brasil; BR hasta el 21/10)</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -31799,7 +31785,7 @@
       </c>
       <c r="B11" s="7">
         <f ca="1">IF(A11="","",Proyeccion!I11)</f>
-        <v>16862</v>
+        <v>16926</v>
       </c>
       <c r="C11" s="3">
         <f ca="1">IF(A11="","",Proyeccion!K11)</f>
@@ -31819,7 +31805,7 @@
       </c>
       <c r="G11" s="22">
         <f ca="1">IF(A11="","",Proyeccion!M11)</f>
-        <v>8.6206666666666667</v>
+        <v>8.6419999999999995</v>
       </c>
       <c r="H11" t="str">
         <f ca="1">IF(A11="","",Proyeccion!N11)</f>
@@ -31827,7 +31813,7 @@
       </c>
       <c r="I11" t="str">
         <f ca="1">IF(A11="","","Sab "&amp;TEXT(A11,"dd/mm")&amp;": "&amp;FIXED(B11,0)&amp;" cajas - descargan "&amp;Proyeccion!D11&amp;" - vende "&amp;FIXED(Proyeccion!F11,0)&amp;IF(C11&gt;0," -&gt; cargar "&amp;C11&amp;" mas hasta el "&amp;TEXT(Proyeccion!J11,"dd/mm")&amp;" ("&amp;E11&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B11-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 31/10: 16.862 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 27/10 (Brasil; BR hasta el 28/10)</v>
+        <v>Sab 31/10: 16.926 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 27/10 (Brasil; BR hasta el 28/10)</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -31837,7 +31823,7 @@
       </c>
       <c r="B12" s="7">
         <f ca="1">IF(A12="","",Proyeccion!I12)</f>
-        <v>15926</v>
+        <v>15990</v>
       </c>
       <c r="C12" s="3">
         <f ca="1">IF(A12="","",Proyeccion!K12)</f>
@@ -31857,7 +31843,7 @@
       </c>
       <c r="G12" s="22">
         <f ca="1">IF(A12="","",Proyeccion!M12)</f>
-        <v>8.6419999999999995</v>
+        <v>8.663333333333334</v>
       </c>
       <c r="H12" t="str">
         <f ca="1">IF(A12="","",Proyeccion!N12)</f>
@@ -31865,7 +31851,7 @@
       </c>
       <c r="I12" t="str">
         <f ca="1">IF(A12="","","Sab "&amp;TEXT(A12,"dd/mm")&amp;": "&amp;FIXED(B12,0)&amp;" cajas - descargan "&amp;Proyeccion!D12&amp;" - vende "&amp;FIXED(Proyeccion!F12,0)&amp;IF(C12&gt;0," -&gt; cargar "&amp;C12&amp;" mas hasta el "&amp;TEXT(Proyeccion!J12,"dd/mm")&amp;" ("&amp;E12&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B12-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 07/11: 15.926 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
+        <v>Sab 07/11: 15.990 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 03/11 (Bolivia; BR hasta el 04/11)</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -31875,11 +31861,11 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IF(A13="","",Proyeccion!I13)</f>
-        <v>15990</v>
+        <v>16054</v>
       </c>
       <c r="C13" s="3">
         <f ca="1">IF(A13="","",Proyeccion!K13)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(A13="","","BR "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B13-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B13-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31895,15 +31881,15 @@
       </c>
       <c r="G13" s="22">
         <f ca="1">IF(A13="","",Proyeccion!M13)</f>
-        <v>8.663333333333334</v>
+        <v>8.3513333333333328</v>
       </c>
       <c r="H13" t="str">
         <f ca="1">IF(A13="","",Proyeccion!N13)</f>
-        <v>CARGAR 10</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="I13" t="str">
         <f ca="1">IF(A13="","","Sab "&amp;TEXT(A13,"dd/mm")&amp;": "&amp;FIXED(B13,0)&amp;" cajas - descargan "&amp;Proyeccion!D13&amp;" - vende "&amp;FIXED(Proyeccion!F13,0)&amp;IF(C13&gt;0," -&gt; cargar "&amp;C13&amp;" mas hasta el "&amp;TEXT(Proyeccion!J13,"dd/mm")&amp;" ("&amp;E13&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B13-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 14/11: 15.990 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
+        <v>Sab 14/11: 16.054 cajas - descargan 8 - vende 18.000 -&gt; cargar 9 mas hasta el 10/11 (Bolivia; BR hasta el 11/11)</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -31913,11 +31899,11 @@
       </c>
       <c r="B14" s="7">
         <f ca="1">IF(A14="","",Proyeccion!I14)</f>
-        <v>16054</v>
+        <v>15118</v>
       </c>
       <c r="C14" s="3">
         <f ca="1">IF(A14="","",Proyeccion!K14)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" t="str">
         <f ca="1">IF(A14="","","BR "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B14-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B14-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31933,15 +31919,15 @@
       </c>
       <c r="G14" s="22">
         <f ca="1">IF(A14="","",Proyeccion!M14)</f>
-        <v>8.3513333333333328</v>
+        <v>8.3726666666666674</v>
       </c>
       <c r="H14" t="str">
         <f ca="1">IF(A14="","",Proyeccion!N14)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 10</v>
       </c>
       <c r="I14" t="str">
         <f ca="1">IF(A14="","","Sab "&amp;TEXT(A14,"dd/mm")&amp;": "&amp;FIXED(B14,0)&amp;" cajas - descargan "&amp;Proyeccion!D14&amp;" - vende "&amp;FIXED(Proyeccion!F14,0)&amp;IF(C14&gt;0," -&gt; cargar "&amp;C14&amp;" mas hasta el "&amp;TEXT(Proyeccion!J14,"dd/mm")&amp;" ("&amp;E14&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B14-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 21/11: 16.054 cajas - descargan 8 - vende 18.000 -&gt; cargar 9 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
+        <v>Sab 21/11: 15.118 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 17/11 (Bolivia; BR hasta el 18/11)</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -31951,7 +31937,7 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(A15="","",Proyeccion!I15)</f>
-        <v>15118</v>
+        <v>15182</v>
       </c>
       <c r="C15" s="3">
         <f ca="1">IF(A15="","",Proyeccion!K15)</f>
@@ -31971,7 +31957,7 @@
       </c>
       <c r="G15" s="22">
         <f ca="1">IF(A15="","",Proyeccion!M15)</f>
-        <v>8.3726666666666674</v>
+        <v>8.3940000000000001</v>
       </c>
       <c r="H15" t="str">
         <f ca="1">IF(A15="","",Proyeccion!N15)</f>
@@ -31979,7 +31965,7 @@
       </c>
       <c r="I15" t="str">
         <f ca="1">IF(A15="","","Sab "&amp;TEXT(A15,"dd/mm")&amp;": "&amp;FIXED(B15,0)&amp;" cajas - descargan "&amp;Proyeccion!D15&amp;" - vende "&amp;FIXED(Proyeccion!F15,0)&amp;IF(C15&gt;0," -&gt; cargar "&amp;C15&amp;" mas hasta el "&amp;TEXT(Proyeccion!J15,"dd/mm")&amp;" ("&amp;E15&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B15-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 28/11: 15.118 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
+        <v>Sab 28/11: 15.182 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 24/11 (Bolivia; BR hasta el 25/11)</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -31989,7 +31975,7 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(A16="","",Proyeccion!I16)</f>
-        <v>15182</v>
+        <v>15246</v>
       </c>
       <c r="C16" s="3">
         <f ca="1">IF(A16="","",Proyeccion!K16)</f>
@@ -32009,7 +31995,7 @@
       </c>
       <c r="G16" s="22">
         <f ca="1">IF(A16="","",Proyeccion!M16)</f>
-        <v>8.3940000000000001</v>
+        <v>8.4153333333333329</v>
       </c>
       <c r="H16" t="str">
         <f ca="1">IF(A16="","",Proyeccion!N16)</f>
@@ -32017,7 +32003,7 @@
       </c>
       <c r="I16" t="str">
         <f ca="1">IF(A16="","","Sab "&amp;TEXT(A16,"dd/mm")&amp;": "&amp;FIXED(B16,0)&amp;" cajas - descargan "&amp;Proyeccion!D16&amp;" - vende "&amp;FIXED(Proyeccion!F16,0)&amp;IF(C16&gt;0," -&gt; cargar "&amp;C16&amp;" mas hasta el "&amp;TEXT(Proyeccion!J16,"dd/mm")&amp;" ("&amp;E16&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B16-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 05/12: 15.182 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
+        <v>Sab 05/12: 15.246 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 01/12 (Bolivia; BR hasta el 02/12)</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -32027,7 +32013,7 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(A17="","",Proyeccion!I17)</f>
-        <v>15246</v>
+        <v>15310</v>
       </c>
       <c r="C17" s="3">
         <f ca="1">IF(A17="","",Proyeccion!K17)</f>
@@ -32047,7 +32033,7 @@
       </c>
       <c r="G17" s="22">
         <f ca="1">IF(A17="","",Proyeccion!M17)</f>
-        <v>8.4153333333333329</v>
+        <v>8.4366666666666674</v>
       </c>
       <c r="H17" t="str">
         <f ca="1">IF(A17="","",Proyeccion!N17)</f>
@@ -32055,7 +32041,7 @@
       </c>
       <c r="I17" t="str">
         <f ca="1">IF(A17="","","Sab "&amp;TEXT(A17,"dd/mm")&amp;": "&amp;FIXED(B17,0)&amp;" cajas - descargan "&amp;Proyeccion!D17&amp;" - vende "&amp;FIXED(Proyeccion!F17,0)&amp;IF(C17&gt;0," -&gt; cargar "&amp;C17&amp;" mas hasta el "&amp;TEXT(Proyeccion!J17,"dd/mm")&amp;" ("&amp;E17&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B17-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 12/12: 15.246 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
+        <v>Sab 12/12: 15.310 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 08/12 (Bolivia; BR hasta el 09/12)</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -32065,7 +32051,7 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(A18="","",Proyeccion!I18)</f>
-        <v>15310</v>
+        <v>15374</v>
       </c>
       <c r="C18" s="3">
         <f ca="1">IF(A18="","",Proyeccion!K18)</f>
@@ -32085,7 +32071,7 @@
       </c>
       <c r="G18" s="22">
         <f ca="1">IF(A18="","",Proyeccion!M18)</f>
-        <v>8.4366666666666674</v>
+        <v>8.4580000000000002</v>
       </c>
       <c r="H18" t="str">
         <f ca="1">IF(A18="","",Proyeccion!N18)</f>
@@ -32093,7 +32079,7 @@
       </c>
       <c r="I18" t="str">
         <f ca="1">IF(A18="","","Sab "&amp;TEXT(A18,"dd/mm")&amp;": "&amp;FIXED(B18,0)&amp;" cajas - descargan "&amp;Proyeccion!D18&amp;" - vende "&amp;FIXED(Proyeccion!F18,0)&amp;IF(C18&gt;0," -&gt; cargar "&amp;C18&amp;" mas hasta el "&amp;TEXT(Proyeccion!J18,"dd/mm")&amp;" ("&amp;E18&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B18-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 19/12: 15.310 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
+        <v>Sab 19/12: 15.374 cajas - descargan 8 - vende 18.000 -&gt; cargar 10 mas hasta el 15/12 (Bolivia; BR hasta el 16/12)</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="33.950000000000003" customHeight="1">
@@ -32318,11 +32304,11 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>11851</v>
+        <v>12859</v>
       </c>
       <c r="C13" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>6.4024851431658565</v>
+        <v>6.9470556455969747</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(B13="","",IF(B13&lt;0,"FALTA",IF(C13&lt;2,"CRITICO",IF(C13&lt;CoberturaObjetivo,"JUSTO",IF(C13&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32381,19 +32367,19 @@
       </c>
       <c r="B16" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="C16" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>8.6053333333333342</v>
+        <v>8.6080000000000005</v>
       </c>
       <c r="D16" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>CARGAR 1</v>
+        <v>OK</v>
       </c>
       <c r="E16" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 1 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
+        <v>ok, cierra sobre 25.000</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -32429,11 +32415,11 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>5713</v>
+        <v>4777</v>
       </c>
       <c r="C20" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>3.0864397622906536</v>
+        <v>2.5807671528903295</v>
       </c>
       <c r="D20" t="str">
         <f ca="1">IF(B20="","",IF(B20&lt;0,"FALTA",IF(C20&lt;2,"CRITICO",IF(C20&lt;CoberturaObjetivo,"JUSTO",IF(C20&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32492,19 +32478,19 @@
       </c>
       <c r="B23" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>18734</v>
+        <v>16798</v>
       </c>
       <c r="C23" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>8.5779999999999994</v>
+        <v>8.5993333333333339</v>
       </c>
       <c r="D23" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>CARGAR 7</v>
+        <v>CARGAR 9</v>
       </c>
       <c r="E23" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 7 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
+        <v>cargar 9 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30">
@@ -32549,7 +32535,7 @@
     <row r="29" spans="1:5">
       <c r="A29" s="45" t="str">
         <f>"Dictados que Aloha aun no tiene: "&amp;COUNTIFS(CgEstado,"Dictado",CgCuenta,1)&amp;" camiones. Pasan a Aloha cuando se cargan en el sistema."</f>
-        <v>Dictados que Aloha aun no tiene: 32 camiones. Pasan a Aloha cuando se cargan en el sistema.</v>
+        <v>Dictados que Aloha aun no tiene: 31 camiones. Pasan a Aloha cuando se cargan en el sistema.</v>
       </c>
       <c r="B29" s="46"/>
       <c r="C29" s="46"/>
@@ -32559,7 +32545,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.880 (plan: 24.816).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.880 (plan: 25.824).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32876,7 +32862,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>19918</v>
+        <v>20926</v>
       </c>
       <c r="D8" s="7">
         <f>Proyeccion!F8</f>
@@ -32884,7 +32870,7 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>28216</v>
+        <v>29224</v>
       </c>
       <c r="F8">
         <f ca="1">IF(AND(E8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-E8)/CajasProm,0),0)</f>
@@ -32892,19 +32878,19 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>24816</v>
+        <v>25824</v>
       </c>
       <c r="H8">
         <f ca="1">IF(AND(G8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-G8)/CajasProm,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>21416</v>
+        <v>22424</v>
       </c>
       <c r="J8">
         <f ca="1">IF(AND(I8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-I8)/CajasProm,0),0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
@@ -32920,15 +32906,15 @@
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>21876</v>
+        <v>22884</v>
       </c>
       <c r="O8" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>23816</v>
+        <v>24824</v>
       </c>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>23766</v>
+        <v>24774</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -32942,7 +32928,7 @@
       </c>
       <c r="C9" s="7">
         <f>Proyeccion!E9</f>
-        <v>10918</v>
+        <v>8974</v>
       </c>
       <c r="D9" s="7">
         <f>Proyeccion!F9</f>
@@ -32950,35 +32936,35 @@
       </c>
       <c r="E9" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>22934</v>
+        <v>21998</v>
       </c>
       <c r="F9">
         <f ca="1">IF(AND(E9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-E9)/CajasProm,0),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>18734</v>
+        <v>16798</v>
       </c>
       <c r="H9">
         <f ca="1">IF(AND(G9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-G9)/CajasProm,0),0)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I9" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>16534</v>
+        <v>14598</v>
       </c>
       <c r="J9">
         <f ca="1">IF(AND(I9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-I9)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
-        <v>18854</v>
+        <v>17918</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>26734</v>
+        <v>25798</v>
       </c>
       <c r="M9">
         <f ca="1">IF(AND(L9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-L9)/CajasProm,0),0)</f>
@@ -32986,15 +32972,15 @@
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>15794</v>
+        <v>13858</v>
       </c>
       <c r="O9" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>17734</v>
+        <v>15798</v>
       </c>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>16634</v>
+        <v>14698</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -33016,7 +33002,7 @@
       </c>
       <c r="E10" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>23748</v>
+        <v>23812</v>
       </c>
       <c r="F10">
         <f ca="1">IF(AND(E10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-E10)/CajasProm,0),0)</f>
@@ -33024,7 +33010,7 @@
       </c>
       <c r="G10" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>21748</v>
+        <v>21812</v>
       </c>
       <c r="H10">
         <f ca="1">IF(AND(G10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-G10)/CajasProm,0),0)</f>
@@ -33032,7 +33018,7 @@
       </c>
       <c r="I10" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>19748</v>
+        <v>19812</v>
       </c>
       <c r="J10">
         <f ca="1">IF(AND(I10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-I10)/CajasProm,0),0)</f>
@@ -33044,23 +33030,23 @@
       </c>
       <c r="L10" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>22748</v>
+        <v>21812</v>
       </c>
       <c r="M10">
         <f ca="1">IF(AND(L10&lt;MinimoSabado,Proyeccion!J10&gt;=FechaHoy),ROUNDUP((MinimoSabado-L10)/CajasProm,0),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>18808</v>
+        <v>18872</v>
       </c>
       <c r="O10" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>20748</v>
+        <v>20812</v>
       </c>
       <c r="P10" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>19648</v>
+        <v>19712</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -33082,7 +33068,7 @@
       </c>
       <c r="E11" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>18662</v>
+        <v>18726</v>
       </c>
       <c r="F11">
         <f ca="1">IF(AND(E11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-E11)/CajasProm,0),0)</f>
@@ -33090,7 +33076,7 @@
       </c>
       <c r="G11" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16862</v>
+        <v>16926</v>
       </c>
       <c r="H11">
         <f ca="1">IF(AND(G11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-G11)/CajasProm,0),0)</f>
@@ -33098,7 +33084,7 @@
       </c>
       <c r="I11" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>15062</v>
+        <v>15126</v>
       </c>
       <c r="J11">
         <f ca="1">IF(AND(I11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-I11)/CajasProm,0),0)</f>
@@ -33110,7 +33096,7 @@
       </c>
       <c r="L11" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16862</v>
+        <v>16926</v>
       </c>
       <c r="M11">
         <f ca="1">IF(AND(L11&lt;MinimoSabado,Proyeccion!J11&gt;=FechaHoy),ROUNDUP((MinimoSabado-L11)/CajasProm,0),0)</f>
@@ -33118,15 +33104,15 @@
       </c>
       <c r="N11" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13922</v>
+        <v>13986</v>
       </c>
       <c r="O11" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15862</v>
+        <v>15926</v>
       </c>
       <c r="P11" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14762</v>
+        <v>14826</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -33148,7 +33134,7 @@
       </c>
       <c r="E12" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17526</v>
+        <v>17590</v>
       </c>
       <c r="F12">
         <f ca="1">IF(AND(E12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-E12)/CajasProm,0),0)</f>
@@ -33156,7 +33142,7 @@
       </c>
       <c r="G12" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15926</v>
+        <v>15990</v>
       </c>
       <c r="H12">
         <f ca="1">IF(AND(G12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-G12)/CajasProm,0),0)</f>
@@ -33164,7 +33150,7 @@
       </c>
       <c r="I12" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13326</v>
+        <v>13390</v>
       </c>
       <c r="J12">
         <f ca="1">IF(AND(I12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-I12)/CajasProm,0),0)</f>
@@ -33176,7 +33162,7 @@
       </c>
       <c r="L12" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15926</v>
+        <v>15990</v>
       </c>
       <c r="M12">
         <f ca="1">IF(AND(L12&lt;MinimoSabado,Proyeccion!J12&gt;=FechaHoy),ROUNDUP((MinimoSabado-L12)/CajasProm,0),0)</f>
@@ -33184,15 +33170,15 @@
       </c>
       <c r="N12" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12986</v>
+        <v>13050</v>
       </c>
       <c r="O12" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14926</v>
+        <v>14990</v>
       </c>
       <c r="P12" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13826</v>
+        <v>13890</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -33214,7 +33200,7 @@
       </c>
       <c r="E13" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17390</v>
+        <v>17454</v>
       </c>
       <c r="F13">
         <f ca="1">IF(AND(E13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-E13)/CajasProm,0),0)</f>
@@ -33222,15 +33208,15 @@
       </c>
       <c r="G13" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15990</v>
+        <v>16054</v>
       </c>
       <c r="H13">
         <f ca="1">IF(AND(G13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-G13)/CajasProm,0),0)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I13" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13590</v>
+        <v>13654</v>
       </c>
       <c r="J13">
         <f ca="1">IF(AND(I13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-I13)/CajasProm,0),0)</f>
@@ -33242,23 +33228,23 @@
       </c>
       <c r="L13" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15990</v>
+        <v>16054</v>
       </c>
       <c r="M13">
         <f ca="1">IF(AND(L13&lt;MinimoSabado,Proyeccion!J13&gt;=FechaHoy),ROUNDUP((MinimoSabado-L13)/CajasProm,0),0)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N13" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13050</v>
+        <v>13114</v>
       </c>
       <c r="O13" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14990</v>
+        <v>15054</v>
       </c>
       <c r="P13" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13890</v>
+        <v>13954</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -33280,7 +33266,7 @@
       </c>
       <c r="E14" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17254</v>
+        <v>17318</v>
       </c>
       <c r="F14">
         <f ca="1">IF(AND(E14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-E14)/CajasProm,0),0)</f>
@@ -33288,15 +33274,15 @@
       </c>
       <c r="G14" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16054</v>
+        <v>15118</v>
       </c>
       <c r="H14">
         <f ca="1">IF(AND(G14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-G14)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I14" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13854</v>
+        <v>13918</v>
       </c>
       <c r="J14">
         <f ca="1">IF(AND(I14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-I14)/CajasProm,0),0)</f>
@@ -33308,23 +33294,23 @@
       </c>
       <c r="L14" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>16054</v>
+        <v>15118</v>
       </c>
       <c r="M14">
         <f ca="1">IF(AND(L14&lt;MinimoSabado,Proyeccion!J14&gt;=FechaHoy),ROUNDUP((MinimoSabado-L14)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N14" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13114</v>
+        <v>12178</v>
       </c>
       <c r="O14" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15054</v>
+        <v>14118</v>
       </c>
       <c r="P14" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13954</v>
+        <v>13018</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -33346,7 +33332,7 @@
       </c>
       <c r="E15" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17118</v>
+        <v>17182</v>
       </c>
       <c r="F15">
         <f ca="1">IF(AND(E15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-E15)/CajasProm,0),0)</f>
@@ -33354,7 +33340,7 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15118</v>
+        <v>15182</v>
       </c>
       <c r="H15">
         <f ca="1">IF(AND(G15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-G15)/CajasProm,0),0)</f>
@@ -33362,7 +33348,7 @@
       </c>
       <c r="I15" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14118</v>
+        <v>14182</v>
       </c>
       <c r="J15">
         <f ca="1">IF(AND(I15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-I15)/CajasProm,0),0)</f>
@@ -33374,7 +33360,7 @@
       </c>
       <c r="L15" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15118</v>
+        <v>15182</v>
       </c>
       <c r="M15">
         <f ca="1">IF(AND(L15&lt;MinimoSabado,Proyeccion!J15&gt;=FechaHoy),ROUNDUP((MinimoSabado-L15)/CajasProm,0),0)</f>
@@ -33382,15 +33368,15 @@
       </c>
       <c r="N15" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12178</v>
+        <v>12242</v>
       </c>
       <c r="O15" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14118</v>
+        <v>14182</v>
       </c>
       <c r="P15" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13018</v>
+        <v>13082</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -33412,15 +33398,15 @@
       </c>
       <c r="E16" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>16982</v>
+        <v>17046</v>
       </c>
       <c r="F16">
         <f ca="1">IF(AND(E16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-E16)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G16" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15182</v>
+        <v>15246</v>
       </c>
       <c r="H16">
         <f ca="1">IF(AND(G16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-G16)/CajasProm,0),0)</f>
@@ -33428,7 +33414,7 @@
       </c>
       <c r="I16" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13382</v>
+        <v>13446</v>
       </c>
       <c r="J16">
         <f ca="1">IF(AND(I16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-I16)/CajasProm,0),0)</f>
@@ -33440,7 +33426,7 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15182</v>
+        <v>15246</v>
       </c>
       <c r="M16">
         <f ca="1">IF(AND(L16&lt;MinimoSabado,Proyeccion!J16&gt;=FechaHoy),ROUNDUP((MinimoSabado-L16)/CajasProm,0),0)</f>
@@ -33448,15 +33434,15 @@
       </c>
       <c r="N16" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12242</v>
+        <v>12306</v>
       </c>
       <c r="O16" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14182</v>
+        <v>14246</v>
       </c>
       <c r="P16" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13082</v>
+        <v>13146</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -33478,15 +33464,15 @@
       </c>
       <c r="E17" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17846</v>
+        <v>16910</v>
       </c>
       <c r="F17">
         <f ca="1">IF(AND(E17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-E17)/CajasProm,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G17" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15246</v>
+        <v>15310</v>
       </c>
       <c r="H17">
         <f ca="1">IF(AND(G17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-G17)/CajasProm,0),0)</f>
@@ -33494,7 +33480,7 @@
       </c>
       <c r="I17" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13646</v>
+        <v>13710</v>
       </c>
       <c r="J17">
         <f ca="1">IF(AND(I17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-I17)/CajasProm,0),0)</f>
@@ -33506,7 +33492,7 @@
       </c>
       <c r="L17" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15246</v>
+        <v>15310</v>
       </c>
       <c r="M17">
         <f ca="1">IF(AND(L17&lt;MinimoSabado,Proyeccion!J17&gt;=FechaHoy),ROUNDUP((MinimoSabado-L17)/CajasProm,0),0)</f>
@@ -33514,15 +33500,15 @@
       </c>
       <c r="N17" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12306</v>
+        <v>12370</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14246</v>
+        <v>14310</v>
       </c>
       <c r="P17" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13146</v>
+        <v>13210</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -33544,7 +33530,7 @@
       </c>
       <c r="E18" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>17710</v>
+        <v>17774</v>
       </c>
       <c r="F18">
         <f ca="1">IF(AND(E18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-E18)/CajasProm,0),0)</f>
@@ -33552,7 +33538,7 @@
       </c>
       <c r="G18" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>15310</v>
+        <v>15374</v>
       </c>
       <c r="H18">
         <f ca="1">IF(AND(G18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-G18)/CajasProm,0),0)</f>
@@ -33560,7 +33546,7 @@
       </c>
       <c r="I18" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>13910</v>
+        <v>13974</v>
       </c>
       <c r="J18">
         <f ca="1">IF(AND(I18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-I18)/CajasProm,0),0)</f>
@@ -33572,7 +33558,7 @@
       </c>
       <c r="L18" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>15310</v>
+        <v>15374</v>
       </c>
       <c r="M18">
         <f ca="1">IF(AND(L18&lt;MinimoSabado,Proyeccion!J18&gt;=FechaHoy),ROUNDUP((MinimoSabado-L18)/CajasProm,0),0)</f>
@@ -33580,15 +33566,15 @@
       </c>
       <c r="N18" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>12370</v>
+        <v>12434</v>
       </c>
       <c r="O18" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>14310</v>
+        <v>14374</v>
       </c>
       <c r="P18" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>13210</v>
+        <v>13274</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="63.95" customHeight="1">

</xml_diff>

<commit_message>
plan de compras: Gilson vuelve al viernes 09/10
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan_compras/Plan_Compras_Simulado.xlsx
+++ b/plan_compras/Plan_Compras_Simulado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\plan_compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F346E5D6-36FE-4E2A-ABFB-9222F388B35D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817C7567-DC03-4B8B-B936-FA9FEF41E80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -115,7 +115,7 @@
     <t>PLAN DE COMPRAS SIMULADO - Almar S.R.L. (banana Brasil + Paraguay + Bolivia)</t>
   </si>
   <si>
-    <t>Generado el 01/10/2026 18:41 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
+    <t>Generado el 01/10/2026 18:45 a partir de plan_compras.json (conteo del 26/09/2026). Planilla de trabajo: se edita a mano, no la pisa el script.</t>
   </si>
   <si>
     <t>PARA QUE SIRVE</t>
@@ -814,10 +814,10 @@
     <t>nota 01/10: cuarta (antes martes, sacada el 30/09); transportista supuesto</t>
   </si>
   <si>
-    <t>nota 01/10 (v3): cuarta (antes sexta); transportista supuesto = semana anterior</t>
-  </si>
-  <si>
     <t>nota 30/09: sexta; transportista supuesto = semana anterior</t>
+  </si>
+  <si>
+    <t>nota 01/10 (v4): sexta (Gonzalo: "prefiero cerrar en casi 25 mil que casi 26 mil"); transportista supuesto = semana anterior</t>
   </si>
   <si>
     <t>Paraguay (supuesto)</t>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>20926</v>
+        <v>19918</v>
       </c>
       <c r="D8" s="7">
         <f>Demanda!H9</f>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="H8" s="7">
         <f ca="1">Proyeccion!L8</f>
-        <v>25824</v>
+        <v>25816</v>
       </c>
       <c r="I8" s="7" t="str">
         <f t="shared" si="3"/>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="C9" s="7">
         <f>Proyeccion!E9</f>
-        <v>8974</v>
+        <v>9982</v>
       </c>
       <c r="D9" s="7">
         <f>Demanda!H10</f>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B9" s="25">
         <f ca="1">IFERROR(INDEX(PrACargar,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>303</v>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B10" s="24">
         <f ca="1">AVERAGEIFS(PrCobertura,PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>8.3610000000000007</v>
+        <v>8.3603333333333332</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>305</v>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B11" s="25">
         <f ca="1">COUNTIFS(PrACargar,"&gt;0",PrSemana,"&gt;="&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1),PrSemana,"&lt;"&amp;(FechaHoy-WEEKDAY(FechaHoy,2)+1+28))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>307</v>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="O10">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P10" t="s">
         <v>3</v>
@@ -12513,10 +12513,10 @@
         <v>58</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G37" s="8">
         <v>1008</v>
@@ -12554,7 +12554,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q37" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="R37" s="5">
         <f t="shared" si="9"/>
@@ -12579,20 +12579,20 @@
         <v>34</v>
       </c>
       <c r="B38" s="6">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="1"/>
-        <v>mié</v>
+        <v>vie</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>58</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="G38" s="8">
         <v>1008</v>
@@ -12611,11 +12611,11 @@
       </c>
       <c r="L38" s="5">
         <f t="shared" si="4"/>
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="M38" s="5">
         <f t="shared" si="5"/>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="N38">
         <f t="shared" si="6"/>
@@ -12630,11 +12630,11 @@
         <v>7146.72</v>
       </c>
       <c r="Q38" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="R38" s="5">
         <f t="shared" si="9"/>
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="S38" s="5">
         <f t="shared" si="10"/>
@@ -12665,10 +12665,10 @@
         <v>58</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="G39" s="8">
         <v>1008</v>
@@ -12782,7 +12782,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q40" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R40" s="5">
         <f t="shared" si="9"/>
@@ -12858,7 +12858,7 @@
         <v>7146.72</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R41" s="5">
         <f t="shared" si="9"/>
@@ -30537,11 +30537,11 @@
       </c>
       <c r="D8" s="7">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="2"/>
-        <v>20926</v>
+        <v>19918</v>
       </c>
       <c r="F8" s="7">
         <f>ROUND(Demanda!H8,0)</f>
@@ -30549,7 +30549,7 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" si="3"/>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="H8" s="7">
         <f ca="1">SUM($K$6:K7)*CajasProm</f>
@@ -30557,7 +30557,7 @@
       </c>
       <c r="I8" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="J8" s="21">
         <f t="shared" si="5"/>
@@ -30565,27 +30565,27 @@
       </c>
       <c r="K8" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" ca="1" si="7"/>
-        <v>25824</v>
+        <v>25816</v>
       </c>
       <c r="M8" s="22">
         <f ca="1">IF(Demanda!H9=0,"",L8/(Demanda!H9/DiasVenta))</f>
-        <v>8.6080000000000005</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>OK</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="O8" s="7">
         <f>O7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L8,0)</f>
-        <v>12859</v>
+        <v>11851</v>
       </c>
       <c r="P8" s="22">
         <f>IF(Demanda!L9=0,"",O8/(Demanda!L9/DiasVenta))</f>
-        <v>6.9470556455969747</v>
+        <v>6.4024851431658565</v>
       </c>
       <c r="Q8" s="7">
         <f>Q7+SUMIFS(CgCajas,CgSemana,A8,CgCuenta,1,CgOrigen,"PY")-ROUND(Demanda!M8,0)</f>
@@ -30605,7 +30605,7 @@
       </c>
       <c r="U8" t="str">
         <f t="shared" si="9"/>
-        <v>Bolivia</v>
+        <v>Brasil</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -30619,15 +30619,15 @@
       </c>
       <c r="C9" s="7">
         <f t="shared" si="10"/>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" si="2"/>
-        <v>8974</v>
+        <v>9982</v>
       </c>
       <c r="F9" s="7">
         <f>ROUND(Demanda!H9,0)</f>
@@ -30639,11 +30639,11 @@
       </c>
       <c r="H9" s="7">
         <f ca="1">SUM($K$6:K8)*CajasProm</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="12">
         <f t="shared" ca="1" si="4"/>
-        <v>16798</v>
+        <v>17798</v>
       </c>
       <c r="J9" s="21">
         <f t="shared" si="5"/>
@@ -30651,7 +30651,7 @@
       </c>
       <c r="K9" s="3">
         <f t="shared" ca="1" si="6"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L9" s="7">
         <f t="shared" ca="1" si="7"/>
@@ -30663,7 +30663,7 @@
       </c>
       <c r="N9" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>CARGAR 9</v>
+        <v>CARGAR 8</v>
       </c>
       <c r="O9" s="7">
         <f>O8+SUMIFS(CgCajas,CgSemana,A9,CgCuenta,1,CgOrigen,"BR")-ROUND(Demanda!L9,0)</f>
@@ -31671,11 +31671,11 @@
       </c>
       <c r="B8" s="7">
         <f ca="1">IF(A8="","",Proyeccion!I8)</f>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="C8" s="3">
         <f ca="1">IF(A8="","",Proyeccion!K8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="str">
         <f ca="1">IF(A8="","","BR "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B8-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B8-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="E8" t="str">
         <f ca="1">IF(A8="","",IF(C8&gt;0,Proyeccion!U8,"-"))</f>
-        <v>-</v>
+        <v>Brasil</v>
       </c>
       <c r="F8" t="str">
         <f ca="1">IF(A8="","","PY mie "&amp;TEXT(Proyeccion!A8-5,"dd/mm")&amp;" / BR jue "&amp;TEXT(Proyeccion!A8-4,"dd/mm"))</f>
@@ -31691,15 +31691,15 @@
       </c>
       <c r="G8" s="22">
         <f ca="1">IF(A8="","",Proyeccion!M8)</f>
-        <v>8.6080000000000005</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="H8" t="str">
         <f ca="1">IF(A8="","",Proyeccion!N8)</f>
-        <v>OK</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="I8" t="str">
         <f ca="1">IF(A8="","","Sab "&amp;TEXT(A8,"dd/mm")&amp;": "&amp;FIXED(B8,0)&amp;" cajas - descargan "&amp;Proyeccion!D8&amp;" - vende "&amp;FIXED(Proyeccion!F8,0)&amp;IF(C8&gt;0," -&gt; cargar "&amp;C8&amp;" mas hasta el "&amp;TEXT(Proyeccion!J8,"dd/mm")&amp;" ("&amp;E8&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B8-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 10/10: 25.824 cajas - descargan 21 - vende 18.000 -&gt; ok</v>
+        <v>Sab 10/10: 24.816 cajas - descargan 20 - vende 18.000 -&gt; cargar 1 mas hasta el 06/10 (Brasil; BR hasta el 07/10)</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -31709,11 +31709,11 @@
       </c>
       <c r="B9" s="7">
         <f ca="1">IF(A9="","",Proyeccion!I9)</f>
-        <v>16798</v>
+        <v>17798</v>
       </c>
       <c r="C9" s="3">
         <f ca="1">IF(A9="","",Proyeccion!K9)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D9" t="str">
         <f ca="1">IF(A9="","","BR "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"ddd dd/mm")&amp;" · PY "&amp;TEXT(Proyeccion!B9-LagPY-AtrasoDias,"ddd dd/mm")&amp;" · BO "&amp;TEXT(Proyeccion!B9-LagBO-AtrasoDias,"ddd dd/mm"))</f>
@@ -31733,11 +31733,11 @@
       </c>
       <c r="H9" t="str">
         <f ca="1">IF(A9="","",Proyeccion!N9)</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 8</v>
       </c>
       <c r="I9" t="str">
         <f ca="1">IF(A9="","","Sab "&amp;TEXT(A9,"dd/mm")&amp;": "&amp;FIXED(B9,0)&amp;" cajas - descargan "&amp;Proyeccion!D9&amp;" - vende "&amp;FIXED(Proyeccion!F9,0)&amp;IF(C9&gt;0," -&gt; cargar "&amp;C9&amp;" mas hasta el "&amp;TEXT(Proyeccion!J9,"dd/mm")&amp;" ("&amp;E9&amp;"; BR hasta el "&amp;TEXT(Proyeccion!B9-LagBR-AtrasoDias,"dd/mm")&amp;")"," -&gt; ok"))</f>
-        <v>Sab 17/10: 16.798 cajas - descargan 9 - vende 18.000 -&gt; cargar 9 mas hasta el 13/10 (Brasil; BR hasta el 14/10)</v>
+        <v>Sab 17/10: 17.798 cajas - descargan 10 - vende 18.000 -&gt; cargar 8 mas hasta el 13/10 (Brasil; BR hasta el 14/10)</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -32304,11 +32304,11 @@
       </c>
       <c r="B13" s="7">
         <f ca="1">IFERROR(INDEX(PrBR,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>12859</v>
+        <v>11851</v>
       </c>
       <c r="C13" s="22">
         <f ca="1">IFERROR(INDEX(PrBRd,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>6.9470556455969747</v>
+        <v>6.4024851431658565</v>
       </c>
       <c r="D13" t="str">
         <f ca="1">IF(B13="","",IF(B13&lt;0,"FALTA",IF(C13&lt;2,"CRITICO",IF(C13&lt;CoberturaObjetivo,"JUSTO",IF(C13&gt;VidaVerde,"EXCESO","OK")))))</f>
@@ -32367,19 +32367,19 @@
       </c>
       <c r="B16" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="C16" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>8.6080000000000005</v>
+        <v>8.6053333333333342</v>
       </c>
       <c r="D16" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"")</f>
-        <v>OK</v>
+        <v>CARGAR 1</v>
       </c>
       <c r="E16" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+7),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>ok, cierra sobre 25.000</v>
+        <v>cargar 1 camion(es) mas hasta el mar 06/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -32478,7 +32478,7 @@
       </c>
       <c r="B23" s="40">
         <f ca="1">IFERROR(INDEX(PrProy,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>16798</v>
+        <v>17798</v>
       </c>
       <c r="C23" s="41">
         <f ca="1">IFERROR(INDEX(PrCobertura,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
@@ -32486,11 +32486,11 @@
       </c>
       <c r="D23" s="42" t="str">
         <f ca="1">IFERROR(INDEX(PrEstado,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"")</f>
-        <v>CARGAR 9</v>
+        <v>CARGAR 8</v>
       </c>
       <c r="E23" s="42" t="str">
         <f ca="1">IFERROR(IF(INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&gt;0,"cargar "&amp;INDEX(PrACargar,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0))&amp;" camion(es) mas hasta el "&amp;TEXT(INDEX(PrLimite,MATCH((FechaHoy-WEEKDAY(FechaHoy,2)+1+14),PrSemana,0)),"ddd dd/mm")&amp;" para cerrar en "&amp;FIXED(MinimoSabado,0),"ok, cierra sobre "&amp;FIXED(MinimoSabado,0)),"")</f>
-        <v>cargar 9 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
+        <v>cargar 8 camion(es) mas hasta el mar 13/10 para cerrar en 25.000</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30">
@@ -32545,7 +32545,7 @@
     <row r="30" spans="1:5">
       <c r="A30" s="45" t="str">
         <f ca="1">IFERROR("Frontera lenta (P90): el sabado "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),"dd/mm")&amp;" cerraria en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" cajas ("&amp;IF(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))&gt;INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0))-INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1,PrSemana,0)),0)&amp;" menos que el plan","igual o mas que el plan")&amp;") y el "&amp;TEXT(INDEX(PrSab,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),"dd/mm")&amp;" en "&amp;FIXED(INDEX(Escenarios!L6:L18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;" (plan: "&amp;FIXED(INDEX(Escenarios!G6:G18,MATCH(FechaHoy-WEEKDAY(FechaHoy,2)+1+7,PrSemana,0)),0)&amp;").","")</f>
-        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.880 (plan: 25.824).</v>
+        <v>Frontera lenta (P90): el sabado 03/10 cerraria en 17.886 cajas (5.012 menos que el plan) y el 10/10 en 16.880 (plan: 24.816).</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -32862,7 +32862,7 @@
       </c>
       <c r="C8" s="7">
         <f>Proyeccion!E8</f>
-        <v>20926</v>
+        <v>19918</v>
       </c>
       <c r="D8" s="7">
         <f>Proyeccion!F8</f>
@@ -32870,7 +32870,7 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="4"/>
-        <v>29224</v>
+        <v>28216</v>
       </c>
       <c r="F8">
         <f ca="1">IF(AND(E8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-E8)/CajasProm,0),0)</f>
@@ -32878,19 +32878,19 @@
       </c>
       <c r="G8" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>25824</v>
+        <v>24816</v>
       </c>
       <c r="H8">
         <f ca="1">IF(AND(G8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-G8)/CajasProm,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>22424</v>
+        <v>21416</v>
       </c>
       <c r="J8">
         <f ca="1">IF(AND(I8&lt;MinimoSabado,Proyeccion!J8&gt;=FechaHoy),ROUNDUP((MinimoSabado-I8)/CajasProm,0),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
@@ -32906,15 +32906,15 @@
       </c>
       <c r="N8" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>22884</v>
+        <v>21876</v>
       </c>
       <c r="O8" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>24824</v>
+        <v>23816</v>
       </c>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>24774</v>
+        <v>23766</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="C9" s="7">
         <f>Proyeccion!E9</f>
-        <v>8974</v>
+        <v>9982</v>
       </c>
       <c r="D9" s="7">
         <f>Proyeccion!F9</f>
@@ -32944,19 +32944,19 @@
       </c>
       <c r="G9" s="7">
         <f t="shared" ca="1" si="5"/>
-        <v>16798</v>
+        <v>17798</v>
       </c>
       <c r="H9">
         <f ca="1">IF(AND(G9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-G9)/CajasProm,0),0)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I9" s="7">
         <f t="shared" ca="1" si="6"/>
-        <v>14598</v>
+        <v>15598</v>
       </c>
       <c r="J9">
         <f ca="1">IF(AND(I9&lt;MinimoSabado,Proyeccion!J9&gt;=FechaHoy),ROUNDUP((MinimoSabado-I9)/CajasProm,0),0)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
@@ -32972,15 +32972,15 @@
       </c>
       <c r="N9" s="7">
         <f t="shared" ca="1" si="1"/>
-        <v>13858</v>
+        <v>14858</v>
       </c>
       <c r="O9" s="7">
         <f t="shared" ca="1" si="2"/>
-        <v>15798</v>
+        <v>16798</v>
       </c>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="3"/>
-        <v>14698</v>
+        <v>15698</v>
       </c>
     </row>
     <row r="10" spans="1:16">

</xml_diff>